<commit_message>
Daily dashboard update — 2026-09-14
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -39,7 +39,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="\฿#,##0;[Red]&quot;(฿&quot;#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.00%;[Red]\(0.00%\);\-"/>
@@ -50,6 +50,7 @@
     <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
     <numFmt numFmtId="173" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="174" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -380,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -563,6 +564,7 @@
     <xf numFmtId="0" fontId="21" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21450,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L109"/>
+  <dimension ref="B2:L110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25101,6 +25103,40 @@
         <v>33.04</v>
       </c>
       <c r="K109" s="32" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="72" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C110" t="n">
+        <v>26306593</v>
+      </c>
+      <c r="D110" t="n">
+        <v>22820086</v>
+      </c>
+      <c r="E110" t="n">
+        <v>3486507</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0.1528</v>
+      </c>
+      <c r="G110" t="n">
+        <v>18567190</v>
+      </c>
+      <c r="H110" t="n">
+        <v>4906306</v>
+      </c>
+      <c r="I110" t="n">
+        <v>1442002</v>
+      </c>
+      <c r="J110" t="n">
+        <v>33.09</v>
+      </c>
+      <c r="K110" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25678,7 +25714,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25693,11 +25729,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.04</v>
+        <v>33.09</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-13</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -25742,11 +25778,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.0753</v>
+        <v>26.1154</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-13</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -25861,27 +25897,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>19.9269</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>20.6605</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>20.457</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -25906,27 +25942,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7028</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7026</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7024</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -25951,27 +25987,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3986</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.4352</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.5398</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -25996,27 +26032,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.5502</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.6533</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.631500000000001</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26041,27 +26077,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.673999999999999</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.724600000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.7386</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26086,27 +26122,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.0676</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.0998</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.0907</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26131,27 +26167,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.198</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.1621</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.214</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26176,27 +26212,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.2553</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.1105</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.2194</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26221,27 +26257,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.6446</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.928</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.9527</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26266,27 +26302,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.3034</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.45</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.4623</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26311,27 +26347,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.2087</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.3462</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46273</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.651</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -26356,27 +26392,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.39870000000001</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>83.035</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>83.14149999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26401,27 +26437,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.8345</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>55.146</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>55.2169</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26446,27 +26482,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5105</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5226</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5321</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26491,7 +26527,7 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
-        <v>23.4437</v>
+        <v>23.4445</v>
       </c>
       <c r="F19" s="34" t="inlineStr">
         <is>
@@ -26499,7 +26535,7 @@
         </is>
       </c>
       <c r="G19" s="28" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H19" s="34" t="inlineStr">
         <is>
@@ -26507,11 +26543,11 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>23.4433</v>
+        <v>23.444</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26536,7 +26572,7 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
-        <v>41.7417</v>
+        <v>41.321</v>
       </c>
       <c r="F20" s="34" t="inlineStr">
         <is>
@@ -26544,7 +26580,7 @@
         </is>
       </c>
       <c r="G20" s="28" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="H20" s="34" t="inlineStr">
         <is>
@@ -26552,11 +26588,11 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>42.0101</v>
+        <v>41.565</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26581,27 +26617,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.6558</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.7197</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.7483</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26626,27 +26662,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9751</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0259</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.1639</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26671,27 +26707,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.2128</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.2917</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.3018</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26716,27 +26752,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.3866</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.534</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.5272</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26761,27 +26797,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.723599999999999</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.8774</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8202</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26806,27 +26842,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.6353</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.8562</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7748</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26851,27 +26887,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.3081</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.4161</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.4336</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26896,27 +26932,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.1126</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.3163</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.3868</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26941,27 +26977,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.5527</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.625</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.5184</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26986,27 +27022,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>35.424</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>36.0094</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.2568</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -27031,27 +27067,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.3072</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.3978</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.4173</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27076,27 +27112,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7204</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7202</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.72</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27121,27 +27157,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.0227</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1264</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1708</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27166,27 +27202,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2364</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2361</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2357</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27211,27 +27247,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.0761</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.5269</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.3339</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -27256,27 +27292,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0128</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0662</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0969</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27301,27 +27337,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.5612</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.7242</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.7647</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27354,7 +27390,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27394,7 +27430,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27434,7 +27470,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27474,7 +27510,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27514,7 +27550,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27554,7 +27590,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27594,7 +27630,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -27634,7 +27670,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27674,7 +27710,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27751,7 +27787,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27791,7 +27827,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -27831,7 +27867,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -27871,7 +27907,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -27911,7 +27947,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -27951,7 +27987,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -27991,7 +28027,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28031,7 +28067,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28071,7 +28107,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28111,7 +28147,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28151,7 +28187,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28191,7 +28227,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28231,7 +28267,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28271,7 +28307,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28311,7 +28347,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28351,7 +28387,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28391,7 +28427,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28431,7 +28467,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28471,7 +28507,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28511,7 +28547,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28551,7 +28587,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28591,7 +28627,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28631,7 +28667,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28671,7 +28707,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28711,7 +28747,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28751,7 +28787,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28791,7 +28827,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28831,7 +28867,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -28871,7 +28907,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -28911,7 +28947,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -28951,7 +28987,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -28991,7 +29027,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29031,7 +29067,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29071,7 +29107,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29111,7 +29147,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29151,7 +29187,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29183,7 +29219,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>126.22</v>
+        <v>125.01</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29191,7 +29227,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29199,7 +29235,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>124.75997</v>
+        <v>126.155085</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29223,7 +29259,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>729.2</v>
+        <v>717.03</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29231,7 +29267,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29239,7 +29275,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>729.248335</v>
+        <v>728.936635</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29263,7 +29299,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>77284</v>
+        <v>76833</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29271,7 +29307,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29279,7 +29315,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>77306.27473600001</v>
+        <v>77260.464033</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29303,7 +29339,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007305</v>
+        <v>0.007024</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29311,7 +29347,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29319,7 +29355,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007203</v>
+        <v>0.0073</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29343,7 +29379,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01317</v>
+        <v>0.012896</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29351,7 +29387,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29359,7 +29395,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.013593</v>
+        <v>0.013206</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29383,7 +29419,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>102.02</v>
+        <v>99.65000000000001</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29391,7 +29427,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29399,7 +29435,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>102.070088</v>
+        <v>101.978348</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29423,7 +29459,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.99</v>
+        <v>1.95</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29431,7 +29467,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29439,7 +29475,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.987399</v>
+        <v>1.983589</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29471,7 +29507,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29503,7 +29539,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.024528</v>
+        <v>0.02413</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29511,7 +29547,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29519,7 +29555,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.024855</v>
+        <v>0.024522</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29543,7 +29579,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>4.666966</v>
+        <v>4.459672</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29551,7 +29587,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29559,7 +29595,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>4.692606</v>
+        <v>4.67025</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29583,7 +29619,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.106546</v>
+        <v>23.28454</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29591,7 +29627,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29599,7 +29635,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.063977</v>
+        <v>24.110243</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29623,7 +29659,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.147921</v>
+        <v>0.1366</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29631,7 +29667,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29639,7 +29675,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.151886</v>
+        <v>0.148123</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29663,7 +29699,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>24092.768</v>
+        <v>23726.5227</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29671,7 +29707,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29679,7 +29715,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>24094.364996</v>
+        <v>24120.513247</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29703,7 +29739,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2553463.36</v>
+        <v>2542403.97</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29711,7 +29747,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29719,7 +29755,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2554199.317275</v>
+        <v>2556548.754856</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29743,7 +29779,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.806252</v>
+        <v>2.737734</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29751,7 +29787,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29759,7 +29795,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.786902</v>
+        <v>2.80963</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29783,7 +29819,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>83422.3656</v>
+        <v>82197.8763</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29791,7 +29827,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29799,7 +29835,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>83052.24193800001</v>
+        <v>83529.791075</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29823,7 +29859,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.015731</v>
+        <v>19.682164</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -29831,7 +29867,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -29839,7 +29875,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>19.717056</v>
+        <v>20.045873</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -29863,7 +29899,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>77284</v>
+        <v>76833</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -29871,7 +29907,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -29879,7 +29915,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>77306.27473600001</v>
+        <v>77260.464033</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -29903,7 +29939,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>20.19</v>
+        <v>19.5</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -29911,7 +29947,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -29919,7 +29955,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>20.101408</v>
+        <v>20.166768</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30017,7 +30053,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007305</v>
+        <v>0.007024</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30025,7 +30061,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30033,7 +30069,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007203</v>
+        <v>0.0073</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30057,7 +30093,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>102.02</v>
+        <v>99.65000000000001</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30065,7 +30101,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30073,7 +30109,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>102.070088</v>
+        <v>101.978348</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30105,7 +30141,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30137,27 +30173,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.3998</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46274</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.6311</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46273</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.5123</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-15
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L110"/>
+  <dimension ref="B2:L111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25137,6 +25137,40 @@
         <v>33.09</v>
       </c>
       <c r="K110" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="72" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C111" t="n">
+        <v>26277279</v>
+      </c>
+      <c r="D111" t="n">
+        <v>22833992</v>
+      </c>
+      <c r="E111" t="n">
+        <v>3443287</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0.1508</v>
+      </c>
+      <c r="G111" t="n">
+        <v>18567190</v>
+      </c>
+      <c r="H111" t="n">
+        <v>4859202</v>
+      </c>
+      <c r="I111" t="n">
+        <v>1463521</v>
+      </c>
+      <c r="J111" t="n">
+        <v>33.22</v>
+      </c>
+      <c r="K111" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25714,7 +25748,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25729,11 +25763,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.09</v>
+        <v>33.22</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-14</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -25778,11 +25812,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1154</v>
+        <v>26.1404</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-14</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27390,7 +27424,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27422,7 +27456,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.081</v>
+        <v>1.061</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27430,7 +27464,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27438,7 +27472,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.081</v>
+        <v>1.061</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27470,7 +27504,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27478,7 +27512,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>758.080017</v>
+        <v>737.909973</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27510,7 +27544,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27550,7 +27584,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27558,7 +27592,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>206.639999</v>
+        <v>206.699997</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27582,23 +27616,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.8</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>15.3</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27622,23 +27656,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>192</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>188</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>190</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27670,7 +27704,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27710,7 +27744,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27787,7 +27821,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27819,23 +27853,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>61.75</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>62.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -27867,7 +27901,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -27899,7 +27933,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.2</v>
+        <v>16</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -27907,7 +27941,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -27939,7 +27973,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -27947,7 +27981,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -27955,7 +27989,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -27987,7 +28021,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28019,7 +28053,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.3</v>
+        <v>22.2</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28027,7 +28061,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28035,7 +28069,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.299999</v>
+        <v>22.200001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28059,7 +28093,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.44</v>
+        <v>3.46</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28067,7 +28101,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28075,7 +28109,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.44</v>
+        <v>3.46</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28099,7 +28133,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.32</v>
+        <v>4.26</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28107,7 +28141,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28115,7 +28149,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.32</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28139,7 +28173,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.28</v>
+        <v>3.22</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28147,7 +28181,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28155,7 +28189,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.28</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28179,7 +28213,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28187,7 +28221,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28195,7 +28229,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28227,7 +28261,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28259,7 +28293,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>113.43</v>
+        <v>105.31</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28267,7 +28301,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28299,7 +28333,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>252.23</v>
+        <v>265.6</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28307,7 +28341,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28339,7 +28373,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>456.49</v>
+        <v>424.21</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28347,7 +28381,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28379,7 +28413,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>118.79</v>
+        <v>116.34</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28387,7 +28421,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28419,7 +28453,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>36.35</v>
+        <v>36.66</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28427,7 +28461,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28459,7 +28493,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>188.72</v>
+        <v>176.22</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28467,7 +28501,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28499,7 +28533,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>156.07</v>
+        <v>170.18</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28507,7 +28541,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28539,7 +28573,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>179.59</v>
+        <v>197.07</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28547,7 +28581,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28579,7 +28613,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>180.64</v>
+        <v>169.09</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28587,7 +28621,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28619,7 +28653,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1115.7</v>
+        <v>1138.28</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28627,7 +28661,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28659,7 +28693,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>74.2</v>
+        <v>71.48</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28667,7 +28701,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28699,7 +28733,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1234.46</v>
+        <v>1143.24</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28707,7 +28741,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28739,7 +28773,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>165.37</v>
+        <v>161.84</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28747,7 +28781,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28779,7 +28813,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>218.29</v>
+        <v>210.96</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -28787,7 +28821,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28819,7 +28853,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>83.56</v>
+        <v>76.62</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -28827,7 +28861,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28859,7 +28893,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>116.65</v>
+        <v>107.98</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -28867,7 +28901,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -28899,7 +28933,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>379.72</v>
+        <v>329.2</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -28907,7 +28941,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -28939,7 +28973,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>365.44</v>
+        <v>358.97</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -28947,7 +28981,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -28979,7 +29013,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>42.23</v>
+        <v>42.24</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -28987,7 +29021,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29019,7 +29053,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>70.56</v>
+        <v>68.93000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29027,7 +29061,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29059,7 +29093,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>332.27</v>
+        <v>333.08</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29067,7 +29101,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29099,7 +29133,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>175.26</v>
+        <v>191.45</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29107,7 +29141,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29139,7 +29173,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>648.03</v>
+        <v>665.6</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29147,7 +29181,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29179,7 +29213,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>33.5</v>
+        <v>32.34</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29187,7 +29221,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29195,7 +29229,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>37.59</v>
+        <v>32.34</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29219,7 +29253,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>125.01</v>
+        <v>128.26</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29227,7 +29261,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29235,7 +29269,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>126.155085</v>
+        <v>124.984987</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29259,7 +29293,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>717.03</v>
+        <v>719.54</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29267,7 +29301,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29275,7 +29309,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>728.936635</v>
+        <v>717.088195</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29299,7 +29333,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>76833</v>
+        <v>77887</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29307,7 +29341,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29315,7 +29349,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>77260.464033</v>
+        <v>76818.78172</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29339,7 +29373,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007024</v>
+        <v>0.007128</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29347,7 +29381,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29355,7 +29389,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.0073</v>
+        <v>0.007023</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29379,7 +29413,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.012896</v>
+        <v>0.013116</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29387,7 +29421,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29395,7 +29429,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.013206</v>
+        <v>0.01289</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29419,7 +29453,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>99.65000000000001</v>
+        <v>102.31</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29427,7 +29461,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29435,7 +29469,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>101.978348</v>
+        <v>99.62332499999999</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29459,7 +29493,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.95</v>
+        <v>1.99</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29467,7 +29501,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29475,7 +29509,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.983589</v>
+        <v>1.956139</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29507,7 +29541,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29539,7 +29573,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.02413</v>
+        <v>0.024179</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29547,7 +29581,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29555,7 +29589,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.024522</v>
+        <v>0.024135</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29579,7 +29613,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>4.459672</v>
+        <v>4.456496</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29587,7 +29621,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29595,7 +29629,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>4.67025</v>
+        <v>4.472203</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29619,7 +29653,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.28454</v>
+        <v>23.889631</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29627,7 +29661,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29635,7 +29669,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>24.110243</v>
+        <v>23.382384</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29659,7 +29693,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.1366</v>
+        <v>0.142283</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29667,7 +29701,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29675,7 +29709,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.148123</v>
+        <v>0.137122</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29699,7 +29733,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>23726.5227</v>
+        <v>23903.1188</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29707,7 +29741,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29715,7 +29749,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>24120.513247</v>
+        <v>23821.669833</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29739,7 +29773,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2542403.97</v>
+        <v>2587406.14</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29747,7 +29781,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29755,7 +29789,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2556548.754856</v>
+        <v>2551919.928727</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29779,7 +29813,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.737734</v>
+        <v>2.780514</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29787,7 +29821,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29795,7 +29829,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.80963</v>
+        <v>2.748095</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29819,7 +29853,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>82197.8763</v>
+        <v>83497.1412</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29827,7 +29861,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29835,7 +29869,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>83529.791075</v>
+        <v>82482.251109</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29859,7 +29893,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>19.682164</v>
+        <v>20.016279</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -29867,7 +29901,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -29875,7 +29909,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.045873</v>
+        <v>19.741623</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -29899,7 +29933,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>76833</v>
+        <v>77887</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -29907,7 +29941,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -29915,7 +29949,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>77260.464033</v>
+        <v>76818.78172</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -29939,7 +29973,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>19.5</v>
+        <v>19.61</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -29947,7 +29981,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -29955,7 +29989,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>20.166768</v>
+        <v>19.516404</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30053,7 +30087,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007024</v>
+        <v>0.007128</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30061,7 +30095,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30069,7 +30103,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.0073</v>
+        <v>0.007023</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30093,7 +30127,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>99.65000000000001</v>
+        <v>102.31</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30101,7 +30135,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30109,7 +30143,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>101.978348</v>
+        <v>99.62332499999999</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30141,7 +30175,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-16
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L111"/>
+  <dimension ref="B2:L112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25171,6 +25171,40 @@
         <v>33.22</v>
       </c>
       <c r="K111" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="72" t="n">
+        <v>46281</v>
+      </c>
+      <c r="C112" t="n">
+        <v>26379342</v>
+      </c>
+      <c r="D112" t="n">
+        <v>22840432</v>
+      </c>
+      <c r="E112" t="n">
+        <v>3538910</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.1549</v>
+      </c>
+      <c r="G112" t="n">
+        <v>18727576</v>
+      </c>
+      <c r="H112" t="n">
+        <v>4848763</v>
+      </c>
+      <c r="I112" t="n">
+        <v>1429497</v>
+      </c>
+      <c r="J112" t="n">
+        <v>33.28</v>
+      </c>
+      <c r="K112" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25748,7 +25782,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25763,11 +25797,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.22</v>
+        <v>33.28</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-15</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -25812,11 +25846,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1404</v>
+        <v>26.1526</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-15</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -25931,27 +25965,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>19.9564</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>19.9269</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>20.6605</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -25976,27 +26010,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7033</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7028</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7026</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26021,27 +26055,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3992</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3986</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.4352</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26066,27 +26100,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.509399999999999</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.5502</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.6533</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26111,27 +26145,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.6075</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.673999999999999</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.724600000000001</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26156,27 +26190,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>12.9564</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.0676</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.0998</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26201,27 +26235,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.0292</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.198</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.1621</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26246,27 +26280,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>28.7847</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.2553</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.1105</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26291,27 +26325,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.4572</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.6446</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.928</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26336,27 +26370,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.2295</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.3034</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.45</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26381,27 +26415,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.0809</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.2087</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.3462</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26426,27 +26460,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.8845</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.39870000000001</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>83.035</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26471,27 +26505,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.6456</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.8345</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>55.146</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26516,27 +26550,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5078</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5105</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5226</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26561,27 +26595,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4459</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4445</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.444</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26606,27 +26640,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.6729</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.321</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.565</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26651,27 +26685,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.5698</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.6558</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.7197</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26696,27 +26730,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9551</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9751</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0259</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26741,27 +26775,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.1753</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.2128</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.2917</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26786,27 +26820,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.5536</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.3866</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.534</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26831,27 +26865,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.7195</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.723599999999999</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8774</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26876,27 +26910,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.6354</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.6353</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.8562</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26921,27 +26955,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.2171</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.3081</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.4161</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26966,27 +27000,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.9136</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.1126</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.3163</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27011,27 +27045,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.3625</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.5527</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.625</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27056,27 +27090,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>35.8478</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>35.424</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>36.0094</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27101,27 +27135,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.1923</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.3072</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.3978</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27146,27 +27180,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7209</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7204</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7202</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27191,27 +27225,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.9865</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.0227</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1264</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27236,27 +27270,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2374</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2364</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2361</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27281,27 +27315,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.3577</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.0761</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.5269</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27326,27 +27360,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0188</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0128</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0662</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27371,27 +27405,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.4228</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.5612</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.7242</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27424,7 +27458,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27464,7 +27498,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27496,7 +27530,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>758.08</v>
+        <v>737.91</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27504,7 +27538,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27544,7 +27578,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27576,7 +27610,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>206.64</v>
+        <v>206.7</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27584,7 +27618,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27592,7 +27626,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>206.699997</v>
+        <v>205.710007</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27616,23 +27650,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.7</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.8</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27656,23 +27690,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>192</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>188</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27704,7 +27738,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27744,7 +27778,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27821,7 +27855,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27853,23 +27887,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>61</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>60.75</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>61.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -27893,7 +27927,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -27901,7 +27935,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -27941,7 +27975,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -27981,7 +28015,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28013,7 +28047,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.7</v>
+        <v>5.65</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28021,7 +28055,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28029,7 +28063,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.7</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28053,7 +28087,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.2</v>
+        <v>22.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28061,7 +28095,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28069,7 +28103,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.200001</v>
+        <v>22.799999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28093,7 +28127,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.46</v>
+        <v>3.44</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28101,7 +28135,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28109,7 +28143,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.46</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28133,7 +28167,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.26</v>
+        <v>4.38</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28141,7 +28175,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28149,7 +28183,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.26</v>
+        <v>4.38</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28173,7 +28207,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.22</v>
+        <v>3.26</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28181,7 +28215,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28189,7 +28223,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.22</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28213,7 +28247,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28221,7 +28255,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28229,7 +28263,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28253,7 +28287,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.8</v>
+        <v>18.1</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28261,7 +28295,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28269,7 +28303,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.799999</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28293,7 +28327,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>105.31</v>
+        <v>105.04</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28301,7 +28335,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28309,7 +28343,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>113.43</v>
+        <v>105.309998</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28333,7 +28367,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>265.6</v>
+        <v>257.76</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28341,7 +28375,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28349,7 +28383,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>252.229996</v>
+        <v>265.600006</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28373,7 +28407,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>424.21</v>
+        <v>421.17</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28381,7 +28415,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28389,7 +28423,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>456.48999</v>
+        <v>424.209991</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28413,7 +28447,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>116.34</v>
+        <v>122.21</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28421,7 +28455,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28429,7 +28463,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>118.790001</v>
+        <v>116.339996</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28453,23 +28487,23 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
+        <v>36.72</v>
+      </c>
+      <c r="F64" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G64" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H64" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
         <v>36.66</v>
-      </c>
-      <c r="F64" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G64" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H64" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I64" t="n">
-        <v>36.349998</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28493,7 +28527,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>176.22</v>
+        <v>176.49</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28501,7 +28535,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28509,7 +28543,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>188.720001</v>
+        <v>176.220001</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28533,7 +28567,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>170.18</v>
+        <v>172.37</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28541,7 +28575,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28549,7 +28583,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>156.070007</v>
+        <v>170.179993</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28573,7 +28607,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>197.07</v>
+        <v>195.62</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28581,7 +28615,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28589,7 +28623,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>179.589996</v>
+        <v>197.070007</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28613,7 +28647,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>169.09</v>
+        <v>168.02</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28621,7 +28655,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28629,7 +28663,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>180.639999</v>
+        <v>169.089996</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28653,7 +28687,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1138.28</v>
+        <v>1136.11</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28661,7 +28695,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28669,7 +28703,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1115.699951</v>
+        <v>1138.280029</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28693,7 +28727,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>71.48</v>
+        <v>71.48999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28701,7 +28735,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28709,7 +28743,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>74.199997</v>
+        <v>71.480003</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -28733,7 +28767,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1143.24</v>
+        <v>1142.46</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28741,7 +28775,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28749,7 +28783,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1234.459961</v>
+        <v>1143.23999</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -28773,7 +28807,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>161.84</v>
+        <v>160.72</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28781,7 +28815,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28789,7 +28823,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>165.369995</v>
+        <v>161.839996</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -28813,7 +28847,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>210.96</v>
+        <v>212.17</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -28821,7 +28855,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28829,7 +28863,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>218.289993</v>
+        <v>210.960007</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -28853,7 +28887,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>76.62</v>
+        <v>77.89</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -28861,7 +28895,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28869,7 +28903,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>83.55999799999999</v>
+        <v>76.620003</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -28893,7 +28927,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>107.98</v>
+        <v>118.06</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -28901,7 +28935,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -28909,7 +28943,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>116.650002</v>
+        <v>107.980003</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -28933,7 +28967,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>329.2</v>
+        <v>332.85</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -28941,7 +28975,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -28949,7 +28983,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>379.720001</v>
+        <v>329.200012</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -28973,7 +29007,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>358.97</v>
+        <v>356.58</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -28981,7 +29015,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -28989,7 +29023,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>365.440002</v>
+        <v>358.970001</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29013,7 +29047,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>42.24</v>
+        <v>41.58</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29021,7 +29055,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29029,7 +29063,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>42.23</v>
+        <v>42.240002</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29053,23 +29087,23 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="F79" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G79" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H79" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
         <v>68.93000000000001</v>
-      </c>
-      <c r="F79" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G79" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H79" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I79" t="n">
-        <v>70.55999799999999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29093,7 +29127,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>333.08</v>
+        <v>331.34</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29101,7 +29135,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29109,7 +29143,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>332.269989</v>
+        <v>333.079987</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29133,7 +29167,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>191.45</v>
+        <v>172.11</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29141,7 +29175,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29149,7 +29183,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>175.259995</v>
+        <v>191.449997</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29173,7 +29207,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>665.6</v>
+        <v>670.24</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29181,7 +29215,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29189,7 +29223,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>648.030029</v>
+        <v>665.599976</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29213,7 +29247,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>32.34</v>
+        <v>30.1</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29221,7 +29255,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29229,7 +29263,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>32.34</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29253,7 +29287,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>128.26</v>
+        <v>121.32</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29261,7 +29295,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29269,7 +29303,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>124.984987</v>
+        <v>128.372117</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29293,7 +29327,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>719.54</v>
+        <v>712.12</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29301,7 +29335,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29309,7 +29343,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>717.088195</v>
+        <v>719.684781</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29333,7 +29367,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>77887</v>
+        <v>75671</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29341,7 +29375,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29349,7 +29383,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>76818.78172</v>
+        <v>77934.287587</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29373,23 +29407,23 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
+        <v>0.006814</v>
+      </c>
+      <c r="F87" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G87" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H87" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
         <v>0.007128</v>
-      </c>
-      <c r="F87" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G87" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H87" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I87" t="n">
-        <v>0.007023</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29413,7 +29447,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.013116</v>
+        <v>0.012389</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29421,7 +29455,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29429,7 +29463,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.01289</v>
+        <v>0.013095</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29453,7 +29487,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>102.31</v>
+        <v>96.84</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29461,7 +29495,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29469,7 +29503,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>99.62332499999999</v>
+        <v>102.322216</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29493,7 +29527,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.99</v>
+        <v>1.86</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29501,7 +29535,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29509,7 +29543,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.956139</v>
+        <v>1.98936</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29541,7 +29575,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29573,7 +29607,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.024179</v>
+        <v>0.022729</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29581,7 +29615,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29589,7 +29623,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.024135</v>
+        <v>0.024189</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29613,7 +29647,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>4.456496</v>
+        <v>4.996127</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29621,7 +29655,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29629,7 +29663,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>4.472203</v>
+        <v>4.468399</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29653,7 +29687,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.889631</v>
+        <v>22.812874</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29661,7 +29695,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29669,7 +29703,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>23.382384</v>
+        <v>23.928266</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29693,7 +29727,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.142283</v>
+        <v>0.131654</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29701,7 +29735,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29709,7 +29743,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.137122</v>
+        <v>0.142014</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29733,7 +29767,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>23903.1188</v>
+        <v>23699.3536</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29741,7 +29775,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29749,7 +29783,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>23821.669833</v>
+        <v>23951.109502</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29773,7 +29807,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2587406.14</v>
+        <v>2518330.88</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29781,7 +29815,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29789,7 +29823,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2551919.928727</v>
+        <v>2593653.090879</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29813,7 +29847,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.780514</v>
+        <v>2.65804</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29821,7 +29855,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29829,7 +29863,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.748095</v>
+        <v>2.787503</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29853,7 +29887,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>83497.1412</v>
+        <v>79803.44319999999</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29861,7 +29895,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29869,7 +29903,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>82482.251109</v>
+        <v>83629.01332899999</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29893,7 +29927,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.016279</v>
+        <v>19.727352</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -29901,7 +29935,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -29909,7 +29943,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>19.741623</v>
+        <v>20.094738</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -29933,7 +29967,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>77887</v>
+        <v>75671</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -29941,7 +29975,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -29949,7 +29983,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>76818.78172</v>
+        <v>77934.287587</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -29973,7 +30007,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>19.61</v>
+        <v>18.76</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -29981,7 +30015,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -29989,7 +30023,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>19.516404</v>
+        <v>19.554105</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30087,23 +30121,23 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
+        <v>0.006814</v>
+      </c>
+      <c r="F105" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G105" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H105" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
         <v>0.007128</v>
-      </c>
-      <c r="F105" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G105" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H105" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I105" t="n">
-        <v>0.007023</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30127,7 +30161,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>102.31</v>
+        <v>96.84</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30135,7 +30169,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30143,7 +30177,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>99.62332499999999</v>
+        <v>102.322216</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30175,7 +30209,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30207,27 +30241,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.0869</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.3998</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.6311</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-17
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L112"/>
+  <dimension ref="B2:L113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25205,6 +25205,40 @@
         <v>33.28</v>
       </c>
       <c r="K112" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="72" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C113" t="n">
+        <v>26048190</v>
+      </c>
+      <c r="D113" t="n">
+        <v>22849258</v>
+      </c>
+      <c r="E113" t="n">
+        <v>3198932</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G113" t="n">
+        <v>18382554</v>
+      </c>
+      <c r="H113" t="n">
+        <v>4837769</v>
+      </c>
+      <c r="I113" t="n">
+        <v>1456759</v>
+      </c>
+      <c r="J113" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="K113" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25782,7 +25816,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25797,11 +25831,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.28</v>
+        <v>33.37</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-16</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -25846,11 +25880,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1526</v>
+        <v>26.1457</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-16</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -25965,27 +25999,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>18.8659</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>19.9564</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>19.9269</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26010,27 +26044,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7035</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7033</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7028</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26055,27 +26089,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.4342</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3992</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.3986</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26100,27 +26134,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.420400000000001</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.509399999999999</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.5502</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26145,27 +26179,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.5448</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.6075</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.673999999999999</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26190,27 +26224,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.0836</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>12.9564</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.0676</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26235,27 +26269,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.0984</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.0292</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.198</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26280,27 +26314,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>28.7218</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>28.7847</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.2553</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26325,27 +26359,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.2026</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.4572</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.6446</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26370,27 +26404,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.1505</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.2295</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.3034</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26415,27 +26449,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.0949</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.0809</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.2087</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26460,27 +26494,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.4216</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.8845</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.39870000000001</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26550,27 +26584,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4974</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5078</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5105</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26595,27 +26629,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4463</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4459</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4445</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26640,27 +26674,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.4936</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.6729</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.321</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26685,27 +26719,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.4127</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.5698</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.6558</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26730,27 +26764,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0344</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9551</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.9751</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26775,27 +26809,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.1696</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.1753</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.2128</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26820,27 +26854,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.3892</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.5536</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.3866</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26865,27 +26899,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.858700000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.7195</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.723599999999999</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26910,27 +26944,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.8314</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.6354</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.6353</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26955,27 +26989,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.254</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.2171</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.3081</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27000,27 +27034,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.7589</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.9136</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.1126</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27045,27 +27079,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>23.6884</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.3625</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.5527</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27090,27 +27124,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>33.9841</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>35.8478</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>35.424</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27135,27 +27169,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.0952</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.1923</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.3072</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27180,27 +27214,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7211</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7209</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7204</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27225,27 +27259,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.924</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.9865</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.0227</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27270,27 +27304,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2378</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2374</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2364</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27315,27 +27349,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.1131</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.3577</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.0761</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27360,27 +27394,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.9908</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0188</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0128</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27405,27 +27439,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.3241</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.4228</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.5612</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27458,7 +27492,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27466,7 +27500,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.27</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27490,7 +27524,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.061</v>
+        <v>1.055</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27498,7 +27532,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27506,7 +27540,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.061</v>
+        <v>1.064</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27538,7 +27572,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27546,7 +27580,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>737.909973</v>
+        <v>739.98999</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27578,7 +27612,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27610,7 +27644,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>206.7</v>
+        <v>205.71</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27618,7 +27652,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27650,23 +27684,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.6</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.7</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27690,23 +27724,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>192</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>192.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>192</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27730,7 +27764,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -27738,7 +27772,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27746,7 +27780,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -27770,7 +27804,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27812,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27786,7 +27820,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -27855,7 +27889,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27887,23 +27921,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>60.25</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>61</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>60.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -27927,7 +27961,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -27935,7 +27969,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -27943,7 +27977,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -27975,7 +28009,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28007,7 +28041,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28015,7 +28049,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28023,7 +28057,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28047,7 +28081,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.65</v>
+        <v>5.55</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28055,7 +28089,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28063,7 +28097,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.65</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28087,7 +28121,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.8</v>
+        <v>22.5</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28095,7 +28129,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28127,7 +28161,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.44</v>
+        <v>3.4</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28135,7 +28169,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28143,7 +28177,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.44</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28167,7 +28201,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.38</v>
+        <v>4.48</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28175,7 +28209,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28183,7 +28217,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.38</v>
+        <v>4.48</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28207,7 +28241,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.26</v>
+        <v>3.18</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28215,7 +28249,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28223,7 +28257,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.26</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28255,7 +28289,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28287,7 +28321,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>18.1</v>
+        <v>17.9</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28295,7 +28329,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28303,7 +28337,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>18.1</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28327,7 +28361,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>105.04</v>
+        <v>103.75</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28335,7 +28369,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28343,7 +28377,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>105.309998</v>
+        <v>105.040001</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28367,7 +28401,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>257.76</v>
+        <v>250.5</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28375,7 +28409,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28383,7 +28417,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>265.600006</v>
+        <v>257.76001</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28407,7 +28441,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>421.17</v>
+        <v>415.38</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28415,7 +28449,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28423,7 +28457,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>424.209991</v>
+        <v>415.380005</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28447,7 +28481,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>122.21</v>
+        <v>118</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28455,7 +28489,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28463,7 +28497,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>116.339996</v>
+        <v>122.209999</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28487,7 +28521,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>36.72</v>
+        <v>35.56</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28495,7 +28529,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28503,7 +28537,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>36.66</v>
+        <v>36.720001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28527,7 +28561,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>176.49</v>
+        <v>175.54</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28535,7 +28569,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28543,7 +28577,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>176.220001</v>
+        <v>175.539993</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28567,7 +28601,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>172.37</v>
+        <v>171.77</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28575,7 +28609,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28583,7 +28617,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>170.179993</v>
+        <v>171.770004</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28607,7 +28641,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>195.62</v>
+        <v>191.57</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28615,7 +28649,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28623,7 +28657,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>197.070007</v>
+        <v>191.570007</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28647,7 +28681,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>168.02</v>
+        <v>167.36</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28655,7 +28689,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28663,7 +28697,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>169.089996</v>
+        <v>167.360001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28687,7 +28721,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1136.11</v>
+        <v>1137.82</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28695,7 +28729,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28703,7 +28737,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1138.280029</v>
+        <v>1137.819946</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28727,7 +28761,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>71.48999999999999</v>
+        <v>69.59</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28735,7 +28769,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28743,7 +28777,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>71.480003</v>
+        <v>69.589996</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -28767,7 +28801,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1142.46</v>
+        <v>1147.61</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28775,7 +28809,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28783,7 +28817,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1143.23999</v>
+        <v>1147.609985</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -28807,7 +28841,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>160.72</v>
+        <v>165.19</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28815,7 +28849,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28823,7 +28857,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>161.839996</v>
+        <v>165.190002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -28847,7 +28881,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>212.17</v>
+        <v>213.9</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -28855,7 +28889,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28863,7 +28897,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>210.960007</v>
+        <v>213.899994</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -28887,7 +28921,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.89</v>
+        <v>76.30500000000001</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -28895,7 +28929,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28903,7 +28937,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>76.620003</v>
+        <v>76.30999799999999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -28927,7 +28961,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>118.06</v>
+        <v>113.97</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -28935,7 +28969,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -28943,7 +28977,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>107.980003</v>
+        <v>118.059998</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -28967,7 +29001,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>332.85</v>
+        <v>341.15</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -28975,7 +29009,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -28983,7 +29017,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>329.200012</v>
+        <v>341.149994</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29007,7 +29041,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>356.58</v>
+        <v>358.08</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29015,7 +29049,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29023,7 +29057,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>358.970001</v>
+        <v>358.079987</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29047,7 +29081,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>41.58</v>
+        <v>40.67</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29055,7 +29089,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29063,7 +29097,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>42.240002</v>
+        <v>41.580002</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29087,7 +29121,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>68.3</v>
+        <v>67.61</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29095,7 +29129,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29103,7 +29137,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>68.93000000000001</v>
+        <v>67.610001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29127,7 +29161,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>331.34</v>
+        <v>332.41</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29135,7 +29169,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29143,7 +29177,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>333.079987</v>
+        <v>332.410004</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29167,7 +29201,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>172.11</v>
+        <v>164.51</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29175,7 +29209,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29183,7 +29217,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>191.449997</v>
+        <v>172.110001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29207,7 +29241,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>670.24</v>
+        <v>673.3099999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29215,7 +29249,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29223,7 +29257,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>665.599976</v>
+        <v>670.23999</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29247,7 +29281,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.1</v>
+        <v>30.39</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29255,7 +29289,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29263,7 +29297,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.1</v>
+        <v>30.389999</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29287,7 +29321,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>121.32</v>
+        <v>121.58</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29295,7 +29329,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29303,7 +29337,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>128.372117</v>
+        <v>121.721319</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29327,7 +29361,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>712.12</v>
+        <v>727.1799999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29335,7 +29369,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29343,7 +29377,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>719.684781</v>
+        <v>713.718371</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29367,7 +29401,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>75671</v>
+        <v>76562</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29375,7 +29409,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29383,7 +29417,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>77934.287587</v>
+        <v>75820.35404799999</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29407,7 +29441,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.006814</v>
+        <v>0.007018</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29415,7 +29449,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29423,7 +29457,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007128</v>
+        <v>0.006853</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29447,7 +29481,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.012389</v>
+        <v>0.012468</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29455,7 +29489,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29463,7 +29497,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.013095</v>
+        <v>0.012459</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29487,7 +29521,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>96.84</v>
+        <v>99.2</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29495,7 +29529,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29503,7 +29537,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>102.322216</v>
+        <v>97.13801100000001</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29527,7 +29561,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.86</v>
+        <v>1.93</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29535,7 +29569,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29543,7 +29577,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.98936</v>
+        <v>1.865897</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29575,7 +29609,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29607,7 +29641,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.022729</v>
+        <v>0.023329</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29615,7 +29649,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29623,7 +29657,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.024189</v>
+        <v>0.022799</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29647,7 +29681,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>4.996127</v>
+        <v>5.591177</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29655,7 +29689,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29663,7 +29697,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>4.468399</v>
+        <v>5.007568</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29687,7 +29721,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>22.812874</v>
+        <v>23.893954</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29695,7 +29729,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29703,7 +29737,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>23.928266</v>
+        <v>22.966162</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29727,7 +29761,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.131654</v>
+        <v>0.133518</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29735,7 +29769,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29743,7 +29777,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.142014</v>
+        <v>0.132388</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29767,7 +29801,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>23699.3536</v>
+        <v>24265.9966</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29775,7 +29809,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29783,7 +29817,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>23951.109502</v>
+        <v>23816.782049</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29807,7 +29841,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2518330.88</v>
+        <v>2554873.94</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29815,7 +29849,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29823,7 +29857,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2593653.090879</v>
+        <v>2530125.214568</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29847,7 +29881,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.65804</v>
+        <v>2.704105</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29855,7 +29889,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29863,7 +29897,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.787503</v>
+        <v>2.675416</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29887,7 +29921,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>79803.44319999999</v>
+        <v>81165.51730000001</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29895,7 +29929,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29903,7 +29937,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>83629.01332899999</v>
+        <v>80222.109148</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29927,7 +29961,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>19.727352</v>
+        <v>19.777431</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -29935,7 +29969,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -29943,7 +29977,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.094738</v>
+        <v>19.813636</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -29967,7 +30001,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>75671</v>
+        <v>76562</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -29975,7 +30009,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -29983,7 +30017,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>77934.287587</v>
+        <v>75820.35404799999</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30007,7 +30041,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>18.76</v>
+        <v>19.16</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30015,7 +30049,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30023,7 +30057,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>19.554105</v>
+        <v>18.800261</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30121,7 +30155,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.006814</v>
+        <v>0.007018</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30129,7 +30163,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30137,7 +30171,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007128</v>
+        <v>0.006853</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30161,7 +30195,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>96.84</v>
+        <v>99.2</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30169,7 +30203,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30177,7 +30211,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>102.322216</v>
+        <v>97.13801100000001</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30209,7 +30243,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30241,27 +30275,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.627</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46276</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.0869</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46275</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.3998</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-18
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L113"/>
+  <dimension ref="B2:L114"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25239,6 +25239,40 @@
         <v>33.37</v>
       </c>
       <c r="K113" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="72" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C114" t="n">
+        <v>26081652</v>
+      </c>
+      <c r="D114" t="n">
+        <v>22831314</v>
+      </c>
+      <c r="E114" t="n">
+        <v>3250338</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0.1424</v>
+      </c>
+      <c r="G114" t="n">
+        <v>18342757</v>
+      </c>
+      <c r="H114" t="n">
+        <v>4907064</v>
+      </c>
+      <c r="I114" t="n">
+        <v>1463593</v>
+      </c>
+      <c r="J114" t="n">
+        <v>33.22</v>
+      </c>
+      <c r="K114" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25816,7 +25850,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25831,11 +25865,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.37</v>
+        <v>33.22</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-17</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -25880,11 +25914,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1457</v>
+        <v>26.0595</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-17</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -25999,27 +26033,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>18.9065</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>18.8659</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>19.9564</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26044,27 +26078,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7037</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7035</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7033</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26089,27 +26123,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.4015</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.4342</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.3992</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26134,27 +26168,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.363099999999999</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.420400000000001</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.509399999999999</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26179,27 +26213,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.515700000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.5448</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.6075</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26224,27 +26258,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>12.9886</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.0836</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>12.9564</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26269,27 +26303,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>14.9009</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.0984</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.0292</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26314,27 +26348,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>28.4866</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>28.7218</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>28.7847</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26359,27 +26393,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>35.8364</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.2026</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.4572</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26404,27 +26438,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.9418</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.1505</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.2295</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26449,27 +26483,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.3313</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.0949</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.0809</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26494,27 +26528,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>80.6232</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.4216</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.8845</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26539,7 +26573,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>54.6456</v>
+        <v>54.0841</v>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -26547,7 +26581,7 @@
         </is>
       </c>
       <c r="G17" s="28" t="n">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
@@ -26555,11 +26589,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.8345</v>
+        <v>54.5141</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26584,27 +26618,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4882</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4974</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5078</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26629,27 +26663,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4468</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4463</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4459</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26674,27 +26708,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.309</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.4936</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.6729</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26719,27 +26753,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.5025</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.4127</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.5698</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26764,27 +26798,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9246</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0344</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.9551</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26809,27 +26843,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.0329</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.1696</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.1753</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26854,27 +26888,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.4446</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.3892</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.5536</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26899,27 +26933,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.8544</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.858700000000001</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.7195</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26944,27 +26978,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.8281</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.8314</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.6354</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26989,27 +27023,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.254</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.2171</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27034,27 +27068,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.0241</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.7589</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.9136</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27079,27 +27113,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>23.7286</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>23.6884</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.3625</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27124,27 +27158,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>33.9117</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>33.9841</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>35.8478</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27169,27 +27203,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9644</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.0952</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.1923</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27214,27 +27248,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7213</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7211</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7209</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27259,27 +27293,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.7759</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.924</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.9865</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27304,27 +27338,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2381</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2378</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2374</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27349,27 +27383,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.2534</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.1131</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46279</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.3577</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27394,27 +27428,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.979699999999999</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>9.9908</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0188</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27439,27 +27473,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.0448</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.3241</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.4228</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27484,7 +27518,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.27</v>
+        <v>22.1</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27492,7 +27526,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27500,7 +27534,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.1</v>
+        <v>22.23</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27524,7 +27558,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.055</v>
+        <v>1.064</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27532,7 +27566,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27540,7 +27574,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.064</v>
+        <v>1.059</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27564,7 +27598,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>737.91</v>
+        <v>739.99</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27572,7 +27606,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27580,7 +27614,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>739.98999</v>
+        <v>751.159973</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27612,7 +27646,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27652,7 +27686,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27660,7 +27694,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>205.710007</v>
+        <v>205.809998</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27684,23 +27718,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.7</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.6</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27724,23 +27758,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>193</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>192</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>192.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27764,7 +27798,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -27772,7 +27806,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27780,7 +27814,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -27812,7 +27846,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27889,7 +27923,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27921,23 +27955,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>61</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>60.25</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>61</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -27961,7 +27995,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -27969,7 +28003,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -27977,7 +28011,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.7</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28001,7 +28035,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16</v>
+        <v>16.2</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28009,7 +28043,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28041,7 +28075,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28049,7 +28083,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28057,7 +28091,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>14.9</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28081,7 +28115,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.55</v>
+        <v>5.6</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28089,7 +28123,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28097,7 +28131,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.55</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28121,7 +28155,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.5</v>
+        <v>22.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28129,7 +28163,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28161,7 +28195,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28169,7 +28203,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28177,7 +28211,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28209,7 +28243,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28241,7 +28275,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.18</v>
+        <v>3.3</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28249,7 +28283,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28257,7 +28291,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.18</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28281,7 +28315,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28289,7 +28323,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28297,7 +28331,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28321,7 +28355,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28329,7 +28363,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28361,23 +28395,23 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="F60" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G60" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H60" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
         <v>103.75</v>
-      </c>
-      <c r="F60" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G60" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H60" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I60" t="n">
-        <v>105.040001</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28401,23 +28435,23 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
+        <v>252.67</v>
+      </c>
+      <c r="F61" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G61" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H61" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
         <v>250.5</v>
-      </c>
-      <c r="F61" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G61" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H61" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I61" t="n">
-        <v>257.76001</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28441,7 +28475,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>415.38</v>
+        <v>417.4</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28449,7 +28483,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28481,23 +28515,23 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
+        <v>120.37</v>
+      </c>
+      <c r="F63" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G63" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H63" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
         <v>118</v>
-      </c>
-      <c r="F63" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G63" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H63" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I63" t="n">
-        <v>122.209999</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28521,7 +28555,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>35.56</v>
+        <v>36.02</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28529,7 +28563,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28537,7 +28571,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>36.720001</v>
+        <v>35.560001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28561,7 +28595,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>175.54</v>
+        <v>182.39</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28569,7 +28603,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28601,7 +28635,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>171.77</v>
+        <v>172.58</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28609,7 +28643,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28641,7 +28675,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>191.57</v>
+        <v>187.8</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28649,7 +28683,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28681,7 +28715,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>167.36</v>
+        <v>168.98</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28689,7 +28723,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28721,7 +28755,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1137.82</v>
+        <v>1152.44</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28729,7 +28763,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28761,7 +28795,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>69.59</v>
+        <v>70.81999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28769,7 +28803,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28801,7 +28835,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1147.61</v>
+        <v>1169.58</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28809,7 +28843,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28841,7 +28875,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>165.19</v>
+        <v>154.65</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28849,7 +28883,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28881,7 +28915,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>213.9</v>
+        <v>219.34</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -28889,7 +28923,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28921,7 +28955,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>76.30500000000001</v>
+        <v>77.33</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -28929,7 +28963,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28961,7 +28995,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>113.97</v>
+        <v>119.51</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -28969,7 +29003,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -28977,7 +29011,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>118.059998</v>
+        <v>113.970001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29001,7 +29035,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>341.15</v>
+        <v>353.13</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29009,7 +29043,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29041,7 +29075,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>358.08</v>
+        <v>366.2</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29049,7 +29083,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29081,7 +29115,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>40.67</v>
+        <v>40.11</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29089,7 +29123,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29097,7 +29131,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>41.580002</v>
+        <v>40.669998</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29121,7 +29155,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>67.61</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29129,7 +29163,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29161,7 +29195,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>332.41</v>
+        <v>337</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29169,7 +29203,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29201,7 +29235,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>164.51</v>
+        <v>173.97</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29209,7 +29243,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29217,7 +29251,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>172.110001</v>
+        <v>164.509995</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29241,7 +29275,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>673.3099999999999</v>
+        <v>682.3099999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29249,7 +29283,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29257,7 +29291,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>670.23999</v>
+        <v>673.309998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29281,7 +29315,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.39</v>
+        <v>31.17</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29289,7 +29323,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29297,7 +29331,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.389999</v>
+        <v>31.17</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29321,7 +29355,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>121.58</v>
+        <v>129.39</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29329,7 +29363,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29337,7 +29371,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>121.721319</v>
+        <v>121.6696</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29361,7 +29395,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>727.1799999999999</v>
+        <v>740.5700000000001</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29369,7 +29403,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29377,7 +29411,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>713.718371</v>
+        <v>727.666543</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29401,7 +29435,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>76562</v>
+        <v>76523</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29409,7 +29443,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29417,7 +29451,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>75820.35404799999</v>
+        <v>76567.918028</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29441,7 +29475,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007018</v>
+        <v>0.007353</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29449,7 +29483,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29457,7 +29491,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.006853</v>
+        <v>0.007028</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29481,7 +29515,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.012468</v>
+        <v>0.013268</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29489,7 +29523,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29497,7 +29531,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.012459</v>
+        <v>0.012484</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29521,7 +29555,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>99.2</v>
+        <v>101.68</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29529,7 +29563,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29537,7 +29571,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>97.13801100000001</v>
+        <v>99.273984</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29561,7 +29595,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.93</v>
+        <v>1.98</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29569,7 +29603,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29577,7 +29611,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.865897</v>
+        <v>1.936688</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29609,7 +29643,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29641,7 +29675,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.023329</v>
+        <v>0.024876</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29649,7 +29683,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29657,7 +29691,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.022799</v>
+        <v>0.023354</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29681,7 +29715,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>5.591177</v>
+        <v>6.084675</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29689,7 +29723,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29697,7 +29731,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>5.007568</v>
+        <v>5.573195</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29721,7 +29755,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>23.893954</v>
+        <v>24.997718</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29729,7 +29763,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29737,7 +29771,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>22.966162</v>
+        <v>23.835947</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29761,7 +29795,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.133518</v>
+        <v>0.133709</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29769,7 +29803,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29777,7 +29811,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.132388</v>
+        <v>0.132826</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29801,7 +29835,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>24265.9966</v>
+        <v>24601.7354</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29809,7 +29843,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29817,7 +29851,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>23816.782049</v>
+        <v>24173.082561</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29841,7 +29875,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2554873.94</v>
+        <v>2542094.06</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29849,7 +29883,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29857,7 +29891,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2530125.214568</v>
+        <v>2543586.236906</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29881,7 +29915,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.704105</v>
+        <v>2.722911</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29889,7 +29923,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29897,7 +29931,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.675416</v>
+        <v>2.693829</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29921,7 +29955,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>81165.51730000001</v>
+        <v>81338.1734</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29929,7 +29963,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29937,7 +29971,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>80222.109148</v>
+        <v>80909.63725699999</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29961,7 +29995,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>19.777431</v>
+        <v>19.871639</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -29969,7 +30003,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -29977,7 +30011,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>19.813636</v>
+        <v>19.690237</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30001,7 +30035,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>76562</v>
+        <v>76523</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30009,7 +30043,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30017,7 +30051,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>75820.35404799999</v>
+        <v>76567.918028</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30041,7 +30075,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>19.16</v>
+        <v>19.58</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30049,7 +30083,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30057,7 +30091,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>18.800261</v>
+        <v>19.179383</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30155,7 +30189,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007018</v>
+        <v>0.007353</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30163,7 +30197,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30171,7 +30205,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.006853</v>
+        <v>0.007028</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30195,7 +30229,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>99.2</v>
+        <v>101.68</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30203,7 +30237,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30211,7 +30245,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>97.13801100000001</v>
+        <v>99.273984</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30243,7 +30277,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30275,27 +30309,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.15</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46279</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.627</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46276</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.0869</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-19
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L114"/>
+  <dimension ref="B2:L115"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25273,6 +25273,40 @@
         <v>33.22</v>
       </c>
       <c r="K114" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="72" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C115" t="n">
+        <v>26600915</v>
+      </c>
+      <c r="D115" t="n">
+        <v>22839842</v>
+      </c>
+      <c r="E115" t="n">
+        <v>3761073</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.1647</v>
+      </c>
+      <c r="G115" t="n">
+        <v>18746611</v>
+      </c>
+      <c r="H115" t="n">
+        <v>4924493</v>
+      </c>
+      <c r="I115" t="n">
+        <v>1550772</v>
+      </c>
+      <c r="J115" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="K115" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25850,7 +25884,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25865,11 +25899,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.22</v>
+        <v>33.29</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-18</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -25914,11 +25948,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.0595</v>
+        <v>26.1044</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-18</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -26033,7 +26067,7 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
-        <v>18.9065</v>
+        <v>18.8659</v>
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
@@ -26041,7 +26075,7 @@
         </is>
       </c>
       <c r="G5" s="28" t="n">
-        <v>46280</v>
+        <v>46279</v>
       </c>
       <c r="H5" s="34" t="inlineStr">
         <is>
@@ -26184,11 +26218,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8.420400000000001</v>
+        <v>8.6533</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-09</t>
         </is>
       </c>
     </row>
@@ -26213,7 +26247,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.515700000000001</v>
+        <v>9.6021</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26221,7 +26255,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26229,11 +26263,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9.5448</v>
+        <v>9.673999999999999</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -26258,7 +26292,7 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
-        <v>12.9886</v>
+        <v>13.4336</v>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
@@ -26266,7 +26300,7 @@
         </is>
       </c>
       <c r="G10" s="28" t="n">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="H10" s="34" t="inlineStr">
         <is>
@@ -26303,7 +26337,7 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>14.9009</v>
+        <v>15.0292</v>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -26311,7 +26345,7 @@
         </is>
       </c>
       <c r="G11" s="28" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
@@ -26438,7 +26472,7 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
-        <v>25.9418</v>
+        <v>26.2295</v>
       </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
@@ -26446,7 +26480,7 @@
         </is>
       </c>
       <c r="G14" s="28" t="n">
-        <v>46281</v>
+        <v>46279</v>
       </c>
       <c r="H14" s="34" t="inlineStr">
         <is>
@@ -26483,7 +26517,7 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
-        <v>16.3313</v>
+        <v>16.2087</v>
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
@@ -26491,7 +26525,7 @@
         </is>
       </c>
       <c r="G15" s="28" t="n">
-        <v>46279</v>
+        <v>46274</v>
       </c>
       <c r="H15" s="34" t="inlineStr">
         <is>
@@ -26499,11 +26533,11 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>16.0949</v>
+        <v>16.3462</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -26528,7 +26562,7 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
-        <v>80.6232</v>
+        <v>81.5758</v>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
@@ -26536,7 +26570,7 @@
         </is>
       </c>
       <c r="G16" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
@@ -26544,11 +26578,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>81.4216</v>
+        <v>83.035</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26573,7 +26607,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>54.0841</v>
+        <v>54.5141</v>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -26581,7 +26615,7 @@
         </is>
       </c>
       <c r="G17" s="28" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
@@ -26589,11 +26623,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.5141</v>
+        <v>55.1703</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
@@ -26618,27 +26652,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5005</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4882</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4974</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26663,27 +26697,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4472</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4468</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4463</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26708,7 +26742,7 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
-        <v>41.309</v>
+        <v>41.6729</v>
       </c>
       <c r="F20" s="34" t="inlineStr">
         <is>
@@ -26716,7 +26750,7 @@
         </is>
       </c>
       <c r="G20" s="28" t="n">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="H20" s="34" t="inlineStr">
         <is>
@@ -26724,11 +26758,11 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>41.4936</v>
+        <v>41.7417</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-08</t>
         </is>
       </c>
     </row>
@@ -26798,7 +26832,7 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
-        <v>13.9246</v>
+        <v>14.0081</v>
       </c>
       <c r="F22" s="34" t="inlineStr">
         <is>
@@ -26806,7 +26840,7 @@
         </is>
       </c>
       <c r="G22" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H22" s="34" t="inlineStr">
         <is>
@@ -26843,7 +26877,7 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>13.0329</v>
+        <v>13.3018</v>
       </c>
       <c r="F23" s="34" t="inlineStr">
         <is>
@@ -26851,7 +26885,7 @@
         </is>
       </c>
       <c r="G23" s="28" t="n">
-        <v>46281</v>
+        <v>46274</v>
       </c>
       <c r="H23" s="34" t="inlineStr">
         <is>
@@ -26888,7 +26922,7 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
-        <v>11.4446</v>
+        <v>16.6955</v>
       </c>
       <c r="F24" s="34" t="inlineStr">
         <is>
@@ -26896,7 +26930,7 @@
         </is>
       </c>
       <c r="G24" s="28" t="n">
-        <v>46280</v>
+        <v>46276</v>
       </c>
       <c r="H24" s="34" t="inlineStr">
         <is>
@@ -26904,11 +26938,11 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>11.3892</v>
+        <v>15.3452</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26933,27 +26967,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.9785</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.8544</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.858700000000001</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27023,7 +27057,7 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>18.06</v>
+        <v>18.5131</v>
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
@@ -27031,7 +27065,7 @@
         </is>
       </c>
       <c r="G27" s="28" t="n">
-        <v>46281</v>
+        <v>46273</v>
       </c>
       <c r="H27" s="34" t="inlineStr">
         <is>
@@ -27068,7 +27102,7 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
-        <v>19.0241</v>
+        <v>18.9562</v>
       </c>
       <c r="F28" s="34" t="inlineStr">
         <is>
@@ -27076,7 +27110,7 @@
         </is>
       </c>
       <c r="G28" s="28" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="H28" s="34" t="inlineStr">
         <is>
@@ -27113,7 +27147,7 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>23.7286</v>
+        <v>23.5912</v>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
@@ -27121,7 +27155,7 @@
         </is>
       </c>
       <c r="G29" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H29" s="34" t="inlineStr">
         <is>
@@ -27158,7 +27192,7 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
-        <v>33.9117</v>
+        <v>34.4558</v>
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
@@ -27166,7 +27200,7 @@
         </is>
       </c>
       <c r="G30" s="28" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="H30" s="34" t="inlineStr">
         <is>
@@ -27203,7 +27237,7 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>12.9644</v>
+        <v>13.0952</v>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
@@ -27211,7 +27245,7 @@
         </is>
       </c>
       <c r="G31" s="28" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="H31" s="34" t="inlineStr">
         <is>
@@ -27248,27 +27282,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7215</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7213</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7211</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27293,7 +27327,7 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>12.7759</v>
+        <v>13.1708</v>
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
@@ -27301,7 +27335,7 @@
         </is>
       </c>
       <c r="G33" s="28" t="n">
-        <v>46281</v>
+        <v>46274</v>
       </c>
       <c r="H33" s="34" t="inlineStr">
         <is>
@@ -27338,27 +27372,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2385</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2381</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2378</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27383,7 +27417,7 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>28.2534</v>
+        <v>28.5269</v>
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
@@ -27391,7 +27425,7 @@
         </is>
       </c>
       <c r="G35" s="28" t="n">
-        <v>46280</v>
+        <v>46274</v>
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
@@ -27428,7 +27462,7 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
-        <v>9.979699999999999</v>
+        <v>10.0128</v>
       </c>
       <c r="F36" s="34" t="inlineStr">
         <is>
@@ -27436,7 +27470,7 @@
         </is>
       </c>
       <c r="G36" s="28" t="n">
-        <v>46281</v>
+        <v>46276</v>
       </c>
       <c r="H36" s="34" t="inlineStr">
         <is>
@@ -27444,11 +27478,11 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>9.9908</v>
+        <v>10.1337</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>
@@ -27473,7 +27507,7 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>23.0448</v>
+        <v>23.3241</v>
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
@@ -27481,7 +27515,7 @@
         </is>
       </c>
       <c r="G37" s="28" t="n">
-        <v>46281</v>
+        <v>46280</v>
       </c>
       <c r="H37" s="34" t="inlineStr">
         <is>
@@ -27489,11 +27523,11 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>23.3241</v>
+        <v>23.7242</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27518,7 +27552,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.1</v>
+        <v>22.23</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27526,7 +27560,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27534,7 +27568,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.23</v>
+        <v>22.08</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27558,7 +27592,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.064</v>
+        <v>1.059</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27566,7 +27600,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27574,7 +27608,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.059</v>
+        <v>1.069</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27598,7 +27632,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>739.99</v>
+        <v>751.16</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27606,7 +27640,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27614,7 +27648,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>751.159973</v>
+        <v>754.940002</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27646,7 +27680,7 @@
         </is>
       </c>
       <c r="G41" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
@@ -27678,7 +27712,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>205.71</v>
+        <v>205.81</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27686,7 +27720,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27694,7 +27728,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>205.809998</v>
+        <v>207.360001</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27726,7 +27760,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27734,7 +27768,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27758,23 +27792,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>193.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>193</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>192</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27798,7 +27832,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -27806,7 +27840,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27814,7 +27848,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -27838,7 +27872,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -27846,7 +27880,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27923,7 +27957,7 @@
         </is>
       </c>
       <c r="G48" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
@@ -27955,23 +27989,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>61.25</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>61</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>60.25</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28003,7 +28037,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28035,7 +28069,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28043,7 +28077,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28051,7 +28085,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.200001</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28075,7 +28109,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28083,7 +28117,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28091,7 +28125,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.1</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28115,7 +28149,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.6</v>
+        <v>5.75</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28123,7 +28157,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28155,7 +28189,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28163,7 +28197,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28171,7 +28205,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.799999</v>
+        <v>22.700001</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28203,7 +28237,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28235,7 +28269,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.48</v>
+        <v>4.46</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28243,7 +28277,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28251,7 +28285,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.48</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28275,7 +28309,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28283,7 +28317,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28291,7 +28325,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28315,7 +28349,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28323,7 +28357,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28331,7 +28365,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28355,7 +28389,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28363,7 +28397,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28371,7 +28405,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.9</v>
+        <v>17.799999</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28395,7 +28429,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>104.6</v>
+        <v>109.32</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28403,7 +28437,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28411,7 +28445,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>103.75</v>
+        <v>109.32</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28435,7 +28469,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>252.67</v>
+        <v>248.92</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28443,7 +28477,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28451,7 +28485,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>250.5</v>
+        <v>248.919998</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28475,7 +28509,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>417.4</v>
+        <v>444.57</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28483,7 +28517,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28491,7 +28525,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>415.380005</v>
+        <v>444.570007</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28515,7 +28549,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>120.37</v>
+        <v>118.82</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28523,7 +28557,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28531,7 +28565,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>118</v>
+        <v>118.82</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28555,23 +28589,23 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
+        <v>34.64</v>
+      </c>
+      <c r="F64" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G64" s="28" t="n">
+        <v>46284</v>
+      </c>
+      <c r="H64" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
         <v>36.02</v>
-      </c>
-      <c r="F64" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G64" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H64" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I64" t="n">
-        <v>35.560001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28595,7 +28629,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>182.39</v>
+        <v>181.31</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28603,7 +28637,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28611,7 +28645,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>175.539993</v>
+        <v>181.309998</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28635,7 +28669,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>172.58</v>
+        <v>169.84</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28643,7 +28677,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28651,7 +28685,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>171.770004</v>
+        <v>169.839996</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28675,7 +28709,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>187.8</v>
+        <v>185.78</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28683,7 +28717,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28691,7 +28725,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>191.570007</v>
+        <v>185.779999</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28715,7 +28749,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>168.98</v>
+        <v>176.99</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28723,7 +28757,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28731,7 +28765,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>167.360001</v>
+        <v>176.990005</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28755,7 +28789,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1152.44</v>
+        <v>1152.93</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28763,7 +28797,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28771,7 +28805,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1137.819946</v>
+        <v>1152.930054</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28795,7 +28829,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>70.81999999999999</v>
+        <v>73.27</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28803,7 +28837,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28811,7 +28845,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>69.589996</v>
+        <v>73.269997</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -28835,7 +28869,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1169.58</v>
+        <v>1217.8</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28843,7 +28877,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28851,7 +28885,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1147.609985</v>
+        <v>1217.800049</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -28875,7 +28909,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>154.65</v>
+        <v>154.91</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28883,7 +28917,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28891,7 +28925,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>165.190002</v>
+        <v>154.910004</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -28915,7 +28949,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>219.34</v>
+        <v>222.27</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -28923,7 +28957,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28931,7 +28965,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>213.899994</v>
+        <v>222.270004</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -28955,7 +28989,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.33</v>
+        <v>78.3</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -28963,7 +28997,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -28971,7 +29005,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>76.30999799999999</v>
+        <v>78.300003</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -28995,7 +29029,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>119.51</v>
+        <v>117.18</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29003,7 +29037,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29011,7 +29045,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>113.970001</v>
+        <v>119.510002</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29035,7 +29069,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>353.13</v>
+        <v>371.47</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29043,7 +29077,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29051,7 +29085,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>341.149994</v>
+        <v>371.470001</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29075,7 +29109,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>366.2</v>
+        <v>364.27</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29083,7 +29117,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29091,7 +29125,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>358.079987</v>
+        <v>364.269989</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29115,7 +29149,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>40.11</v>
+        <v>38.1</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29123,7 +29157,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29131,7 +29165,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>40.669998</v>
+        <v>40.110001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29155,7 +29189,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>69.09999999999999</v>
+        <v>69.06</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29163,7 +29197,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29171,7 +29205,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>67.610001</v>
+        <v>69.05999799999999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29195,7 +29229,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>337</v>
+        <v>336.13</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29203,7 +29237,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29211,7 +29245,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>332.410004</v>
+        <v>336.130005</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29235,7 +29269,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>173.97</v>
+        <v>194.25</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29243,7 +29277,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29251,7 +29285,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>164.509995</v>
+        <v>173.970001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29275,7 +29309,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>682.3099999999999</v>
+        <v>665.75</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29283,7 +29317,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29291,7 +29325,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>673.309998</v>
+        <v>682.309998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29315,7 +29349,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>31.17</v>
+        <v>31.41</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29323,7 +29357,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29331,7 +29365,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>31.17</v>
+        <v>31.41</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29355,7 +29389,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>129.39</v>
+        <v>140.41</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29363,7 +29397,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29371,7 +29405,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>121.6696</v>
+        <v>129.516159</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29395,7 +29429,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>740.5700000000001</v>
+        <v>763.15</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29403,7 +29437,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29411,7 +29445,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>727.666543</v>
+        <v>741.018587</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29435,7 +29469,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>76523</v>
+        <v>81291</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29443,7 +29477,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29451,7 +29485,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>76567.918028</v>
+        <v>76527.29248400001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29475,7 +29509,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007353</v>
+        <v>0.00788</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29483,7 +29517,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29491,7 +29525,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007028</v>
+        <v>0.007378</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29515,7 +29549,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.013268</v>
+        <v>0.014208</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29523,7 +29557,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29531,7 +29565,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.012484</v>
+        <v>0.013278</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29555,7 +29589,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>101.68</v>
+        <v>113.43</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29563,7 +29597,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29571,7 +29605,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>99.273984</v>
+        <v>101.722237</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29595,7 +29629,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.98</v>
+        <v>2.06</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29603,7 +29637,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29611,7 +29645,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.936688</v>
+        <v>1.981949</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29643,7 +29677,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29675,7 +29709,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.024876</v>
+        <v>0.027246</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29683,7 +29717,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29691,7 +29725,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.023354</v>
+        <v>0.024888</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29715,7 +29749,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.084675</v>
+        <v>7.252093</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29723,7 +29757,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29731,7 +29765,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>5.573195</v>
+        <v>6.096772</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29755,7 +29789,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>24.997718</v>
+        <v>27.088339</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29763,7 +29797,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29771,7 +29805,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>23.835947</v>
+        <v>25.050637</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29795,7 +29829,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.133709</v>
+        <v>0.143433</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29803,7 +29837,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29811,7 +29845,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.132826</v>
+        <v>0.13423</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29835,7 +29869,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>24601.7354</v>
+        <v>25405.2635</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29843,7 +29877,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29851,7 +29885,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>24173.082561</v>
+        <v>24668.508761</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29875,7 +29909,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2542094.06</v>
+        <v>2706177.39</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29883,7 +29917,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29891,7 +29925,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2543586.236906</v>
+        <v>2547593.566789</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29915,7 +29949,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.722911</v>
+        <v>2.923728</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29923,7 +29957,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29931,7 +29965,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.693829</v>
+        <v>2.730043</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29955,7 +29989,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>81338.1734</v>
+        <v>86986.4371</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29963,7 +29997,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -29971,7 +30005,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>80909.63725699999</v>
+        <v>81528.721494</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -29995,7 +30029,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>19.871639</v>
+        <v>20.277039</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30003,7 +30037,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30011,7 +30045,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>19.690237</v>
+        <v>19.851612</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30035,7 +30069,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>76523</v>
+        <v>81291</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30043,7 +30077,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30051,7 +30085,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>76567.918028</v>
+        <v>76527.29248400001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30075,7 +30109,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>19.58</v>
+        <v>20.94</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30083,7 +30117,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30091,7 +30125,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>19.179383</v>
+        <v>19.580795</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30189,7 +30223,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007353</v>
+        <v>0.00788</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30197,7 +30231,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30205,7 +30239,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007028</v>
+        <v>0.007378</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30229,7 +30263,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>101.68</v>
+        <v>113.43</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30237,7 +30271,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30245,7 +30279,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>99.273984</v>
+        <v>101.722237</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30277,7 +30311,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30309,7 +30343,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>24.15</v>
+        <v>24.0972</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -30317,7 +30351,7 @@
         </is>
       </c>
       <c r="G108" s="47" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-20
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L115"/>
+  <dimension ref="B2:L116"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25307,6 +25307,40 @@
         <v>33.29</v>
       </c>
       <c r="K115" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="72" t="n">
+        <v>46285</v>
+      </c>
+      <c r="C116" t="n">
+        <v>26457758</v>
+      </c>
+      <c r="D116" t="n">
+        <v>22839842</v>
+      </c>
+      <c r="E116" t="n">
+        <v>3617916</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0.1584</v>
+      </c>
+      <c r="G116" t="n">
+        <v>18606006</v>
+      </c>
+      <c r="H116" t="n">
+        <v>4924493</v>
+      </c>
+      <c r="I116" t="n">
+        <v>1548220</v>
+      </c>
+      <c r="J116" t="n">
+        <v>33.29</v>
+      </c>
+      <c r="K116" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25884,7 +25918,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25903,7 +25937,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-19</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-20</t>
         </is>
       </c>
     </row>
@@ -25952,7 +25986,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-19</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-20</t>
         </is>
       </c>
     </row>
@@ -26067,7 +26101,7 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
-        <v>18.8659</v>
+        <v>19.7228</v>
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
@@ -26075,7 +26109,7 @@
         </is>
       </c>
       <c r="G5" s="28" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="H5" s="34" t="inlineStr">
         <is>
@@ -26083,11 +26117,11 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>18.8659</v>
+        <v>19.2267</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26112,7 +26146,7 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>10.7037</v>
+        <v>10.7039</v>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -26120,7 +26154,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -26128,11 +26162,11 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10.7035</v>
+        <v>10.7039</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26157,7 +26191,7 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
-        <v>7.4015</v>
+        <v>7.4649</v>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
@@ -26165,7 +26199,7 @@
         </is>
       </c>
       <c r="G7" s="28" t="n">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
@@ -26177,7 +26211,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26202,7 +26236,7 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
-        <v>8.363099999999999</v>
+        <v>8.4726</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
@@ -26210,7 +26244,7 @@
         </is>
       </c>
       <c r="G8" s="28" t="n">
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
@@ -26218,11 +26252,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8.6533</v>
+        <v>8.475</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26255,7 +26289,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26263,11 +26297,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9.673999999999999</v>
+        <v>9.6021</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26292,7 +26326,7 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
-        <v>13.4336</v>
+        <v>13.1751</v>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
@@ -26300,7 +26334,7 @@
         </is>
       </c>
       <c r="G10" s="28" t="n">
-        <v>46272</v>
+        <v>46282</v>
       </c>
       <c r="H10" s="34" t="inlineStr">
         <is>
@@ -26308,11 +26342,11 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>13.0836</v>
+        <v>13.0852</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26337,7 +26371,7 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>15.0292</v>
+        <v>15.1584</v>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -26345,7 +26379,7 @@
         </is>
       </c>
       <c r="G11" s="28" t="n">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
@@ -26353,11 +26387,11 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>15.0984</v>
+        <v>15.104</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26382,7 +26416,7 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
-        <v>28.4866</v>
+        <v>28.8544</v>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
@@ -26390,7 +26424,7 @@
         </is>
       </c>
       <c r="G12" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H12" s="34" t="inlineStr">
         <is>
@@ -26398,11 +26432,11 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>28.7218</v>
+        <v>28.8573</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26427,7 +26461,7 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
-        <v>35.8364</v>
+        <v>36.2634</v>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
@@ -26435,7 +26469,7 @@
         </is>
       </c>
       <c r="G13" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H13" s="34" t="inlineStr">
         <is>
@@ -26443,11 +26477,11 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>36.2026</v>
+        <v>36.2622</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26472,7 +26506,7 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
-        <v>26.2295</v>
+        <v>26.1664</v>
       </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
@@ -26480,7 +26514,7 @@
         </is>
       </c>
       <c r="G14" s="28" t="n">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="H14" s="34" t="inlineStr">
         <is>
@@ -26488,11 +26522,11 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>26.1505</v>
+        <v>26.1666</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26517,7 +26551,7 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
-        <v>16.2087</v>
+        <v>16.1811</v>
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
@@ -26525,7 +26559,7 @@
         </is>
       </c>
       <c r="G15" s="28" t="n">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="H15" s="34" t="inlineStr">
         <is>
@@ -26533,11 +26567,11 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>16.3462</v>
+        <v>16.1916</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26562,27 +26596,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.62779999999999</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>81.5758</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>83.035</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26607,7 +26641,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>54.5141</v>
+        <v>54.6003</v>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -26615,7 +26649,7 @@
         </is>
       </c>
       <c r="G17" s="28" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
@@ -26623,11 +26657,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>55.1703</v>
+        <v>54.5904</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26652,27 +26686,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.519</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5005</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4882</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26697,27 +26731,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4473</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4472</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4468</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26742,7 +26776,7 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
-        <v>41.6729</v>
+        <v>41.5907</v>
       </c>
       <c r="F20" s="34" t="inlineStr">
         <is>
@@ -26750,7 +26784,7 @@
         </is>
       </c>
       <c r="G20" s="28" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="H20" s="34" t="inlineStr">
         <is>
@@ -26758,11 +26792,11 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>41.7417</v>
+        <v>41.1276</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26787,7 +26821,7 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
-        <v>12.5025</v>
+        <v>12.5598</v>
       </c>
       <c r="F21" s="34" t="inlineStr">
         <is>
@@ -26795,7 +26829,7 @@
         </is>
       </c>
       <c r="G21" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H21" s="34" t="inlineStr">
         <is>
@@ -26803,11 +26837,11 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>12.4127</v>
+        <v>12.4633</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26832,27 +26866,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0819</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0081</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0344</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26877,7 +26911,7 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>13.3018</v>
+        <v>13.1818</v>
       </c>
       <c r="F23" s="34" t="inlineStr">
         <is>
@@ -26885,7 +26919,7 @@
         </is>
       </c>
       <c r="G23" s="28" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="H23" s="34" t="inlineStr">
         <is>
@@ -26893,11 +26927,11 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>13.1696</v>
+        <v>13.1766</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26922,7 +26956,7 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
-        <v>16.6955</v>
+        <v>11.5822</v>
       </c>
       <c r="F24" s="34" t="inlineStr">
         <is>
@@ -26930,7 +26964,7 @@
         </is>
       </c>
       <c r="G24" s="28" t="n">
-        <v>46276</v>
+        <v>46282</v>
       </c>
       <c r="H24" s="34" t="inlineStr">
         <is>
@@ -26938,11 +26972,11 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>15.3452</v>
+        <v>11.5024</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26967,27 +27001,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.8436</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.9785</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8544</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27012,7 +27046,7 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
-        <v>13.8281</v>
+        <v>13.7976</v>
       </c>
       <c r="F26" s="34" t="inlineStr">
         <is>
@@ -27020,7 +27054,7 @@
         </is>
       </c>
       <c r="G26" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H26" s="34" t="inlineStr">
         <is>
@@ -27028,11 +27062,11 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>13.8314</v>
+        <v>13.9987</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27057,7 +27091,7 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>18.5131</v>
+        <v>18.357</v>
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
@@ -27065,7 +27099,7 @@
         </is>
       </c>
       <c r="G27" s="28" t="n">
-        <v>46273</v>
+        <v>46283</v>
       </c>
       <c r="H27" s="34" t="inlineStr">
         <is>
@@ -27073,11 +27107,11 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>18.254</v>
+        <v>18.2902</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27102,27 +27136,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.3116</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.9562</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.7589</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27147,27 +27181,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.5262</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>23.5912</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>23.6884</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27192,27 +27226,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>35.1929</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>34.4558</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>33.9841</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27237,7 +27271,7 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>13.0952</v>
+        <v>13.1495</v>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
@@ -27245,7 +27279,7 @@
         </is>
       </c>
       <c r="G31" s="28" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="H31" s="34" t="inlineStr">
         <is>
@@ -27253,11 +27287,11 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>13.0952</v>
+        <v>13.144</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27290,7 +27324,7 @@
         </is>
       </c>
       <c r="G32" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H32" s="34" t="inlineStr">
         <is>
@@ -27298,11 +27332,11 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>21.7213</v>
+        <v>21.7215</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27327,7 +27361,7 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>13.1708</v>
+        <v>12.9572</v>
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
@@ -27335,7 +27369,7 @@
         </is>
       </c>
       <c r="G33" s="28" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="H33" s="34" t="inlineStr">
         <is>
@@ -27343,11 +27377,11 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>12.924</v>
+        <v>12.9269</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27372,27 +27406,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2386</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2385</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2381</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27417,7 +27451,7 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>28.5269</v>
+        <v>28.597</v>
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
@@ -27425,7 +27459,7 @@
         </is>
       </c>
       <c r="G35" s="28" t="n">
-        <v>46274</v>
+        <v>46282</v>
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
@@ -27433,11 +27467,11 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>28.1131</v>
+        <v>28.0542</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27462,7 +27496,7 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
-        <v>10.0128</v>
+        <v>10.0938</v>
       </c>
       <c r="F36" s="34" t="inlineStr">
         <is>
@@ -27470,7 +27504,7 @@
         </is>
       </c>
       <c r="G36" s="28" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="H36" s="34" t="inlineStr">
         <is>
@@ -27478,11 +27512,11 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>10.1337</v>
+        <v>10.0352</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27507,7 +27541,7 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>23.3241</v>
+        <v>23.3109</v>
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
@@ -27515,7 +27549,7 @@
         </is>
       </c>
       <c r="G37" s="28" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="H37" s="34" t="inlineStr">
         <is>
@@ -27523,11 +27557,11 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>23.7242</v>
+        <v>23.3215</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27560,7 +27594,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27600,7 +27634,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27640,7 +27674,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27684,7 +27718,7 @@
       </c>
       <c r="H41" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I41" t="n">
@@ -27720,7 +27754,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27760,7 +27794,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27800,7 +27834,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -27840,7 +27874,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27880,7 +27914,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -27961,7 +27995,7 @@
       </c>
       <c r="H48" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -27997,7 +28031,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28037,7 +28071,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28077,7 +28111,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28117,7 +28151,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28157,7 +28191,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28197,7 +28231,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28237,7 +28271,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28277,7 +28311,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28317,7 +28351,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28357,7 +28391,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28397,7 +28431,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28437,7 +28471,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28477,7 +28511,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28517,7 +28551,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28557,7 +28591,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28597,7 +28631,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28605,7 +28639,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>36.02</v>
+        <v>34.639999</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28637,7 +28671,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28677,7 +28711,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28717,7 +28751,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28757,7 +28791,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28797,7 +28831,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28837,7 +28871,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28877,7 +28911,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28917,7 +28951,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28957,7 +28991,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -28997,7 +29031,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29037,7 +29071,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29045,7 +29079,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>119.510002</v>
+        <v>117.18</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29077,7 +29111,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29117,7 +29151,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29157,7 +29191,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29165,7 +29199,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>40.110001</v>
+        <v>38.099998</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29197,7 +29231,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29237,7 +29271,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29277,7 +29311,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29317,7 +29351,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29357,7 +29391,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29389,7 +29423,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>140.41</v>
+        <v>140.46</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29397,7 +29431,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29405,7 +29439,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>129.516159</v>
+        <v>140.315616</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29429,7 +29463,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>763.15</v>
+        <v>762.28</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29437,7 +29471,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29445,7 +29479,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>741.018587</v>
+        <v>762.811197</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29469,7 +29503,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>81291</v>
+        <v>81128</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29477,7 +29511,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29485,7 +29519,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>76527.29248400001</v>
+        <v>81241.614506</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29509,7 +29543,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00788</v>
+        <v>0.007913</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29517,7 +29551,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29525,7 +29559,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007378</v>
+        <v>0.007873</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29549,7 +29583,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.014208</v>
+        <v>0.014194</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29557,7 +29591,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29565,7 +29599,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.013278</v>
+        <v>0.014206</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29589,7 +29623,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>113.43</v>
+        <v>110.34</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29597,7 +29631,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29605,7 +29639,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>101.722237</v>
+        <v>113.338318</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29629,7 +29663,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.06</v>
+        <v>2.1</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29637,7 +29671,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29645,7 +29679,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.981949</v>
+        <v>2.055673</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29677,7 +29711,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29709,7 +29743,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.027246</v>
+        <v>0.028118</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29717,7 +29751,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29725,7 +29759,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.024888</v>
+        <v>0.027247</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29749,7 +29783,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.252093</v>
+        <v>6.823684</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29757,7 +29791,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29765,7 +29799,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.096772</v>
+        <v>7.237303</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29789,7 +29823,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>27.088339</v>
+        <v>28.631664</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29797,7 +29831,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29805,7 +29839,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>25.050637</v>
+        <v>27.08356</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29829,7 +29863,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.143433</v>
+        <v>0.147554</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29837,7 +29871,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29845,7 +29879,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.13423</v>
+        <v>0.143437</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29869,7 +29903,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25405.2635</v>
+        <v>25376.3012</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29877,7 +29911,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29885,7 +29919,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>24668.508761</v>
+        <v>25393.984745</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29909,7 +29943,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2706177.39</v>
+        <v>2700751.12</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29917,7 +29951,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29925,7 +29959,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2547593.566789</v>
+        <v>2704533.346904</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29949,7 +29983,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.923728</v>
+        <v>2.900092</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29957,7 +29991,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29965,7 +29999,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.730043</v>
+        <v>2.917216</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -29989,7 +30023,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>86986.4371</v>
+        <v>87282.3852</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -29997,7 +30031,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30005,7 +30039,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>81528.721494</v>
+        <v>86946.501859</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30029,7 +30063,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.277039</v>
+        <v>20.452344</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30037,7 +30071,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30045,7 +30079,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>19.851612</v>
+        <v>20.279328</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30069,7 +30103,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>81291</v>
+        <v>81128</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30077,7 +30111,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30085,7 +30119,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>76527.29248400001</v>
+        <v>81241.614506</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30109,7 +30143,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>20.94</v>
+        <v>21.48</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30117,7 +30151,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30125,7 +30159,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>19.580795</v>
+        <v>20.929426</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30223,7 +30257,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00788</v>
+        <v>0.007913</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30231,7 +30265,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30239,7 +30273,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007378</v>
+        <v>0.007873</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30263,7 +30297,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>113.43</v>
+        <v>110.34</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30271,7 +30305,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30279,7 +30313,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>101.722237</v>
+        <v>113.338318</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30311,7 +30345,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30343,27 +30377,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.1072</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46281</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.0972</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46280</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.627</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-21
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L116"/>
+  <dimension ref="B2:L117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25341,6 +25341,40 @@
         <v>33.29</v>
       </c>
       <c r="K116" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="72" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C117" t="n">
+        <v>26452147</v>
+      </c>
+      <c r="D117" t="n">
+        <v>22834051</v>
+      </c>
+      <c r="E117" t="n">
+        <v>3618097</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.1585</v>
+      </c>
+      <c r="G117" t="n">
+        <v>18587663</v>
+      </c>
+      <c r="H117" t="n">
+        <v>4919678</v>
+      </c>
+      <c r="I117" t="n">
+        <v>1566982</v>
+      </c>
+      <c r="J117" t="n">
+        <v>33.24</v>
+      </c>
+      <c r="K117" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25918,7 +25952,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25933,11 +25967,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.29</v>
+        <v>33.24</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-20</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -25982,11 +26016,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1044</v>
+        <v>26.0814</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-20</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26281,7 +26315,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.6021</v>
+        <v>9.515700000000001</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26289,7 +26323,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26297,11 +26331,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9.6021</v>
+        <v>9.724600000000001</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -26371,7 +26405,7 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>15.1584</v>
+        <v>14.9009</v>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -26379,7 +26413,7 @@
         </is>
       </c>
       <c r="G11" s="28" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
@@ -26387,11 +26421,11 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>15.104</v>
+        <v>15.0984</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26612,11 +26646,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>81.5758</v>
+        <v>80.6232</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26686,7 +26720,7 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
-        <v>16.519</v>
+        <v>16.5005</v>
       </c>
       <c r="F18" s="34" t="inlineStr">
         <is>
@@ -26694,7 +26728,7 @@
         </is>
       </c>
       <c r="G18" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H18" s="34" t="inlineStr">
         <is>
@@ -26702,11 +26736,11 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>16.5005</v>
+        <v>16.4882</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26956,7 +26990,7 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
-        <v>11.5822</v>
+        <v>11.3892</v>
       </c>
       <c r="F24" s="34" t="inlineStr">
         <is>
@@ -26964,7 +26998,7 @@
         </is>
       </c>
       <c r="G24" s="28" t="n">
-        <v>46282</v>
+        <v>46279</v>
       </c>
       <c r="H24" s="34" t="inlineStr">
         <is>
@@ -26972,11 +27006,11 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>11.5024</v>
+        <v>11.5536</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>
@@ -27046,7 +27080,7 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
-        <v>13.7976</v>
+        <v>13.9987</v>
       </c>
       <c r="F26" s="34" t="inlineStr">
         <is>
@@ -27054,7 +27088,7 @@
         </is>
       </c>
       <c r="G26" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H26" s="34" t="inlineStr">
         <is>
@@ -27062,11 +27096,11 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>13.9987</v>
+        <v>13.8281</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27242,11 +27276,11 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>34.4558</v>
+        <v>33.9117</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27271,7 +27305,7 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
-        <v>13.1495</v>
+        <v>13.144</v>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
@@ -27279,7 +27313,7 @@
         </is>
       </c>
       <c r="G31" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H31" s="34" t="inlineStr">
         <is>
@@ -27287,11 +27321,11 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>13.144</v>
+        <v>12.9644</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27406,7 +27440,7 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
-        <v>16.2386</v>
+        <v>16.2385</v>
       </c>
       <c r="F34" s="34" t="inlineStr">
         <is>
@@ -27414,7 +27448,7 @@
         </is>
       </c>
       <c r="G34" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H34" s="34" t="inlineStr">
         <is>
@@ -27422,11 +27456,11 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>16.2385</v>
+        <v>16.2381</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27467,11 +27501,11 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>28.0542</v>
+        <v>28.2534</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27594,7 +27628,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27634,7 +27668,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27674,7 +27708,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27754,7 +27788,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27794,7 +27828,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27834,7 +27868,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -27874,7 +27908,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27914,7 +27948,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28031,7 +28065,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28071,7 +28105,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28111,7 +28145,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28151,7 +28185,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28191,7 +28225,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28231,7 +28265,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28271,7 +28305,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28311,7 +28345,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28351,7 +28385,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28391,7 +28425,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28431,7 +28465,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28471,7 +28505,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28511,7 +28545,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28551,7 +28585,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28591,7 +28625,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28631,7 +28665,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28671,7 +28705,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28711,7 +28745,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28751,7 +28785,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28791,7 +28825,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28831,7 +28865,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28871,7 +28905,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28911,7 +28945,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28951,7 +28985,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -28991,7 +29025,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29031,7 +29065,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29071,7 +29105,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29111,7 +29145,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29151,7 +29185,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29191,7 +29225,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29231,7 +29265,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29271,7 +29305,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29311,7 +29345,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29351,7 +29385,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29391,7 +29425,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29423,7 +29457,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>140.46</v>
+        <v>138.6</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29431,7 +29465,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29439,7 +29473,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>140.315616</v>
+        <v>140.346497</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29463,7 +29497,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>762.28</v>
+        <v>780.53</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29471,7 +29505,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29479,7 +29513,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>762.811197</v>
+        <v>762.114556</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29503,7 +29537,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>81128</v>
+        <v>81517</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29511,7 +29545,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29519,7 +29553,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>81241.614506</v>
+        <v>81111.927884</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29543,7 +29577,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.007913</v>
+        <v>0.00808</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29551,7 +29585,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29559,7 +29593,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007873</v>
+        <v>0.007905000000000001</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29583,7 +29617,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.014194</v>
+        <v>0.014087</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29591,7 +29625,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29599,7 +29633,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.014206</v>
+        <v>0.014189</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29623,7 +29657,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>110.34</v>
+        <v>112.23</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29631,7 +29665,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29639,7 +29673,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>113.338318</v>
+        <v>110.298575</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29663,7 +29697,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29671,7 +29705,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29679,7 +29713,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.055673</v>
+        <v>2.091417</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29711,7 +29745,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29743,7 +29777,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.028118</v>
+        <v>0.028595</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29751,7 +29785,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29759,7 +29793,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.027247</v>
+        <v>0.028064</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29783,7 +29817,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.823684</v>
+        <v>7.228736</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29791,7 +29825,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29799,7 +29833,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.237303</v>
+        <v>6.82707</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29823,7 +29857,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>28.631664</v>
+        <v>31.20292</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29831,7 +29865,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29839,7 +29873,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>27.08356</v>
+        <v>28.431929</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29863,7 +29897,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.147554</v>
+        <v>0.151467</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29871,7 +29905,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29879,7 +29913,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.143437</v>
+        <v>0.147318</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29903,7 +29937,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25376.3012</v>
+        <v>25944.8172</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29911,7 +29945,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29919,7 +29953,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25393.984745</v>
+        <v>25332.687835</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29943,7 +29977,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2700751.12</v>
+        <v>2709625.08</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29951,7 +29985,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29959,7 +29993,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2704533.346904</v>
+        <v>2696160.48285</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -29983,7 +30017,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.900092</v>
+        <v>2.951612</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -29991,7 +30025,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -29999,7 +30033,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.917216</v>
+        <v>2.89314</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30023,7 +30057,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>87282.3852</v>
+        <v>88911.3492</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30031,7 +30065,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30039,7 +30073,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>86946.501859</v>
+        <v>87128.616431</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30063,7 +30097,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.452344</v>
+        <v>20.17781</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30071,7 +30105,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30079,7 +30113,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.279328</v>
+        <v>20.42025</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30103,7 +30137,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>81128</v>
+        <v>81517</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30111,7 +30145,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30119,7 +30153,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>81241.614506</v>
+        <v>81111.927884</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30143,7 +30177,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>21.48</v>
+        <v>22.1</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30151,7 +30185,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30159,7 +30193,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>20.929426</v>
+        <v>21.449335</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30257,7 +30291,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.007913</v>
+        <v>0.00808</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30265,7 +30299,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30273,7 +30307,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007873</v>
+        <v>0.007905000000000001</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30297,7 +30331,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>110.34</v>
+        <v>112.23</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30305,7 +30339,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30313,7 +30347,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>113.338318</v>
+        <v>110.298575</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30345,7 +30379,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-22
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L117"/>
+  <dimension ref="B2:L118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25375,6 +25375,40 @@
         <v>33.24</v>
       </c>
       <c r="K117" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="72" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C118" t="n">
+        <v>26620576</v>
+      </c>
+      <c r="D118" t="n">
+        <v>22828745</v>
+      </c>
+      <c r="E118" t="n">
+        <v>3791830</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.1661</v>
+      </c>
+      <c r="G118" t="n">
+        <v>18587056</v>
+      </c>
+      <c r="H118" t="n">
+        <v>5029294</v>
+      </c>
+      <c r="I118" t="n">
+        <v>1624411</v>
+      </c>
+      <c r="J118" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="K118" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25952,7 +25986,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -25967,11 +26001,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.24</v>
+        <v>33.2</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-21</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26016,11 +26050,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.0814</v>
+        <v>26.0427</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-21</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26180,7 +26214,7 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>10.7039</v>
+        <v>10.7035</v>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -26188,7 +26222,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -26196,11 +26230,11 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10.7039</v>
+        <v>10.7033</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26270,7 +26304,7 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
-        <v>8.4726</v>
+        <v>8.475</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
@@ -26278,7 +26312,7 @@
         </is>
       </c>
       <c r="G8" s="28" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
@@ -26286,11 +26320,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8.475</v>
+        <v>8.363099999999999</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26315,7 +26349,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.515700000000001</v>
+        <v>9.6021</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26323,7 +26357,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26331,11 +26365,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9.724600000000001</v>
+        <v>9.6021</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26405,7 +26439,7 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>14.9009</v>
+        <v>15.1584</v>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -26413,7 +26447,7 @@
         </is>
       </c>
       <c r="G11" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
@@ -26421,11 +26455,11 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>15.0984</v>
+        <v>15.104</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26450,7 +26484,7 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
-        <v>28.8544</v>
+        <v>28.4866</v>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
@@ -26458,7 +26492,7 @@
         </is>
       </c>
       <c r="G12" s="28" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="H12" s="34" t="inlineStr">
         <is>
@@ -26466,11 +26500,11 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>28.8573</v>
+        <v>28.7218</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26601,11 +26635,11 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>16.1916</v>
+        <v>16.3313</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26630,7 +26664,7 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
-        <v>81.62779999999999</v>
+        <v>81.5758</v>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
@@ -26638,7 +26672,7 @@
         </is>
       </c>
       <c r="G16" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
@@ -26646,11 +26680,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>80.6232</v>
+        <v>81.8845</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -26691,11 +26725,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.5904</v>
+        <v>54.5141</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -26720,27 +26754,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.519</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5005</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4882</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26990,7 +27024,7 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
-        <v>11.3892</v>
+        <v>11.5822</v>
       </c>
       <c r="F24" s="34" t="inlineStr">
         <is>
@@ -26998,7 +27032,7 @@
         </is>
       </c>
       <c r="G24" s="28" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
       <c r="H24" s="34" t="inlineStr">
         <is>
@@ -27006,11 +27040,11 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>11.5536</v>
+        <v>11.5024</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27035,7 +27069,7 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
-        <v>9.8436</v>
+        <v>9.8544</v>
       </c>
       <c r="F25" s="34" t="inlineStr">
         <is>
@@ -27043,7 +27077,7 @@
         </is>
       </c>
       <c r="G25" s="28" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="H25" s="34" t="inlineStr">
         <is>
@@ -27051,11 +27085,11 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>9.9785</v>
+        <v>9.858700000000001</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27080,27 +27114,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7976</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.9987</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.8281</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27260,7 +27294,7 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
-        <v>35.1929</v>
+        <v>34.4558</v>
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
@@ -27268,7 +27302,7 @@
         </is>
       </c>
       <c r="G30" s="28" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="H30" s="34" t="inlineStr">
         <is>
@@ -27276,11 +27310,11 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>33.9117</v>
+        <v>35.424</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>
@@ -27305,27 +27339,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.1495</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.144</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.9644</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27395,7 +27429,7 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>12.9572</v>
+        <v>12.7759</v>
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
@@ -27403,7 +27437,7 @@
         </is>
       </c>
       <c r="G33" s="28" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="H33" s="34" t="inlineStr">
         <is>
@@ -27411,11 +27445,11 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>12.9269</v>
+        <v>12.924</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
@@ -27440,7 +27474,7 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
-        <v>16.2385</v>
+        <v>16.2386</v>
       </c>
       <c r="F34" s="34" t="inlineStr">
         <is>
@@ -27448,7 +27482,7 @@
         </is>
       </c>
       <c r="G34" s="28" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="H34" s="34" t="inlineStr">
         <is>
@@ -27485,7 +27519,7 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>28.597</v>
+        <v>28.0542</v>
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
@@ -27493,7 +27527,7 @@
         </is>
       </c>
       <c r="G35" s="28" t="n">
-        <v>46282</v>
+        <v>46281</v>
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
@@ -27501,11 +27535,11 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>28.2534</v>
+        <v>28.1131</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -27575,7 +27609,7 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>23.3109</v>
+        <v>23.3215</v>
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
@@ -27583,7 +27617,7 @@
         </is>
       </c>
       <c r="G37" s="28" t="n">
-        <v>46283</v>
+        <v>46282</v>
       </c>
       <c r="H37" s="34" t="inlineStr">
         <is>
@@ -27591,11 +27625,11 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>23.3215</v>
+        <v>23.0448</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -27628,7 +27662,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27660,7 +27694,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.059</v>
+        <v>1.075</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27668,7 +27702,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27676,7 +27710,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.069</v>
+        <v>1.075</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27708,7 +27742,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27788,7 +27822,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27828,7 +27862,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27860,23 +27894,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>195.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>193.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>193</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27900,7 +27934,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -27908,7 +27942,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27916,7 +27950,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -27948,7 +27982,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28057,23 +28091,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>62.25</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>61.25</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>61</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28097,7 +28131,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28105,7 +28139,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28113,7 +28147,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28145,7 +28179,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28177,7 +28211,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28185,7 +28219,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28193,7 +28227,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28217,7 +28251,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.75</v>
+        <v>5.65</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28225,7 +28259,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28233,7 +28267,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.6</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28257,7 +28291,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.7</v>
+        <v>22.9</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28265,7 +28299,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28273,7 +28307,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.700001</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28305,7 +28339,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28337,7 +28371,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.46</v>
+        <v>4.54</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28345,7 +28379,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28353,7 +28387,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.46</v>
+        <v>4.54</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28377,7 +28411,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.28</v>
+        <v>3.34</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28385,7 +28419,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28393,7 +28427,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.28</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28417,7 +28451,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28425,7 +28459,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28433,7 +28467,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28457,7 +28491,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28465,7 +28499,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28473,7 +28507,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.799999</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28497,7 +28531,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>109.32</v>
+        <v>113.15</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28505,7 +28539,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28537,7 +28571,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>248.92</v>
+        <v>249.52</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28545,7 +28579,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28577,7 +28611,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>444.57</v>
+        <v>464.24</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28585,7 +28619,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28617,7 +28651,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>118.82</v>
+        <v>119.98</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28625,7 +28659,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28657,7 +28691,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>34.64</v>
+        <v>34.76</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28665,7 +28699,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28697,7 +28731,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>181.31</v>
+        <v>189.16</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28705,7 +28739,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28737,7 +28771,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>169.84</v>
+        <v>175.23</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28745,7 +28779,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28777,7 +28811,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>185.78</v>
+        <v>183.32</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28785,7 +28819,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28817,7 +28851,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>176.99</v>
+        <v>183.97</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28825,7 +28859,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28857,7 +28891,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1152.93</v>
+        <v>1164.89</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28865,7 +28899,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28897,7 +28931,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>73.27</v>
+        <v>74.78</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28905,7 +28939,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28937,7 +28971,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1217.8</v>
+        <v>1277.68</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28945,7 +28979,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28977,7 +29011,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>154.91</v>
+        <v>156.7</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -28985,7 +29019,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29017,7 +29051,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>222.27</v>
+        <v>227.38</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29025,7 +29059,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29057,7 +29091,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>78.3</v>
+        <v>77.98</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29065,7 +29099,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29097,7 +29131,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>117.18</v>
+        <v>117.21</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29105,7 +29139,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29137,7 +29171,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>371.47</v>
+        <v>381.54</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29145,7 +29179,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29177,7 +29211,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>364.27</v>
+        <v>375.3</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29185,7 +29219,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29217,7 +29251,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>38.1</v>
+        <v>39.26</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29225,7 +29259,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29257,7 +29291,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>69.06</v>
+        <v>70.27</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29265,7 +29299,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29297,7 +29331,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>336.13</v>
+        <v>338.98</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29305,7 +29339,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29337,23 +29371,23 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
+        <v>201.05</v>
+      </c>
+      <c r="F81" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G81" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H81" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
         <v>194.25</v>
-      </c>
-      <c r="F81" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G81" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H81" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I81" t="n">
-        <v>173.970001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29377,23 +29411,23 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
+        <v>741.245</v>
+      </c>
+      <c r="F82" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G82" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
         <v>665.75</v>
-      </c>
-      <c r="F82" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G82" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H82" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I82" t="n">
-        <v>682.309998</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29417,7 +29451,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>31.41</v>
+        <v>30.79</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29425,7 +29459,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29433,7 +29467,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>31.41</v>
+        <v>30.790001</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29457,7 +29491,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>138.6</v>
+        <v>144.2</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29465,7 +29499,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29473,7 +29507,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>140.346497</v>
+        <v>138.797659</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29497,7 +29531,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>780.53</v>
+        <v>793.52</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29505,7 +29539,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29513,7 +29547,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>762.114556</v>
+        <v>781.001818</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29537,7 +29571,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>81517</v>
+        <v>85653</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29545,7 +29579,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29553,7 +29587,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>81111.927884</v>
+        <v>81553.90983800001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29577,7 +29611,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00808</v>
+        <v>0.008802000000000001</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29585,7 +29619,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29593,7 +29627,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.007905000000000001</v>
+        <v>0.008097999999999999</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29617,7 +29651,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.014087</v>
+        <v>0.014901</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29625,7 +29659,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29633,7 +29667,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.014189</v>
+        <v>0.014116</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29657,7 +29691,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>112.23</v>
+        <v>117.73</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29665,7 +29699,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29673,7 +29707,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>110.298575</v>
+        <v>112.348521</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29697,7 +29731,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.09</v>
+        <v>2.2</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29705,7 +29739,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29713,7 +29747,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.091417</v>
+        <v>2.096383</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29745,7 +29779,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29777,7 +29811,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.028595</v>
+        <v>0.029807</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29785,7 +29819,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29793,7 +29827,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.028064</v>
+        <v>0.028609</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29817,7 +29851,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.228736</v>
+        <v>7.346762</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29825,7 +29859,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29833,7 +29867,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.82707</v>
+        <v>7.236874</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29857,7 +29891,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>31.20292</v>
+        <v>34.3288</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29865,7 +29899,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29873,7 +29907,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>28.431929</v>
+        <v>31.242764</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29897,7 +29931,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.151467</v>
+        <v>0.164706</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29905,7 +29939,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29913,7 +29947,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.147318</v>
+        <v>0.151115</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29937,7 +29971,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25944.8172</v>
+        <v>26344.864</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29945,7 +29979,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29953,7 +29987,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25332.687835</v>
+        <v>25929.260366</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -29977,7 +30011,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2709625.08</v>
+        <v>2843679.6</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -29985,7 +30019,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -29993,7 +30027,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2696160.48285</v>
+        <v>2707589.806613</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30017,7 +30051,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>2.951612</v>
+        <v>3.287265</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30025,7 +30059,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30033,7 +30067,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.89314</v>
+        <v>2.953902</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30057,7 +30091,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>88911.3492</v>
+        <v>91244.88800000001</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30065,7 +30099,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30073,7 +30107,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>87128.616431</v>
+        <v>88870.275496</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30097,7 +30131,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.17781</v>
+        <v>20.966829</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30105,7 +30139,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30113,7 +30147,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.42025</v>
+        <v>20.15354</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30137,7 +30171,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>81517</v>
+        <v>85653</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30145,7 +30179,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30153,7 +30187,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>81111.927884</v>
+        <v>81553.90983800001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30177,7 +30211,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>22.1</v>
+        <v>22.75</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30185,7 +30219,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30193,7 +30227,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>21.449335</v>
+        <v>22.14651</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30291,7 +30325,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00808</v>
+        <v>0.008802000000000001</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30299,7 +30333,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30307,7 +30341,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.007905000000000001</v>
+        <v>0.008097999999999999</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30331,7 +30365,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>112.23</v>
+        <v>117.73</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30339,7 +30373,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30347,7 +30381,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>110.298575</v>
+        <v>112.348521</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30379,7 +30413,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-23
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L118"/>
+  <dimension ref="B2:L119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25409,6 +25409,40 @@
         <v>33.2</v>
       </c>
       <c r="K118" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="72" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C119" t="n">
+        <v>26702845</v>
+      </c>
+      <c r="D119" t="n">
+        <v>22819548</v>
+      </c>
+      <c r="E119" t="n">
+        <v>3883298</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.1702</v>
+      </c>
+      <c r="G119" t="n">
+        <v>18630978</v>
+      </c>
+      <c r="H119" t="n">
+        <v>5044021</v>
+      </c>
+      <c r="I119" t="n">
+        <v>1637201</v>
+      </c>
+      <c r="J119" t="n">
+        <v>33.13</v>
+      </c>
+      <c r="K119" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -25986,7 +26020,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26001,11 +26035,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.2</v>
+        <v>33.13</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-22</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26050,11 +26084,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.0427</v>
+        <v>25.9776</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-22</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26169,27 +26203,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>20.3767</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>19.7228</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>19.2267</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26214,7 +26248,7 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>10.7035</v>
+        <v>10.7045</v>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -26222,7 +26256,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -26230,11 +26264,11 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10.7033</v>
+        <v>10.7039</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26259,27 +26293,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3806</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.4649</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.4342</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26304,7 +26338,7 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
-        <v>8.475</v>
+        <v>8.615600000000001</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
@@ -26312,7 +26346,7 @@
         </is>
       </c>
       <c r="G8" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
@@ -26320,11 +26354,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8.363099999999999</v>
+        <v>8.4726</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26349,7 +26383,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.6021</v>
+        <v>9.633599999999999</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26357,7 +26391,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26369,7 +26403,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26394,27 +26428,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2265</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.1751</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.0852</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26439,27 +26473,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.3714</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.1584</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.104</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26484,7 +26518,7 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
-        <v>28.4866</v>
+        <v>29.5012</v>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
@@ -26492,7 +26526,7 @@
         </is>
       </c>
       <c r="G12" s="28" t="n">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="H12" s="34" t="inlineStr">
         <is>
@@ -26500,11 +26534,11 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>28.7218</v>
+        <v>28.8544</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26529,27 +26563,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.6096</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.2634</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.2622</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26574,27 +26608,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.3372</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.1664</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.1666</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26619,27 +26653,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.3596</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.1811</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.3313</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
@@ -26664,7 +26698,7 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
-        <v>81.5758</v>
+        <v>82.3896</v>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
@@ -26672,7 +26706,7 @@
         </is>
       </c>
       <c r="G16" s="28" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
@@ -26680,11 +26714,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>81.8845</v>
+        <v>81.62779999999999</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26709,27 +26743,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.9312</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.6003</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.5141</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26754,27 +26788,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5212</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.519</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5005</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26799,27 +26833,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4487</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4473</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4472</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26844,27 +26878,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.6235</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.5907</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.1276</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26889,27 +26923,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.6842</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.5598</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.4633</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26934,27 +26968,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9938</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0819</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0081</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26979,27 +27013,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.286</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.1818</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.1766</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27024,27 +27058,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.6363</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.5822</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.5024</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27069,7 +27103,7 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
-        <v>9.8544</v>
+        <v>9.817</v>
       </c>
       <c r="F25" s="34" t="inlineStr">
         <is>
@@ -27077,7 +27111,7 @@
         </is>
       </c>
       <c r="G25" s="28" t="n">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="H25" s="34" t="inlineStr">
         <is>
@@ -27085,11 +27119,11 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>9.858700000000001</v>
+        <v>9.8436</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27114,27 +27148,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7673</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7976</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.9987</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27159,27 +27193,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.4394</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.357</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.2902</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27204,27 +27238,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>19.1215</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.3116</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.9562</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27249,27 +27283,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.3687</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.5262</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>23.5912</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27339,27 +27373,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.262</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.1495</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.144</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27384,7 +27418,7 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
-        <v>21.7215</v>
+        <v>21.722</v>
       </c>
       <c r="F32" s="34" t="inlineStr">
         <is>
@@ -27392,7 +27426,7 @@
         </is>
       </c>
       <c r="G32" s="28" t="n">
-        <v>46283</v>
+        <v>46286</v>
       </c>
       <c r="H32" s="34" t="inlineStr">
         <is>
@@ -27404,7 +27438,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27429,7 +27463,7 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
-        <v>12.7759</v>
+        <v>13.0817</v>
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
@@ -27437,7 +27471,7 @@
         </is>
       </c>
       <c r="G33" s="28" t="n">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="H33" s="34" t="inlineStr">
         <is>
@@ -27445,11 +27479,11 @@
         </is>
       </c>
       <c r="I33" t="n">
-        <v>12.924</v>
+        <v>12.9572</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27474,27 +27508,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2397</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2386</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2381</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27519,7 +27553,7 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
-        <v>28.0542</v>
+        <v>28.7425</v>
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
@@ -27527,7 +27561,7 @@
         </is>
       </c>
       <c r="G35" s="28" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="H35" s="34" t="inlineStr">
         <is>
@@ -27535,11 +27569,11 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>28.1131</v>
+        <v>28.597</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -27564,27 +27598,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1201</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0938</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0352</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27609,7 +27643,7 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
-        <v>23.3215</v>
+        <v>23.5324</v>
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
@@ -27617,7 +27651,7 @@
         </is>
       </c>
       <c r="G37" s="28" t="n">
-        <v>46282</v>
+        <v>46286</v>
       </c>
       <c r="H37" s="34" t="inlineStr">
         <is>
@@ -27625,11 +27659,11 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>23.0448</v>
+        <v>23.3109</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27654,7 +27688,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.23</v>
+        <v>22.17</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27662,7 +27696,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27670,7 +27704,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.08</v>
+        <v>22.190001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27702,7 +27736,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27734,7 +27768,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>751.16</v>
+        <v>769.21</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27742,7 +27776,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27750,7 +27784,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>754.940002</v>
+        <v>781.869995</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27814,7 +27848,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>205.81</v>
+        <v>209.85</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27822,7 +27856,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27830,7 +27864,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>207.360001</v>
+        <v>211.770004</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27854,7 +27888,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -27862,7 +27896,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -27894,23 +27928,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>197.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>195.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>193.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27934,7 +27968,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -27942,7 +27976,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -27950,7 +27984,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -27982,7 +28016,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28099,7 +28133,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28139,7 +28173,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28179,7 +28213,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28219,7 +28253,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28251,7 +28285,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28259,7 +28293,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28267,7 +28301,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28291,7 +28325,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.9</v>
+        <v>22.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28299,7 +28333,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28307,7 +28341,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.9</v>
+        <v>22.799999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28339,7 +28373,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28371,7 +28405,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.54</v>
+        <v>4.46</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28379,7 +28413,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28387,7 +28421,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.54</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28411,7 +28445,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.34</v>
+        <v>3.3</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28419,7 +28453,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28427,7 +28461,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.34</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28451,7 +28485,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28459,7 +28493,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28499,7 +28533,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28531,7 +28565,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>113.15</v>
+        <v>115.74</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28539,7 +28573,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28547,7 +28581,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>109.32</v>
+        <v>113.150002</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28571,7 +28605,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>249.52</v>
+        <v>238.25</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28579,7 +28613,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28587,7 +28621,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>248.919998</v>
+        <v>249.520004</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28611,7 +28645,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>464.24</v>
+        <v>472.46</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28619,7 +28653,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28627,7 +28661,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>444.570007</v>
+        <v>464.23999</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28651,7 +28685,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>119.98</v>
+        <v>120.38</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28659,7 +28693,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28667,7 +28701,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>118.82</v>
+        <v>119.980003</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28691,7 +28725,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>34.76</v>
+        <v>34.42</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28699,7 +28733,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28707,7 +28741,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>34.639999</v>
+        <v>34.759998</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28731,7 +28765,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>189.16</v>
+        <v>192.62</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28739,7 +28773,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28747,7 +28781,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>181.309998</v>
+        <v>189.160004</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28771,7 +28805,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>175.23</v>
+        <v>174.26</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28779,7 +28813,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28787,7 +28821,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>169.839996</v>
+        <v>175.229996</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28811,7 +28845,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>183.32</v>
+        <v>178.75</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28819,7 +28853,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28827,7 +28861,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>185.779999</v>
+        <v>183.320007</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28851,7 +28885,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>183.97</v>
+        <v>188.32</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28859,7 +28893,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28867,7 +28901,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>176.990005</v>
+        <v>183.970001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28891,7 +28925,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1164.89</v>
+        <v>1170.14</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28899,7 +28933,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28907,7 +28941,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1152.930054</v>
+        <v>1164.890015</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28931,7 +28965,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>74.78</v>
+        <v>75.81999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28939,7 +28973,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28947,7 +28981,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>73.269997</v>
+        <v>74.779999</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -28971,7 +29005,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1277.68</v>
+        <v>1380.62</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -28979,7 +29013,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -28987,7 +29021,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1217.800049</v>
+        <v>1277.680054</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29011,7 +29045,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>156.7</v>
+        <v>156.25</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29019,7 +29053,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29027,7 +29061,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>154.910004</v>
+        <v>156.699997</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29051,7 +29085,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>227.38</v>
+        <v>228.87</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29059,7 +29093,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29067,7 +29101,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>222.270004</v>
+        <v>227.380005</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29091,7 +29125,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.98</v>
+        <v>78.12</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29099,7 +29133,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29107,7 +29141,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>78.300003</v>
+        <v>77.980003</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29131,7 +29165,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>117.21</v>
+        <v>118.44</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29139,7 +29173,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29147,7 +29181,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>117.18</v>
+        <v>117.209999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29171,7 +29205,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>381.54</v>
+        <v>398.69</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29179,7 +29213,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29187,7 +29221,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>371.470001</v>
+        <v>381.540009</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29211,7 +29245,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>375.3</v>
+        <v>378.9</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29219,7 +29253,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29227,7 +29261,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>364.269989</v>
+        <v>375.299988</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29251,7 +29285,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>39.26</v>
+        <v>39.03</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29259,7 +29293,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29267,7 +29301,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>38.099998</v>
+        <v>39.259998</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29291,7 +29325,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>70.27</v>
+        <v>70.97</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29299,7 +29333,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29307,7 +29341,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>69.05999799999999</v>
+        <v>70.269997</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29331,7 +29365,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>338.98</v>
+        <v>339.75</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29339,7 +29373,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29347,7 +29381,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>336.130005</v>
+        <v>338.980011</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29371,7 +29405,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>201.05</v>
+        <v>201.07</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29379,7 +29413,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29387,7 +29421,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>194.25</v>
+        <v>201.050003</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29411,7 +29445,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>741.245</v>
+        <v>736.595</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29419,7 +29453,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29427,7 +29461,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>665.75</v>
+        <v>741.25</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29451,7 +29485,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.79</v>
+        <v>30.83</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29459,7 +29493,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29467,7 +29501,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.790001</v>
+        <v>30.83</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29491,7 +29525,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>144.2</v>
+        <v>148.54</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29499,7 +29533,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29507,7 +29541,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>138.797659</v>
+        <v>144.706142</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29531,7 +29565,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>793.52</v>
+        <v>791</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29539,7 +29573,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29547,7 +29581,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>781.001818</v>
+        <v>795.2331370000001</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29571,7 +29605,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>85653</v>
+        <v>86585</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29579,7 +29613,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29587,7 +29621,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>81553.90983800001</v>
+        <v>85794.57352000001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29611,7 +29645,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.008802000000000001</v>
+        <v>0.010081</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29619,7 +29653,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29627,7 +29661,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.008097999999999999</v>
+        <v>0.00882</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29651,7 +29685,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.014901</v>
+        <v>0.016661</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29659,7 +29693,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29667,7 +29701,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.014116</v>
+        <v>0.014934</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29691,7 +29725,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>117.73</v>
+        <v>118.75</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29699,7 +29733,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29707,7 +29741,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>112.348521</v>
+        <v>118.042831</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29731,7 +29765,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.2</v>
+        <v>2.23</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29739,7 +29773,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29747,7 +29781,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.096383</v>
+        <v>2.203466</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29779,7 +29813,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29811,7 +29845,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.029807</v>
+        <v>0.029775</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29819,7 +29853,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29827,7 +29861,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.028609</v>
+        <v>0.029851</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29851,7 +29885,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.346762</v>
+        <v>8.02074</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29859,7 +29893,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29867,7 +29901,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.236874</v>
+        <v>7.353372</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29891,7 +29925,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>34.3288</v>
+        <v>33.95825</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29899,7 +29933,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29907,7 +29941,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>31.242764</v>
+        <v>34.390364</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29931,7 +29965,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.164706</v>
+        <v>0.158902</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29939,7 +29973,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29947,7 +29981,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.151115</v>
+        <v>0.165386</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -29971,7 +30005,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>26344.864</v>
+        <v>26205.83</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -29979,7 +30013,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -29987,7 +30021,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25929.260366</v>
+        <v>26346.073821</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30011,7 +30045,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2843679.6</v>
+        <v>2868561.05</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30019,7 +30053,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30027,7 +30061,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2707589.806613</v>
+        <v>2842374.220732</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30051,7 +30085,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.287265</v>
+        <v>3.375417</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30059,7 +30093,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30067,7 +30101,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>2.953902</v>
+        <v>3.303722</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30091,7 +30125,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>91244.88800000001</v>
+        <v>91591.8606</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30099,7 +30133,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30107,7 +30141,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>88870.275496</v>
+        <v>91195.750481</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30131,7 +30165,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.966829</v>
+        <v>20.98494</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30139,7 +30173,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30147,7 +30181,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.15354</v>
+        <v>20.932618</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30171,7 +30205,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>85653</v>
+        <v>86585</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30179,7 +30213,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30187,7 +30221,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>81553.90983800001</v>
+        <v>85794.57352000001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30211,7 +30245,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>22.75</v>
+        <v>23.16</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30219,7 +30253,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30227,7 +30261,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>22.14651</v>
+        <v>22.814858</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30325,7 +30359,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.008802000000000001</v>
+        <v>0.010081</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30333,7 +30367,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30341,7 +30375,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.008097999999999999</v>
+        <v>0.00882</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30365,7 +30399,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>117.73</v>
+        <v>118.75</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30373,7 +30407,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30381,7 +30415,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>112.348521</v>
+        <v>118.042831</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30413,7 +30447,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30445,27 +30479,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.463</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.1072</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46281</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.0972</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-24
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L119"/>
+  <dimension ref="B2:L120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25443,6 +25443,40 @@
         <v>33.13</v>
       </c>
       <c r="K119" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="72" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C120" t="n">
+        <v>26961371</v>
+      </c>
+      <c r="D120" t="n">
+        <v>22854370</v>
+      </c>
+      <c r="E120" t="n">
+        <v>4107000</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.1797</v>
+      </c>
+      <c r="G120" t="n">
+        <v>18920098</v>
+      </c>
+      <c r="H120" t="n">
+        <v>5035033</v>
+      </c>
+      <c r="I120" t="n">
+        <v>1602527</v>
+      </c>
+      <c r="J120" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="K120" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26020,7 +26054,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26035,11 +26069,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.13</v>
+        <v>33.43</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-23</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26084,11 +26118,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>25.9776</v>
+        <v>26.1178</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-23</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26203,27 +26237,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.1786</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>20.3767</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>19.7228</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26248,27 +26282,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7047</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7045</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7039</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26293,27 +26327,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.4326</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3806</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.4649</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26338,27 +26372,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.702999999999999</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.615600000000001</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.4726</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26383,27 +26417,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.665800000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.633599999999999</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.6021</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26428,27 +26462,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2155</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2265</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.1751</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26473,27 +26507,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.3488</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.3714</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.1584</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26518,27 +26552,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.6651</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.5012</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>28.8544</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26563,27 +26597,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.7813</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.6096</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.2634</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26608,27 +26642,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.4161</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.3372</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.1664</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26653,27 +26687,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.2475</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.3596</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.1811</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -26698,27 +26732,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.7585</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.3896</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>81.62779999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26743,27 +26777,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>55.113</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.9312</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.6003</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26788,27 +26822,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5269</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5212</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.519</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26833,27 +26867,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4492</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4487</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4473</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26878,27 +26912,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>42.2358</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.6235</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.5907</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26923,27 +26957,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.7198</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.6842</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.5598</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26968,27 +27002,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0611</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9938</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0819</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27013,27 +27047,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.324</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.286</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.1818</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27058,27 +27092,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.8265</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.6363</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.5822</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27103,27 +27137,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.836399999999999</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.817</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8436</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27148,27 +27182,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.793</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7673</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7976</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27193,27 +27227,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.4554</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.4394</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.357</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27238,27 +27272,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.9739</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>19.1215</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.3116</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27283,27 +27317,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.4122</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.3687</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.5262</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27328,7 +27362,7 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
-        <v>34.4558</v>
+        <v>37.2415</v>
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
@@ -27336,7 +27370,7 @@
         </is>
       </c>
       <c r="G30" s="28" t="n">
-        <v>46281</v>
+        <v>46286</v>
       </c>
       <c r="H30" s="34" t="inlineStr">
         <is>
@@ -27344,11 +27378,11 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>35.424</v>
+        <v>35.56</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27373,27 +27407,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.3158</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.262</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.1495</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27418,27 +27452,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7222</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.722</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7215</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27463,27 +27497,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.1377</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.0817</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>12.9572</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27508,27 +27542,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2401</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2397</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2386</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27553,27 +27587,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.5186</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.7425</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.597</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -27598,27 +27632,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1331</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.1201</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0938</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27643,27 +27677,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.6115</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.5324</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.3109</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27688,7 +27722,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.17</v>
+        <v>22.19</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27696,7 +27730,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27728,7 +27762,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.075</v>
+        <v>1.056</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27736,7 +27770,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27744,7 +27778,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.075</v>
+        <v>1.056</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27768,7 +27802,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>769.21</v>
+        <v>781.87</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27776,7 +27810,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27848,7 +27882,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>209.85</v>
+        <v>211.77</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27856,7 +27890,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27888,23 +27922,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.7</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.8</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27928,23 +27962,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>195</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>197.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>195.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -27976,7 +28010,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28008,7 +28042,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28016,7 +28050,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28024,7 +28058,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -28133,7 +28167,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28165,7 +28199,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28173,7 +28207,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28181,7 +28215,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.8</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28205,7 +28239,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28213,7 +28247,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28221,7 +28255,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28245,7 +28279,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.1</v>
+        <v>15.2</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28253,7 +28287,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28261,7 +28295,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.1</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28285,7 +28319,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.6</v>
+        <v>5.65</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28293,7 +28327,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28301,7 +28335,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.6</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28333,7 +28367,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28373,7 +28407,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28413,7 +28447,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28453,7 +28487,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28485,7 +28519,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28493,7 +28527,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28501,7 +28535,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28525,7 +28559,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.9</v>
+        <v>17.7</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28533,7 +28567,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28541,7 +28575,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.9</v>
+        <v>17.700001</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28565,7 +28599,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>115.74</v>
+        <v>118.43</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28573,7 +28607,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28581,7 +28615,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>113.150002</v>
+        <v>118.43</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28605,7 +28639,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>238.25</v>
+        <v>240.69</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28613,7 +28647,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28621,7 +28655,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>249.520004</v>
+        <v>240.690002</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28645,7 +28679,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>472.46</v>
+        <v>474.38</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28653,7 +28687,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28661,7 +28695,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>464.23999</v>
+        <v>474.380005</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28685,7 +28719,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>120.38</v>
+        <v>120.45</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28693,7 +28727,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28701,7 +28735,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>119.980003</v>
+        <v>120.449997</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28725,7 +28759,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>34.42</v>
+        <v>33.07</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28733,7 +28767,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28741,7 +28775,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>34.759998</v>
+        <v>33.07</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28765,7 +28799,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>192.62</v>
+        <v>185.65</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28773,7 +28807,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28781,7 +28815,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>189.160004</v>
+        <v>185.649994</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28805,7 +28839,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>174.26</v>
+        <v>178.74</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28813,7 +28847,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28821,7 +28855,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>175.229996</v>
+        <v>178.740005</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28845,7 +28879,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>178.75</v>
+        <v>178.52</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28853,7 +28887,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28861,7 +28895,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>183.320007</v>
+        <v>178.520004</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28885,7 +28919,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>188.32</v>
+        <v>187.86</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28893,7 +28927,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28901,7 +28935,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>183.970001</v>
+        <v>187.860001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28925,7 +28959,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1170.14</v>
+        <v>1150.99</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28933,7 +28967,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28941,7 +28975,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1164.890015</v>
+        <v>1150.98999</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28965,7 +28999,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>75.81999999999999</v>
+        <v>75.53</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -28973,7 +29007,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -28981,7 +29015,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>74.779999</v>
+        <v>75.529999</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29005,7 +29039,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1380.62</v>
+        <v>1355.47</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29013,7 +29047,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29021,7 +29055,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1277.680054</v>
+        <v>1355.469971</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29045,7 +29079,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>156.25</v>
+        <v>158.25</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29053,7 +29087,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29085,7 +29119,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>228.87</v>
+        <v>225.51</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29093,7 +29127,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29101,7 +29135,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>227.380005</v>
+        <v>225.509995</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29125,7 +29159,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>78.12</v>
+        <v>76.70999999999999</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29133,7 +29167,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29141,7 +29175,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>77.980003</v>
+        <v>76.709999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29165,7 +29199,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>118.44</v>
+        <v>119.59</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29173,7 +29207,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29181,7 +29215,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>117.209999</v>
+        <v>119.589996</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29205,7 +29239,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>398.69</v>
+        <v>389.14</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29213,7 +29247,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29221,7 +29255,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>381.540009</v>
+        <v>389.140015</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29245,7 +29279,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>378.9</v>
+        <v>380.12</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29253,7 +29287,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29261,7 +29295,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>375.299988</v>
+        <v>380.119995</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29285,7 +29319,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>39.03</v>
+        <v>38.9</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29293,7 +29327,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29301,7 +29335,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>39.259998</v>
+        <v>38.900002</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29325,7 +29359,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>70.97</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29333,7 +29367,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29341,7 +29375,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>70.269997</v>
+        <v>68.760002</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29365,7 +29399,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>339.75</v>
+        <v>337.02</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29373,7 +29407,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29381,7 +29415,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>338.980011</v>
+        <v>337.019989</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29405,7 +29439,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>201.07</v>
+        <v>198.13</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29413,7 +29447,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29421,7 +29455,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>201.050003</v>
+        <v>198.130005</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29457,7 +29491,7 @@
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I82" t="n">
@@ -29485,7 +29519,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.83</v>
+        <v>30.6</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29493,7 +29527,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29501,7 +29535,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.83</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29525,7 +29559,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>148.54</v>
+        <v>138.3</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29533,7 +29567,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29541,7 +29575,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>144.706142</v>
+        <v>147.950557</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29565,7 +29599,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>791</v>
+        <v>767.25</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29573,7 +29607,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29581,7 +29615,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>795.2331370000001</v>
+        <v>790.153836</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29605,7 +29639,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>86585</v>
+        <v>84374</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29613,7 +29647,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29621,7 +29655,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>85794.57352000001</v>
+        <v>86478.783706</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29645,7 +29679,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010081</v>
+        <v>0.009690000000000001</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29653,7 +29687,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29661,7 +29695,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.00882</v>
+        <v>0.010121</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29685,7 +29719,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.016661</v>
+        <v>0.015685</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29693,7 +29727,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29701,7 +29735,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.014934</v>
+        <v>0.016517</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29725,7 +29759,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>118.75</v>
+        <v>115.32</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29733,7 +29767,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29741,7 +29775,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>118.042831</v>
+        <v>118.584192</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29765,7 +29799,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.23</v>
+        <v>1.96</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29773,7 +29807,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29781,7 +29815,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.203466</v>
+        <v>2.223066</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29813,7 +29847,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29845,7 +29879,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.029775</v>
+        <v>0.028767</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29853,7 +29887,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29861,7 +29895,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.029851</v>
+        <v>0.02976</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29885,7 +29919,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>8.02074</v>
+        <v>7.316022</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29893,7 +29927,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29901,7 +29935,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.353372</v>
+        <v>8.101755000000001</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29925,7 +29959,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>33.95825</v>
+        <v>32.152071</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29933,7 +29967,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29941,7 +29975,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>34.390364</v>
+        <v>34.233119</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29965,7 +29999,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.158902</v>
+        <v>0.149721</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -29973,7 +30007,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -29981,7 +30015,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.165386</v>
+        <v>0.160425</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30005,7 +30039,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>26205.83</v>
+        <v>25649.1675</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30013,7 +30047,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30021,7 +30055,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>26346.073821</v>
+        <v>26414.842739</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30045,7 +30079,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2868561.05</v>
+        <v>2820622.82</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30053,7 +30087,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30061,7 +30095,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2842374.220732</v>
+        <v>2890985.739277</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30085,7 +30119,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.375417</v>
+        <v>3.117314</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30093,7 +30127,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30101,7 +30135,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.303722</v>
+        <v>3.403605</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30125,7 +30159,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>91591.8606</v>
+        <v>89883.24099999999</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30133,7 +30167,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30141,7 +30175,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>91195.750481</v>
+        <v>92240.74178700001</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30165,7 +30199,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.98494</v>
+        <v>20.59649</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30173,7 +30207,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30181,7 +30215,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.932618</v>
+        <v>21.181361</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30205,7 +30239,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>86585</v>
+        <v>84374</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30213,7 +30247,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30221,7 +30255,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>85794.57352000001</v>
+        <v>86478.783706</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30245,7 +30279,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.16</v>
+        <v>22.42</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30253,7 +30287,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30261,7 +30295,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>22.814858</v>
+        <v>23.129539</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30359,7 +30393,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010081</v>
+        <v>0.009690000000000001</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30367,7 +30401,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30375,7 +30409,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.00882</v>
+        <v>0.010121</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30399,7 +30433,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>118.75</v>
+        <v>115.32</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30407,7 +30441,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30415,7 +30449,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>118.042831</v>
+        <v>118.584192</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30447,7 +30481,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30479,27 +30513,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.4705</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.463</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46282</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.1072</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-25
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L120"/>
+  <dimension ref="B2:L121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25477,6 +25477,40 @@
         <v>33.43</v>
       </c>
       <c r="K120" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="72" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C121" t="n">
+        <v>27047415</v>
+      </c>
+      <c r="D121" t="n">
+        <v>22853983</v>
+      </c>
+      <c r="E121" t="n">
+        <v>4193432</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.1835</v>
+      </c>
+      <c r="G121" t="n">
+        <v>19026619</v>
+      </c>
+      <c r="H121" t="n">
+        <v>5004335</v>
+      </c>
+      <c r="I121" t="n">
+        <v>1609465</v>
+      </c>
+      <c r="J121" t="n">
+        <v>33.42</v>
+      </c>
+      <c r="K121" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26054,7 +26088,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26069,11 +26103,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.43</v>
+        <v>33.42</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-24</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26118,11 +26152,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1178</v>
+        <v>26.1365</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-24</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26237,27 +26271,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.4002</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.1786</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>20.3767</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26282,27 +26316,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7048</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7047</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7045</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26327,27 +26361,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.4357</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.4326</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.3806</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26372,27 +26406,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.682700000000001</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.702999999999999</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.615600000000001</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26417,27 +26451,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.7393</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.665800000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.633599999999999</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26462,27 +26496,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2121</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2155</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2265</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26507,27 +26541,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.5258</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.3488</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.3714</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26552,27 +26586,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.9885</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.6651</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.5012</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26597,27 +26631,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.8549</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.7813</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.6096</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26642,27 +26676,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.4506</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.4161</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.3372</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26687,27 +26721,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.3855</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.2475</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.3596</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
@@ -26732,27 +26766,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.9657</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.7585</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.3896</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26777,27 +26811,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>55.218</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>55.113</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.9312</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26822,27 +26856,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5237</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5269</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5212</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26867,27 +26901,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4496</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4492</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4487</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26912,27 +26946,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>42.2213</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>42.2358</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.6235</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26957,27 +26991,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.6242</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.7198</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.6842</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27002,27 +27036,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0311</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0611</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.9938</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27047,27 +27081,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.3501</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.324</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.286</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27092,27 +27126,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9655</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.8265</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.6363</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27137,27 +27171,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.8409</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.836399999999999</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.817</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27182,27 +27216,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.8025</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.793</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7673</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27227,27 +27261,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.4902</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.4554</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.4394</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27272,27 +27306,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.9628</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.9739</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>19.1215</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27317,27 +27351,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.8626</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.4122</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.3687</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27407,27 +27441,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.365</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.3158</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.262</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27452,27 +27486,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7224</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7222</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.722</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27497,27 +27531,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.1886</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1377</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.0817</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27542,27 +27576,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2404</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2401</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2397</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27587,27 +27621,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.5785</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.5186</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.7425</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -27632,27 +27666,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.1061</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.1331</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.1201</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27677,27 +27711,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.6933</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.6115</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.5324</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27730,7 +27764,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27738,7 +27772,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.190001</v>
+        <v>22.09</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27762,7 +27796,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.056</v>
+        <v>1.065</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27770,7 +27804,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27778,7 +27812,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.056</v>
+        <v>1.064</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27810,7 +27844,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27818,7 +27852,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>781.869995</v>
+        <v>769.429993</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27890,7 +27924,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27898,7 +27932,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>211.770004</v>
+        <v>208.190002</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -27922,23 +27956,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.9</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.7</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27962,23 +27996,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>195</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>197.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28002,7 +28036,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28010,7 +28044,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28018,7 +28052,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28042,7 +28076,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28050,7 +28084,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28159,23 +28193,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>62.25</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>61.25</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28199,7 +28233,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28207,7 +28241,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28239,7 +28273,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28247,7 +28281,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28255,7 +28289,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.4</v>
+        <v>16.299999</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28279,7 +28313,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28287,7 +28321,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28295,7 +28329,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.2</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28319,7 +28353,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28327,7 +28361,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28335,7 +28369,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28359,7 +28393,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.8</v>
+        <v>22.4</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28367,7 +28401,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28375,7 +28409,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.799999</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28399,7 +28433,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.42</v>
+        <v>3.4</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28407,7 +28441,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28415,7 +28449,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.42</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28447,7 +28481,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28479,7 +28513,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.3</v>
+        <v>3.26</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28487,7 +28521,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28495,7 +28529,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.3</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28519,7 +28553,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28527,7 +28561,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28535,7 +28569,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28559,7 +28593,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.7</v>
+        <v>17.2</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28567,7 +28601,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28575,7 +28609,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.700001</v>
+        <v>17.200001</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28599,7 +28633,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>118.43</v>
+        <v>116.14</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28607,7 +28641,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28615,7 +28649,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>118.43</v>
+        <v>116.139999</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28639,7 +28673,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>240.69</v>
+        <v>238.93</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28647,7 +28681,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28655,7 +28689,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>240.690002</v>
+        <v>238.929993</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28679,7 +28713,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>474.38</v>
+        <v>474.25</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28687,7 +28721,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28719,7 +28753,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>120.45</v>
+        <v>118.8</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28727,7 +28761,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28735,7 +28769,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>120.449997</v>
+        <v>118.800003</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28759,7 +28793,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>33.07</v>
+        <v>32.82</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28767,7 +28801,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28775,7 +28809,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>33.07</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28799,7 +28833,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>185.65</v>
+        <v>182.53</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28807,7 +28841,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28815,7 +28849,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>185.649994</v>
+        <v>182.529999</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28839,7 +28873,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>178.74</v>
+        <v>178.67</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28847,7 +28881,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28855,7 +28889,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>178.740005</v>
+        <v>178.669998</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28879,7 +28913,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>178.52</v>
+        <v>179.32</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28887,7 +28921,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28895,7 +28929,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>178.520004</v>
+        <v>179.320007</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -28919,7 +28953,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>187.86</v>
+        <v>187.11</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28927,7 +28961,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28935,7 +28969,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>187.860001</v>
+        <v>187.110001</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -28959,7 +28993,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1150.99</v>
+        <v>1181.89</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -28967,7 +29001,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -28975,7 +29009,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1150.98999</v>
+        <v>1181.890015</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -28999,7 +29033,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>75.53</v>
+        <v>74.69</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29007,7 +29041,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29015,7 +29049,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>75.529999</v>
+        <v>74.69000200000001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29039,7 +29073,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1355.47</v>
+        <v>1335.55</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29047,7 +29081,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29055,7 +29089,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1355.469971</v>
+        <v>1335.550049</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29079,7 +29113,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>158.25</v>
+        <v>159.73</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29087,7 +29121,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29095,7 +29129,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>156.699997</v>
+        <v>159.729996</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29119,7 +29153,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>225.51</v>
+        <v>224.58</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29127,7 +29161,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29135,7 +29169,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>225.509995</v>
+        <v>224.580002</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29159,7 +29193,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>76.70999999999999</v>
+        <v>73.44</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29167,7 +29201,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29175,7 +29209,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>76.709999</v>
+        <v>73.44000200000001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29199,7 +29233,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>119.59</v>
+        <v>116.34</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29207,7 +29241,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29215,7 +29249,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>119.589996</v>
+        <v>116.339996</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29239,7 +29273,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>389.14</v>
+        <v>387.7</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29247,7 +29281,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29255,7 +29289,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>389.140015</v>
+        <v>387.700012</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29279,7 +29313,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>380.12</v>
+        <v>377.94</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29287,7 +29321,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29295,7 +29329,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>380.119995</v>
+        <v>377.940002</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29319,7 +29353,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>38.9</v>
+        <v>38.55</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29327,7 +29361,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29335,7 +29369,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>38.900002</v>
+        <v>38.549999</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29359,7 +29393,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>68.76000000000001</v>
+        <v>66.93000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29367,7 +29401,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29375,7 +29409,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>68.760002</v>
+        <v>66.93000000000001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29399,7 +29433,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>337.02</v>
+        <v>335.92</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29407,7 +29441,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29415,7 +29449,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>337.019989</v>
+        <v>335.920013</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29439,7 +29473,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>198.13</v>
+        <v>199.21</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29447,7 +29481,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29455,7 +29489,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>198.130005</v>
+        <v>199.210007</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29479,7 +29513,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>736.595</v>
+        <v>777.59</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29487,15 +29521,15 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46288</v>
+        <v>46290</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>741.25</v>
+        <v>777.590027</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29519,7 +29553,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.6</v>
+        <v>30</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29527,7 +29561,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29559,7 +29593,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>138.3</v>
+        <v>145.83</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29567,7 +29601,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29575,7 +29609,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>147.950557</v>
+        <v>138.29858</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29599,7 +29633,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>767.25</v>
+        <v>776.15</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29607,7 +29641,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29615,7 +29649,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>790.153836</v>
+        <v>767.253888</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29639,7 +29673,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84374</v>
+        <v>84407</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29647,7 +29681,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29655,7 +29689,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>86478.783706</v>
+        <v>84374.660427</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29679,7 +29713,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009690000000000001</v>
+        <v>0.00971</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29687,7 +29721,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29695,7 +29729,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010121</v>
+        <v>0.009686999999999999</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29719,7 +29753,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.015685</v>
+        <v>0.017721</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29727,7 +29761,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29735,7 +29769,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.016517</v>
+        <v>0.015669</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29759,7 +29793,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>115.32</v>
+        <v>117.2</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29767,7 +29801,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29775,7 +29809,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>118.584192</v>
+        <v>115.313173</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29799,7 +29833,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.96</v>
+        <v>2.09</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29807,7 +29841,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29815,7 +29849,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.223066</v>
+        <v>1.962655</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29847,7 +29881,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29879,23 +29913,23 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
+        <v>0.030339</v>
+      </c>
+      <c r="F92" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G92" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H92" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
         <v>0.028767</v>
-      </c>
-      <c r="F92" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G92" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H92" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I92" t="n">
-        <v>0.02976</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29919,7 +29953,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.316022</v>
+        <v>7.262467</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29927,7 +29961,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29935,7 +29969,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>8.101755000000001</v>
+        <v>7.313846</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29959,7 +29993,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>32.152071</v>
+        <v>34.2555</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -29967,7 +30001,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -29975,7 +30009,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>34.233119</v>
+        <v>32.128488</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -29999,7 +30033,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.149721</v>
+        <v>0.155077</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30007,7 +30041,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30015,7 +30049,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.160425</v>
+        <v>0.149676</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30039,7 +30073,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25649.1675</v>
+        <v>25938.933</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30047,7 +30081,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30055,7 +30089,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>26414.842739</v>
+        <v>25641.624949</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30079,7 +30113,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2820622.82</v>
+        <v>2820881.94</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30087,7 +30121,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30095,7 +30129,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2890985.739277</v>
+        <v>2819801.151471</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30119,7 +30153,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.117314</v>
+        <v>3.205546</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30127,7 +30161,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30135,7 +30169,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.403605</v>
+        <v>3.116386</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30159,7 +30193,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89883.24099999999</v>
+        <v>89689.254</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30167,7 +30201,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30175,7 +30209,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>92240.74178700001</v>
+        <v>89856.394705</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30199,7 +30233,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.59649</v>
+        <v>20.725079</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30207,7 +30241,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30215,7 +30249,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>21.181361</v>
+        <v>20.590323</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30239,7 +30273,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84374</v>
+        <v>84407</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30247,7 +30281,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30255,7 +30289,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>86478.783706</v>
+        <v>84374.660427</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30279,7 +30313,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>22.42</v>
+        <v>23.54</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30287,7 +30321,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30295,7 +30329,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.129539</v>
+        <v>22.425047</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30393,7 +30427,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009690000000000001</v>
+        <v>0.00971</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30401,7 +30435,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30409,7 +30443,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010121</v>
+        <v>0.009686999999999999</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30433,7 +30467,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>115.32</v>
+        <v>117.2</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30441,7 +30475,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30449,7 +30483,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>118.584192</v>
+        <v>115.313173</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30481,7 +30515,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30513,27 +30547,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.9934</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.4705</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46283</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.463</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-26
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L121"/>
+  <dimension ref="B2:L122"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25511,6 +25511,40 @@
         <v>33.42</v>
       </c>
       <c r="K121" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="72" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C122" t="n">
+        <v>26799121</v>
+      </c>
+      <c r="D122" t="n">
+        <v>22848642</v>
+      </c>
+      <c r="E122" t="n">
+        <v>3950478</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.1729</v>
+      </c>
+      <c r="G122" t="n">
+        <v>18777396</v>
+      </c>
+      <c r="H122" t="n">
+        <v>5017016</v>
+      </c>
+      <c r="I122" t="n">
+        <v>1610548</v>
+      </c>
+      <c r="J122" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="K122" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26088,7 +26122,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26103,11 +26137,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.42</v>
+        <v>33.37</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-25</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -26152,11 +26186,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1365</v>
+        <v>26.1271</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-25</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -26271,27 +26305,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.1679</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.4002</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>21.1786</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26316,27 +26350,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.705</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7048</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7047</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26361,27 +26395,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3983</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.4357</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.4326</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26406,27 +26440,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.6309</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.682700000000001</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.702999999999999</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26451,27 +26485,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.7212</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.7393</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.665800000000001</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26496,27 +26530,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.2248</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2121</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2155</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26541,27 +26575,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.3761</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.5258</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.3488</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26586,27 +26620,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.6109</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.9885</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.6651</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26631,27 +26665,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.6601</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.8549</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.7813</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26676,27 +26710,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.3337</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.4506</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.4161</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26721,27 +26755,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.4512</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.3855</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.2475</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -26766,27 +26800,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.50620000000001</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.9657</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.7585</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26811,27 +26845,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.9241</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>55.218</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>55.113</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26856,27 +26890,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.5022</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5237</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5269</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26901,27 +26935,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4501</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4496</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4492</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26946,27 +26980,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.9156</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>42.2213</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>42.2358</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26991,27 +27025,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.4409</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.6242</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.7198</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27036,27 +27070,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0312</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0311</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0611</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27081,27 +27115,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.2785</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.3501</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.324</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27126,27 +27160,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9426</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9655</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.8265</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27171,27 +27205,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.797499999999999</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.8409</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.836399999999999</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27216,27 +27250,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7415</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.8025</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.793</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27261,27 +27295,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.2831</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.4902</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.4554</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27306,27 +27340,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.7148</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.9628</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.9739</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27351,27 +27385,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.9323</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.8626</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.4122</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27396,7 +27430,7 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
-        <v>37.2415</v>
+        <v>37.6929</v>
       </c>
       <c r="F30" s="34" t="inlineStr">
         <is>
@@ -27404,7 +27438,7 @@
         </is>
       </c>
       <c r="G30" s="28" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="H30" s="34" t="inlineStr">
         <is>
@@ -27412,11 +27446,11 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>35.56</v>
+        <v>37.8699</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27441,27 +27475,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.298</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.365</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.3158</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27486,27 +27520,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7226</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7224</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7222</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27531,27 +27565,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.1539</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1886</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1377</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27576,27 +27610,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2408</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2404</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2401</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27621,27 +27655,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.0982</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.5785</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.5186</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -27666,27 +27700,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0415</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.1061</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.1331</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27711,27 +27745,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.5898</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.6933</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.6115</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27756,7 +27790,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.19</v>
+        <v>22.09</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27764,7 +27798,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27772,7 +27806,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>22.09</v>
+        <v>21.959999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27796,7 +27830,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.065</v>
+        <v>1.064</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27804,7 +27838,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27812,7 +27846,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.064</v>
+        <v>1.052</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27836,7 +27870,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>781.87</v>
+        <v>769.4299999999999</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27844,7 +27878,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27852,7 +27886,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>769.429993</v>
+        <v>783.580017</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -27916,7 +27950,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>211.77</v>
+        <v>208.19</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -27924,7 +27958,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27956,23 +27990,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46291</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.7</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.9</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -27996,23 +28030,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>193</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46291</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>192.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>195</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28044,7 +28078,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28076,7 +28110,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28084,7 +28118,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28193,23 +28227,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>60.75</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46291</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>60.5</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>62.25</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28233,7 +28267,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28241,7 +28275,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28249,7 +28283,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>12.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28281,7 +28315,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28313,7 +28347,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28321,7 +28355,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28361,7 +28395,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28393,7 +28427,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.4</v>
+        <v>22.3</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28401,7 +28435,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28409,7 +28443,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.4</v>
+        <v>22.299999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28441,7 +28475,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28481,7 +28515,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28521,7 +28555,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28553,7 +28587,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28561,7 +28595,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28569,7 +28603,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28593,7 +28627,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28601,7 +28635,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28609,7 +28643,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.200001</v>
+        <v>17.299999</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28633,7 +28667,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>116.14</v>
+        <v>123.11</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28641,7 +28675,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28673,7 +28707,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>238.93</v>
+        <v>235.47</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28681,7 +28715,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28713,23 +28747,23 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
+        <v>485</v>
+      </c>
+      <c r="F62" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G62" s="28" t="n">
+        <v>46291</v>
+      </c>
+      <c r="H62" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
         <v>474.25</v>
-      </c>
-      <c r="F62" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G62" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H62" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I62" t="n">
-        <v>474.380005</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28753,7 +28787,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>118.8</v>
+        <v>119.92</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28761,7 +28795,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28793,7 +28827,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>32.82</v>
+        <v>32.4</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28801,7 +28835,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28833,7 +28867,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>182.53</v>
+        <v>187.18</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28841,7 +28875,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28873,7 +28907,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>178.67</v>
+        <v>173.46</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28881,7 +28915,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28913,7 +28947,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>179.32</v>
+        <v>187.9</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -28921,7 +28955,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28953,7 +28987,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>187.11</v>
+        <v>187.92</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -28961,7 +28995,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -28993,7 +29027,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1181.89</v>
+        <v>1183.46</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29001,7 +29035,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29033,7 +29067,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>74.69</v>
+        <v>78.69</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29041,7 +29075,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29073,7 +29107,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1335.55</v>
+        <v>1367.43</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29081,7 +29115,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29113,7 +29147,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>159.73</v>
+        <v>159.03</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29121,7 +29155,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29153,7 +29187,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>224.58</v>
+        <v>225.07</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29161,7 +29195,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29193,7 +29227,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>73.44</v>
+        <v>77.39</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29201,7 +29235,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29233,7 +29267,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>116.34</v>
+        <v>117.97</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29241,7 +29275,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29273,7 +29307,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>387.7</v>
+        <v>398.38</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29281,7 +29315,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29313,7 +29347,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>377.94</v>
+        <v>372.11</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29321,7 +29355,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29353,7 +29387,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>38.55</v>
+        <v>39.6</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29361,7 +29395,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29393,7 +29427,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>66.93000000000001</v>
+        <v>66.66</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29401,7 +29435,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29433,7 +29467,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>335.92</v>
+        <v>341.07</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29441,7 +29475,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29473,7 +29507,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>199.21</v>
+        <v>195.11</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29481,7 +29515,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29513,7 +29547,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>777.59</v>
+        <v>751.66</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29521,7 +29555,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29553,7 +29587,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30</v>
+        <v>30.18</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29561,7 +29595,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29569,7 +29603,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.6</v>
+        <v>30.18</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29593,7 +29627,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>145.83</v>
+        <v>154.71</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29601,7 +29635,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29609,7 +29643,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>138.29858</v>
+        <v>146.291618</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29633,7 +29667,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>776.15</v>
+        <v>775.4299999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29641,7 +29675,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29649,7 +29683,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>767.253888</v>
+        <v>776.842516</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29673,7 +29707,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84407</v>
+        <v>83939</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29681,7 +29715,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29689,7 +29723,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84374.660427</v>
+        <v>84501.78264</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29713,7 +29747,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00971</v>
+        <v>0.010234</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29721,7 +29755,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29729,7 +29763,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009686999999999999</v>
+        <v>0.009731999999999999</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29753,7 +29787,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017721</v>
+        <v>0.018543</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29761,7 +29795,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29769,7 +29803,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.015669</v>
+        <v>0.017756</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29793,7 +29827,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>117.2</v>
+        <v>121.74</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29801,7 +29835,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29809,7 +29843,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>115.313173</v>
+        <v>117.438209</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29833,7 +29867,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.09</v>
+        <v>2.12</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29841,7 +29875,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29849,7 +29883,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.962655</v>
+        <v>2.09893</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29881,7 +29915,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29913,7 +29947,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.030339</v>
+        <v>0.035581</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29921,7 +29955,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29929,7 +29963,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.028767</v>
+        <v>0.030526</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29953,7 +29987,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.262467</v>
+        <v>7.4928</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29961,7 +29995,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -29969,7 +30003,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.313846</v>
+        <v>7.276189</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -29993,7 +30027,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>34.2555</v>
+        <v>39.3766</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30001,7 +30035,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30009,7 +30043,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>32.128488</v>
+        <v>34.516257</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30033,7 +30067,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.155077</v>
+        <v>0.156555</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30041,7 +30075,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30049,7 +30083,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.149676</v>
+        <v>0.155192</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30073,7 +30107,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25938.933</v>
+        <v>25876.0991</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30081,7 +30115,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30089,7 +30123,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25641.624949</v>
+        <v>25923.234757</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30113,7 +30147,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2820881.94</v>
+        <v>2801044.43</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30121,7 +30155,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30129,7 +30163,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2819801.151471</v>
+        <v>2819824.486689</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30153,7 +30187,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.205546</v>
+        <v>3.299225</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30161,7 +30195,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30169,7 +30203,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.116386</v>
+        <v>3.208523</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30193,7 +30227,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89689.254</v>
+        <v>89735.9344</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30201,7 +30235,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30209,7 +30243,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89856.394705</v>
+        <v>89707.053337</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30233,7 +30267,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.725079</v>
+        <v>20.550381</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30241,7 +30275,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30249,7 +30283,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.590323</v>
+        <v>20.694907</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30273,7 +30307,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84407</v>
+        <v>83939</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30281,7 +30315,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30289,7 +30323,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84374.660427</v>
+        <v>84501.78264</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30313,7 +30347,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.54</v>
+        <v>23.99</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30321,7 +30355,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30329,7 +30363,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>22.425047</v>
+        <v>23.600135</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30427,7 +30461,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00971</v>
+        <v>0.010234</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30435,7 +30469,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30443,7 +30477,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009686999999999999</v>
+        <v>0.009731999999999999</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30467,7 +30501,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>117.2</v>
+        <v>121.74</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30475,7 +30509,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30483,7 +30517,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>115.313173</v>
+        <v>117.438209</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30515,7 +30549,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30547,27 +30581,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.9698</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.9934</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.4705</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-09-26
FX 33.37 · 98 updated · 1 MF carried · 5 manual
SEC NAV: matched 33/34 via SEC /v2/fund; no NAV: ASP-FLEXPLUS
Total ฿26,722,925 · P&L +16.96%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25521,25 +25521,25 @@
         <v>46291</v>
       </c>
       <c r="C122" t="n">
-        <v>26799121</v>
+        <v>26722925</v>
       </c>
       <c r="D122" t="n">
         <v>22848642</v>
       </c>
       <c r="E122" t="n">
-        <v>3950478</v>
+        <v>3874283</v>
       </c>
       <c r="F122" t="n">
-        <v>0.1729</v>
+        <v>0.1696</v>
       </c>
       <c r="G122" t="n">
-        <v>18777396</v>
+        <v>18696995</v>
       </c>
       <c r="H122" t="n">
         <v>5017016</v>
       </c>
       <c r="I122" t="n">
-        <v>1610548</v>
+        <v>1609220</v>
       </c>
       <c r="J122" t="n">
         <v>33.37</v>
@@ -26305,27 +26305,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.342</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.1679</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>21.4002</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26350,27 +26350,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7052</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.705</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7048</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26395,27 +26395,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3252</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3983</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.4357</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26440,27 +26440,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.5817</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.6309</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.682700000000001</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26530,27 +26530,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.1793</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.2248</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2121</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26575,27 +26575,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.4245</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.3761</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.5258</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26620,27 +26620,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.8452</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.6109</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.9885</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26665,27 +26665,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.7421</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.6601</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.8549</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26710,27 +26710,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.3637</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.3337</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.4506</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26755,27 +26755,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.1799</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.4512</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.3855</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>
@@ -26800,27 +26800,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.71299999999999</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.50620000000001</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.9657</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26845,27 +26845,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.9916</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.9241</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>55.218</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26890,27 +26890,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.507</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.5022</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5237</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26935,27 +26935,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4506</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4501</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4496</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26980,27 +26980,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.9076</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.9156</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>42.2213</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27070,27 +27070,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>14.0265</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0312</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0311</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27115,27 +27115,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.28</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.2785</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.3501</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27160,27 +27160,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.8488</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9426</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.9655</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27205,27 +27205,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.818300000000001</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.797499999999999</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.8409</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27250,27 +27250,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7694</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7415</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.8025</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27295,27 +27295,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.3119</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.2831</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.4902</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27340,27 +27340,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.8739</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.7148</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.9628</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27385,27 +27385,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.5455</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.9323</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>25.8626</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27430,27 +27430,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>37.3329</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>37.6929</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.8699</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27475,27 +27475,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.3333</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.298</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.365</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27520,27 +27520,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7228</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7226</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7224</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27565,27 +27565,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.1493</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1539</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1886</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27610,27 +27610,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2412</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2408</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2404</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27655,27 +27655,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.2031</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.0982</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.5785</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -27700,27 +27700,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0603</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0415</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.1061</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27745,27 +27745,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.6325</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.5898</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.6933</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27790,7 +27790,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>22.09</v>
+        <v>21.96</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27830,7 +27830,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.064</v>
+        <v>1.052</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27870,7 +27870,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>769.4299999999999</v>
+        <v>783.58</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -28683,7 +28683,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>116.139999</v>
+        <v>123.110001</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28723,7 +28723,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>238.929993</v>
+        <v>235.470001</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28803,7 +28803,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>118.800003</v>
+        <v>119.919998</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28843,7 +28843,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>32.82</v>
+        <v>32.400002</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28883,7 +28883,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>182.529999</v>
+        <v>187.179993</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -28923,7 +28923,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>178.669998</v>
+        <v>173.460007</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -28963,7 +28963,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>179.320007</v>
+        <v>187.899994</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29003,7 +29003,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>187.110001</v>
+        <v>187.919998</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29043,7 +29043,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1181.890015</v>
+        <v>1183.459961</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29083,7 +29083,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>74.69000200000001</v>
+        <v>78.69000200000001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29123,7 +29123,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1335.550049</v>
+        <v>1367.430054</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29163,7 +29163,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>159.729996</v>
+        <v>159.029999</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29203,7 +29203,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>224.580002</v>
+        <v>225.070007</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29243,7 +29243,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>73.44000200000001</v>
+        <v>77.389999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29283,7 +29283,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>116.339996</v>
+        <v>117.970001</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29323,7 +29323,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>387.700012</v>
+        <v>398.380005</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29363,7 +29363,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>377.940002</v>
+        <v>372.109985</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29403,7 +29403,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>38.549999</v>
+        <v>39.599998</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29443,7 +29443,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>66.93000000000001</v>
+        <v>66.660004</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29483,7 +29483,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>335.920013</v>
+        <v>341.070007</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29523,7 +29523,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>199.210007</v>
+        <v>195.110001</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29563,7 +29563,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>777.590027</v>
+        <v>751.659973</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29627,7 +29627,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>154.71</v>
+        <v>153.66</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29643,7 +29643,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>146.291618</v>
+        <v>145.143279</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29667,7 +29667,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>775.4299999999999</v>
+        <v>774.5700000000001</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29683,7 +29683,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>776.842516</v>
+        <v>772.611212</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29707,7 +29707,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83939</v>
+        <v>83923</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29723,7 +29723,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84501.78264</v>
+        <v>84241.286924</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29747,7 +29747,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010234</v>
+        <v>0.010204</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29763,7 +29763,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009731999999999999</v>
+        <v>0.009593000000000001</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29787,7 +29787,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018543</v>
+        <v>0.018744</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29803,7 +29803,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017756</v>
+        <v>0.017546</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29827,7 +29827,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>121.74</v>
+        <v>120.8</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29843,7 +29843,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>117.438209</v>
+        <v>116.887254</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29867,7 +29867,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.12</v>
+        <v>2.13</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29883,7 +29883,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.09893</v>
+        <v>2.068273</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29947,7 +29947,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035581</v>
+        <v>0.037051</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29963,7 +29963,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.030526</v>
+        <v>0.029991</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29987,7 +29987,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.4928</v>
+        <v>7.39646</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30003,7 +30003,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.276189</v>
+        <v>7.200462</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30027,7 +30027,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.3766</v>
+        <v>39.0429</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30043,7 +30043,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>34.516257</v>
+        <v>33.666326</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30067,7 +30067,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.156555</v>
+        <v>0.1564</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30083,7 +30083,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.155192</v>
+        <v>0.153418</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30107,7 +30107,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25876.0991</v>
+        <v>25847.4009</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30123,7 +30123,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25923.234757</v>
+        <v>25782.036133</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30147,7 +30147,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2801044.43</v>
+        <v>2800510.51</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30163,7 +30163,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2819824.486689</v>
+        <v>2811131.744657</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30187,7 +30187,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.299225</v>
+        <v>3.274164</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30203,7 +30203,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.208523</v>
+        <v>3.167804</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30227,7 +30227,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89735.9344</v>
+        <v>89657.18120000001</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30243,7 +30243,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89707.053337</v>
+        <v>89294.722757</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30267,7 +30267,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.550381</v>
+        <v>20.632638</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30283,7 +30283,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.694907</v>
+        <v>20.603877</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30307,7 +30307,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83939</v>
+        <v>83923</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30323,7 +30323,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84501.78264</v>
+        <v>84241.286924</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30347,7 +30347,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.99</v>
+        <v>24.11</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30363,7 +30363,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.600135</v>
+        <v>23.370384</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30461,7 +30461,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010234</v>
+        <v>0.010204</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30477,7 +30477,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009731999999999999</v>
+        <v>0.009593000000000001</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30501,7 +30501,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>121.74</v>
+        <v>120.8</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30517,7 +30517,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>117.438209</v>
+        <v>116.887254</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30581,27 +30581,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.8045</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.9698</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46287</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.9934</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-09-27
FX 33.37 · 94 updated · 5 MF carried · 5 manual
SEC NAV: matched 29/34 via SEC /v2/fund; no NAV: ASP-AIEQ, ASP-EUG, ASP-SME-A, ASP-THGEQ-T, B-EQUITY
Total ฿26,727,295 · P&L +16.98% · 150 history point(s) · perf history 150d
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L122"/>
+  <dimension ref="B2:L123"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25545,6 +25545,40 @@
         <v>33.37</v>
       </c>
       <c r="K122" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="72" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C123" t="n">
+        <v>26727295</v>
+      </c>
+      <c r="D123" t="n">
+        <v>22848642</v>
+      </c>
+      <c r="E123" t="n">
+        <v>3878653</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.1698</v>
+      </c>
+      <c r="G123" t="n">
+        <v>18697211</v>
+      </c>
+      <c r="H123" t="n">
+        <v>5017016</v>
+      </c>
+      <c r="I123" t="n">
+        <v>1613374</v>
+      </c>
+      <c r="J123" t="n">
+        <v>33.37</v>
+      </c>
+      <c r="K123" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26122,7 +26156,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26141,7 +26175,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-26</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-27</t>
         </is>
       </c>
     </row>
@@ -26190,7 +26224,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-26</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-27</t>
         </is>
       </c>
     </row>
@@ -26485,27 +26519,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.764799999999999</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.7212</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.7393</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27798,7 +27832,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27838,7 +27872,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27878,7 +27912,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27958,7 +27992,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -27998,7 +28032,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28038,7 +28072,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -28078,7 +28112,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28118,7 +28152,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28235,7 +28269,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28275,7 +28309,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28315,7 +28349,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28355,7 +28389,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28395,7 +28429,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28435,7 +28469,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28475,7 +28509,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28515,7 +28549,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28555,7 +28589,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28595,7 +28629,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28635,7 +28669,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28675,7 +28709,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28715,7 +28749,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28755,7 +28789,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28795,7 +28829,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28835,7 +28869,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28875,7 +28909,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28915,7 +28949,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28955,7 +28989,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -28995,7 +29029,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29035,7 +29069,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29075,7 +29109,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29115,7 +29149,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29155,7 +29189,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29195,7 +29229,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29235,7 +29269,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29275,7 +29309,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29315,7 +29349,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29355,7 +29389,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29395,7 +29429,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29435,7 +29469,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29475,7 +29509,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29515,7 +29549,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29555,7 +29589,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29595,7 +29629,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29627,7 +29661,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>153.66</v>
+        <v>156.2</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29635,7 +29669,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29643,7 +29677,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>145.143279</v>
+        <v>154.98889</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29667,7 +29701,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>774.5700000000001</v>
+        <v>772.98</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29675,7 +29709,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29683,7 +29717,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>772.611212</v>
+        <v>775.731017</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29707,7 +29741,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83923</v>
+        <v>84363</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29715,7 +29749,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29723,7 +29757,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84241.286924</v>
+        <v>83941.414233</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29747,7 +29781,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010204</v>
+        <v>0.00979</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29755,7 +29789,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29763,7 +29797,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009593000000000001</v>
+        <v>0.010304</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29787,7 +29821,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018744</v>
+        <v>0.017869</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29795,7 +29829,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29803,7 +29837,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017546</v>
+        <v>0.018718</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29827,7 +29861,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>120.8</v>
+        <v>121.05</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29835,7 +29869,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29843,7 +29877,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>116.887254</v>
+        <v>121.846837</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29867,7 +29901,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.13</v>
+        <v>2.1</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29875,7 +29909,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29883,7 +29917,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.068273</v>
+        <v>2.114457</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29915,7 +29949,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29947,7 +29981,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.037051</v>
+        <v>0.036759</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29955,7 +29989,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29963,7 +29997,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.029991</v>
+        <v>0.035602</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -29987,7 +30021,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.39646</v>
+        <v>7.596414</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -29995,7 +30029,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30003,7 +30037,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.200462</v>
+        <v>7.472681</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30035,7 +30069,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30043,7 +30077,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>33.666326</v>
+        <v>39.418493</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30067,7 +30101,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.1564</v>
+        <v>0.156086</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30075,7 +30109,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30083,7 +30117,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.153418</v>
+        <v>0.1567</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30107,7 +30141,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25847.4009</v>
+        <v>25794.3426</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30115,7 +30149,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30123,7 +30157,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25782.036133</v>
+        <v>25886.144052</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30147,7 +30181,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2800510.51</v>
+        <v>2815193.31</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30155,7 +30189,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30163,7 +30197,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2811131.744657</v>
+        <v>2801124.992954</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30187,7 +30221,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.274164</v>
+        <v>3.215934</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30195,7 +30229,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30203,7 +30237,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.167804</v>
+        <v>3.299801</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30227,7 +30261,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89657.18120000001</v>
+        <v>89922.139</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30235,7 +30269,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30243,7 +30277,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89294.722757</v>
+        <v>89759.68412799999</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30267,7 +30301,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.632638</v>
+        <v>20.518546</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30275,7 +30309,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30283,7 +30317,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.603877</v>
+        <v>20.542875</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30307,7 +30341,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83923</v>
+        <v>84363</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30315,7 +30349,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30323,7 +30357,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84241.286924</v>
+        <v>83941.414233</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30347,7 +30381,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.11</v>
+        <v>23.93</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30355,7 +30389,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30363,7 +30397,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.370384</v>
+        <v>23.987701</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30461,7 +30495,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010204</v>
+        <v>0.00979</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30469,7 +30503,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30477,7 +30511,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009593000000000001</v>
+        <v>0.010304</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30501,7 +30535,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>120.8</v>
+        <v>121.05</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30509,7 +30543,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30517,7 +30551,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>116.887254</v>
+        <v>121.846837</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30549,7 +30583,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-27
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25555,16 +25555,16 @@
         <v>46292</v>
       </c>
       <c r="C123" t="n">
-        <v>26727295</v>
+        <v>26725405</v>
       </c>
       <c r="D123" t="n">
         <v>22848642</v>
       </c>
       <c r="E123" t="n">
-        <v>3878653</v>
+        <v>3876763</v>
       </c>
       <c r="F123" t="n">
-        <v>0.1698</v>
+        <v>0.1697</v>
       </c>
       <c r="G123" t="n">
         <v>18697211</v>
@@ -25573,7 +25573,7 @@
         <v>5017016</v>
       </c>
       <c r="I123" t="n">
-        <v>1613374</v>
+        <v>1611483</v>
       </c>
       <c r="J123" t="n">
         <v>33.37</v>
@@ -29661,7 +29661,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>156.2</v>
+        <v>154.73</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29677,7 +29677,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>154.98889</v>
+        <v>154.419218</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29701,7 +29701,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>772.98</v>
+        <v>772.37</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29717,7 +29717,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>775.731017</v>
+        <v>775.32831</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29741,7 +29741,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84363</v>
+        <v>84326</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29757,7 +29757,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83941.414233</v>
+        <v>83934.464097</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29781,7 +29781,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00979</v>
+        <v>0.009733</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29797,7 +29797,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010304</v>
+        <v>0.010213</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29821,7 +29821,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017869</v>
+        <v>0.017742</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29837,7 +29837,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018718</v>
+        <v>0.018545</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29861,7 +29861,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>121.05</v>
+        <v>120.82</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29877,7 +29877,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>121.846837</v>
+        <v>121.60798</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29901,7 +29901,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29917,7 +29917,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.114457</v>
+        <v>2.113396</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29981,7 +29981,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.036759</v>
+        <v>0.036579</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29997,7 +29997,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035602</v>
+        <v>0.035582</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30021,7 +30021,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.596414</v>
+        <v>7.504279</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30037,7 +30037,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.472681</v>
+        <v>7.477642</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30061,7 +30061,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.0429</v>
+        <v>38.7092</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30077,7 +30077,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.418493</v>
+        <v>39.070109</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30101,7 +30101,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.156086</v>
+        <v>0.156124</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30117,7 +30117,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.1567</v>
+        <v>0.156562</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30141,7 +30141,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25794.3426</v>
+        <v>25773.9869</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30157,7 +30157,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25886.144052</v>
+        <v>25872.705707</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30181,7 +30181,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2815193.31</v>
+        <v>2813958.62</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30197,7 +30197,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2801124.992954</v>
+        <v>2800893.066911</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30221,7 +30221,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.215934</v>
+        <v>3.20352</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30237,7 +30237,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.299801</v>
+        <v>3.295711</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30261,7 +30261,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89922.139</v>
+        <v>89861.0719</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30277,7 +30277,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89759.68412799999</v>
+        <v>89716.62892</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30301,7 +30301,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.518546</v>
+        <v>20.405655</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30317,7 +30317,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.542875</v>
+        <v>20.550013</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30341,7 +30341,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84363</v>
+        <v>84326</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30357,7 +30357,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83941.414233</v>
+        <v>83934.464097</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30381,7 +30381,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.93</v>
+        <v>23.83</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30397,7 +30397,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.987701</v>
+        <v>23.989639</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30495,7 +30495,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00979</v>
+        <v>0.009733</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30511,7 +30511,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010304</v>
+        <v>0.010213</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30535,7 +30535,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>121.05</v>
+        <v>120.82</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30551,7 +30551,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>121.846837</v>
+        <v>121.60798</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-09-28
FX 33.45 · 98 updated · 1 MF carried · 5 manual
SEC NAV: matched 33/34 via SEC /v2/fund; no NAV: UTSB-THAIESG
Total ฿26,741,107 · P&L +16.98%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L123"/>
+  <dimension ref="B2:L124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25579,6 +25579,40 @@
         <v>33.37</v>
       </c>
       <c r="K123" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="72" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C124" t="n">
+        <v>26741107</v>
+      </c>
+      <c r="D124" t="n">
+        <v>22858823</v>
+      </c>
+      <c r="E124" t="n">
+        <v>3882284</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.1698</v>
+      </c>
+      <c r="G124" t="n">
+        <v>18697211</v>
+      </c>
+      <c r="H124" t="n">
+        <v>5024946</v>
+      </c>
+      <c r="I124" t="n">
+        <v>1615806</v>
+      </c>
+      <c r="J124" t="n">
+        <v>33.45</v>
+      </c>
+      <c r="K124" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26156,7 +26190,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26171,11 +26205,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.37</v>
+        <v>33.45</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-27</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26220,11 +26254,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1271</v>
+        <v>26.1915</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-27</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27832,7 +27866,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27872,7 +27906,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27912,7 +27946,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27992,7 +28026,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28032,7 +28066,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28072,7 +28106,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -28112,7 +28146,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28152,7 +28186,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28269,7 +28303,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28309,7 +28343,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28349,7 +28383,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28389,7 +28423,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28429,7 +28463,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28469,7 +28503,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28509,7 +28543,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28549,7 +28583,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28589,7 +28623,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28629,7 +28663,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28669,7 +28703,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28709,7 +28743,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28749,7 +28783,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28789,7 +28823,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28829,7 +28863,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28869,7 +28903,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28909,7 +28943,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28949,7 +28983,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -28989,7 +29023,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29029,7 +29063,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29069,7 +29103,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29109,7 +29143,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29149,7 +29183,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29189,7 +29223,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29229,7 +29263,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29269,7 +29303,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29309,7 +29343,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29349,7 +29383,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29389,7 +29423,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29429,7 +29463,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29469,7 +29503,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29509,7 +29543,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29549,7 +29583,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29589,7 +29623,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29629,7 +29663,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29661,7 +29695,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>154.73</v>
+        <v>153.12</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29669,7 +29703,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29677,7 +29711,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>154.419218</v>
+        <v>156.258374</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29701,7 +29735,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>772.37</v>
+        <v>776.96</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29709,7 +29743,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29717,7 +29751,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>775.32831</v>
+        <v>773.227234</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29741,7 +29775,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84326</v>
+        <v>83960</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29749,7 +29783,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29757,7 +29791,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83934.464097</v>
+        <v>84383.371222</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29781,7 +29815,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009733</v>
+        <v>0.010195</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29789,7 +29823,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29797,7 +29831,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010213</v>
+        <v>0.009787000000000001</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29821,7 +29855,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017742</v>
+        <v>0.018469</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29829,7 +29863,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29837,7 +29871,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018545</v>
+        <v>0.017884</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29861,7 +29895,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>120.82</v>
+        <v>121.48</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29869,7 +29903,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29877,7 +29911,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>121.60798</v>
+        <v>121.060563</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29901,7 +29935,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.09</v>
+        <v>2.11</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29909,7 +29943,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29917,7 +29951,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.113396</v>
+        <v>2.104305</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29949,7 +29983,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -29981,7 +30015,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.036579</v>
+        <v>0.035488</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -29989,7 +30023,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -29997,7 +30031,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035582</v>
+        <v>0.036785</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30021,7 +30055,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.504279</v>
+        <v>7.451757</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30029,7 +30063,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30037,7 +30071,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.477642</v>
+        <v>7.611188</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30061,7 +30095,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>38.7092</v>
+        <v>42.147</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30069,7 +30103,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30077,7 +30111,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.070109</v>
+        <v>38.970013</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30101,7 +30135,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.156124</v>
+        <v>0.167404</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30109,7 +30143,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30117,7 +30151,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.156562</v>
+        <v>0.156508</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30141,7 +30175,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25773.9869</v>
+        <v>25989.312</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30149,7 +30183,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30157,7 +30191,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25872.705707</v>
+        <v>25864.450986</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30181,7 +30215,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2813958.62</v>
+        <v>2808462</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30189,7 +30223,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30197,7 +30231,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2800893.066911</v>
+        <v>2822623.767376</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30221,7 +30255,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.20352</v>
+        <v>3.216284</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30229,7 +30263,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30237,7 +30271,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.295711</v>
+        <v>3.224358</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30261,7 +30295,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89861.0719</v>
+        <v>89243.5965</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30269,7 +30303,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30277,7 +30311,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89716.62892</v>
+        <v>90140.93494000001</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30301,7 +30335,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.405655</v>
+        <v>20.667885</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30309,7 +30343,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30317,7 +30351,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.550013</v>
+        <v>20.575942</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30341,7 +30375,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84326</v>
+        <v>83960</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30349,7 +30383,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30357,7 +30391,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83934.464097</v>
+        <v>84383.371222</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30381,7 +30415,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.83</v>
+        <v>24.28</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30389,7 +30423,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30397,7 +30431,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.989639</v>
+        <v>23.947579</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30495,7 +30529,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009733</v>
+        <v>0.010195</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30503,7 +30537,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30511,7 +30545,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010213</v>
+        <v>0.009787000000000001</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30535,7 +30569,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>120.82</v>
+        <v>121.48</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30543,7 +30577,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30551,7 +30585,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>121.60798</v>
+        <v>121.060563</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30583,7 +30617,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-28
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25589,28 +25589,28 @@
         <v>46293</v>
       </c>
       <c r="C124" t="n">
-        <v>26741107</v>
+        <v>26745641</v>
       </c>
       <c r="D124" t="n">
-        <v>22858823</v>
+        <v>22859643</v>
       </c>
       <c r="E124" t="n">
-        <v>3882284</v>
+        <v>3885998</v>
       </c>
       <c r="F124" t="n">
-        <v>0.1698</v>
+        <v>0.17</v>
       </c>
       <c r="G124" t="n">
         <v>18697211</v>
       </c>
       <c r="H124" t="n">
-        <v>5024946</v>
+        <v>5025937</v>
       </c>
       <c r="I124" t="n">
-        <v>1615806</v>
+        <v>1619649</v>
       </c>
       <c r="J124" t="n">
-        <v>33.45</v>
+        <v>33.46</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -26205,7 +26205,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.45</v>
+        <v>33.46</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -26254,7 +26254,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1915</v>
+        <v>26.1859</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -29695,7 +29695,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>153.12</v>
+        <v>153.8</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29711,7 +29711,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>156.258374</v>
+        <v>154.880053</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29735,7 +29735,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>776.96</v>
+        <v>778.87</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29751,7 +29751,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>773.227234</v>
+        <v>772.277725</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29775,7 +29775,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83960</v>
+        <v>84074</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29791,7 +29791,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84383.371222</v>
+        <v>84322.76727500001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29815,7 +29815,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010195</v>
+        <v>0.010307</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29831,7 +29831,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009787000000000001</v>
+        <v>0.009747</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29855,7 +29855,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018469</v>
+        <v>0.018565</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29871,7 +29871,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017884</v>
+        <v>0.017755</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29895,7 +29895,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>121.48</v>
+        <v>121.96</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29911,7 +29911,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>121.060563</v>
+        <v>120.812106</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29935,7 +29935,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29951,7 +29951,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.104305</v>
+        <v>2.092943</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30015,7 +30015,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035488</v>
+        <v>0.035506</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30031,7 +30031,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.036785</v>
+        <v>0.036564</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30055,7 +30055,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.451757</v>
+        <v>7.525355</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30071,7 +30071,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.611188</v>
+        <v>7.534415</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30095,7 +30095,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>42.147</v>
+        <v>42.4942</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30111,7 +30111,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>38.970013</v>
+        <v>38.856133</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30135,7 +30135,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.167404</v>
+        <v>0.167227</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30151,7 +30151,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.156508</v>
+        <v>0.156229</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30175,7 +30175,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25989.312</v>
+        <v>26060.9902</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30191,7 +30191,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25864.450986</v>
+        <v>25840.412676</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30215,7 +30215,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2808462</v>
+        <v>2813116.04</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30231,7 +30231,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2822623.767376</v>
+        <v>2821439.793031</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30255,7 +30255,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.216284</v>
+        <v>3.243713</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30271,7 +30271,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.224358</v>
+        <v>3.214545</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30295,7 +30295,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89243.5965</v>
+        <v>89462.00199999999</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30311,7 +30311,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90140.93494000001</v>
+        <v>90094.316062</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30335,7 +30335,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.667885</v>
+        <v>20.683701</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30351,7 +30351,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.575942</v>
+        <v>20.4607</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30375,7 +30375,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83960</v>
+        <v>84074</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30391,7 +30391,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84383.371222</v>
+        <v>84322.76727500001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30415,7 +30415,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.28</v>
+        <v>24.32</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30431,7 +30431,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.947579</v>
+        <v>23.851576</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30529,7 +30529,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010195</v>
+        <v>0.010307</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30545,7 +30545,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009787000000000001</v>
+        <v>0.009747</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30569,7 +30569,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>121.48</v>
+        <v>121.96</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30585,7 +30585,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>121.060563</v>
+        <v>120.812106</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-09-29
FX 33.58 · 99 updated · 0 MF carried · 5 manual
SEC NAV: matched 34/34 via SEC /v2/fund
Total ฿26,675,509 · P&L +16.61%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L124"/>
+  <dimension ref="B2:L125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25613,6 +25613,40 @@
         <v>33.46</v>
       </c>
       <c r="K124" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="72" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C125" t="n">
+        <v>26675509</v>
+      </c>
+      <c r="D125" t="n">
+        <v>22875046</v>
+      </c>
+      <c r="E125" t="n">
+        <v>3800463</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.1661</v>
+      </c>
+      <c r="G125" t="n">
+        <v>18697211</v>
+      </c>
+      <c r="H125" t="n">
+        <v>4975037</v>
+      </c>
+      <c r="I125" t="n">
+        <v>1594009</v>
+      </c>
+      <c r="J125" t="n">
+        <v>33.58</v>
+      </c>
+      <c r="K125" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26190,7 +26224,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26205,11 +26239,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.46</v>
+        <v>33.58</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-28</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26254,11 +26288,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.1859</v>
+        <v>26.2865</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-28</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27866,7 +27900,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27874,7 +27908,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.959999</v>
+        <v>21.969999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27898,7 +27932,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.052</v>
+        <v>1.056</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27906,7 +27940,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27914,7 +27948,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.052</v>
+        <v>1.056</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27946,7 +27980,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27954,7 +27988,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>783.580017</v>
+        <v>771.570007</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28026,7 +28060,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28034,7 +28068,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>208.190002</v>
+        <v>205.380005</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -28066,7 +28100,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28074,7 +28108,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -28098,23 +28132,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>192</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>193</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>192.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28138,7 +28172,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28146,7 +28180,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28154,7 +28188,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28186,7 +28220,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28303,7 +28337,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28343,7 +28377,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28375,7 +28409,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28383,7 +28417,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28391,7 +28425,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.299999</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28423,7 +28457,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28455,7 +28489,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.6</v>
+        <v>5.55</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28463,7 +28497,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28471,7 +28505,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.6</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28503,7 +28537,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28543,7 +28577,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28575,7 +28609,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.46</v>
+        <v>4.5</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28583,7 +28617,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28615,7 +28649,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.26</v>
+        <v>3.22</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28623,7 +28657,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28631,7 +28665,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.26</v>
+        <v>3.22</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28655,7 +28689,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28663,7 +28697,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28695,7 +28729,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.3</v>
+        <v>17.1</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28703,7 +28737,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28711,7 +28745,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.299999</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28735,7 +28769,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>123.11</v>
+        <v>124.01</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28743,7 +28777,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28775,7 +28809,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>235.47</v>
+        <v>231.01</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28783,7 +28817,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28815,23 +28849,23 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
+        <v>486.76</v>
+      </c>
+      <c r="F62" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G62" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H62" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
         <v>485</v>
-      </c>
-      <c r="F62" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G62" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H62" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I62" t="n">
-        <v>474.25</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28855,7 +28889,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>119.92</v>
+        <v>119.53</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28863,7 +28897,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28895,7 +28929,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>32.4</v>
+        <v>30.91</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28903,7 +28937,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28935,7 +28969,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>187.18</v>
+        <v>183.58</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28943,7 +28977,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -28975,7 +29009,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>173.46</v>
+        <v>176.33</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -28983,7 +29017,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29015,7 +29049,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>187.9</v>
+        <v>185.73</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29023,7 +29057,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29055,7 +29089,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>187.92</v>
+        <v>189.17</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29063,7 +29097,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29095,7 +29129,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1183.46</v>
+        <v>1184.78</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29103,7 +29137,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29135,7 +29169,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>78.69</v>
+        <v>77.97</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29143,7 +29177,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29175,7 +29209,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1367.43</v>
+        <v>1351.2</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29183,7 +29217,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29215,7 +29249,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>159.03</v>
+        <v>155.96</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29223,7 +29257,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29255,7 +29289,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>225.07</v>
+        <v>228.86</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29263,7 +29297,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29295,7 +29329,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.39</v>
+        <v>75.47</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29303,7 +29337,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29335,7 +29369,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>117.97</v>
+        <v>116.3</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29343,7 +29377,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29375,7 +29409,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>398.38</v>
+        <v>401.3</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29383,7 +29417,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29415,7 +29449,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>372.11</v>
+        <v>357.45</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29423,7 +29457,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29455,7 +29489,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>39.6</v>
+        <v>40.36</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29463,7 +29497,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29495,7 +29529,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>66.66</v>
+        <v>64.47</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29503,7 +29537,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29535,7 +29569,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>341.07</v>
+        <v>338.4</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29543,7 +29577,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29575,7 +29609,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>195.11</v>
+        <v>191.79</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29583,7 +29617,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29615,7 +29649,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>751.66</v>
+        <v>715.62</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29623,7 +29657,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29655,7 +29689,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>30.18</v>
+        <v>28.17</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29663,7 +29697,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29671,7 +29705,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>30.18</v>
+        <v>28.17</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29695,7 +29729,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>153.8</v>
+        <v>148.32</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29703,7 +29737,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29711,7 +29745,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>154.880053</v>
+        <v>153.075705</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29735,7 +29769,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>778.87</v>
+        <v>759</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29743,7 +29777,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29751,7 +29785,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>772.277725</v>
+        <v>776.9721919999999</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29775,7 +29809,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84074</v>
+        <v>83003</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29783,7 +29817,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29791,7 +29825,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84322.76727500001</v>
+        <v>83939.33669</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29815,7 +29849,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010307</v>
+        <v>0.009263</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29823,7 +29857,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29831,7 +29865,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009747</v>
+        <v>0.010196</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29855,7 +29889,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018565</v>
+        <v>0.017797</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29863,7 +29897,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29871,7 +29905,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017755</v>
+        <v>0.018415</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29895,7 +29929,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>121.96</v>
+        <v>117.62</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29903,7 +29937,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -29911,7 +29945,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>120.812106</v>
+        <v>121.397702</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29935,7 +29969,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.12</v>
+        <v>1.97</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29943,7 +29977,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -29951,7 +29985,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.092943</v>
+        <v>2.103229</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -29983,7 +30017,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30015,7 +30049,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035506</v>
+        <v>0.034583</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30023,7 +30057,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30031,7 +30065,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.036564</v>
+        <v>0.035428</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30055,7 +30089,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>7.525355</v>
+        <v>6.674059</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30063,7 +30097,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30071,7 +30105,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.534415</v>
+        <v>7.471092</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30095,7 +30129,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>42.4942</v>
+        <v>38.2812</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30103,7 +30137,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30111,7 +30145,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>38.856133</v>
+        <v>42.494846</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30135,7 +30169,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.167227</v>
+        <v>0.162933</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30143,7 +30177,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30151,7 +30185,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.156229</v>
+        <v>0.168201</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30175,7 +30209,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>26060.9902</v>
+        <v>25487.22</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30183,7 +30217,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30191,7 +30225,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25840.412676</v>
+        <v>26090.726219</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30215,7 +30249,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2813116.04</v>
+        <v>2787240.74</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30223,7 +30257,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30231,7 +30265,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2821439.793031</v>
+        <v>2818682.926056</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30255,7 +30289,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.243713</v>
+        <v>3.130227</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30263,7 +30297,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30271,7 +30305,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.214545</v>
+        <v>3.226912</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30295,7 +30329,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89462.00199999999</v>
+        <v>89656.5852</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30303,7 +30337,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30311,7 +30345,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90094.316062</v>
+        <v>89578.405182</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30335,7 +30369,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.683701</v>
+        <v>20.380071</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30343,7 +30377,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30351,7 +30385,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.4607</v>
+        <v>20.748141</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30375,7 +30409,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84074</v>
+        <v>83003</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30383,7 +30417,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30391,7 +30425,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84322.76727500001</v>
+        <v>83939.33669</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30415,7 +30449,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.32</v>
+        <v>23.2</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30423,7 +30457,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30431,7 +30465,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.851576</v>
+        <v>24.245012</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30529,7 +30563,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010307</v>
+        <v>0.009263</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30537,7 +30571,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30545,7 +30579,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009747</v>
+        <v>0.010196</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30569,7 +30603,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>121.96</v>
+        <v>117.62</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30577,7 +30611,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30585,7 +30619,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>120.812106</v>
+        <v>121.397702</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30617,7 +30651,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-29
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25623,16 +25623,16 @@
         <v>46294</v>
       </c>
       <c r="C125" t="n">
-        <v>26675509</v>
+        <v>26671906</v>
       </c>
       <c r="D125" t="n">
-        <v>22875046</v>
+        <v>22875235</v>
       </c>
       <c r="E125" t="n">
-        <v>3800463</v>
+        <v>3796671</v>
       </c>
       <c r="F125" t="n">
-        <v>0.1661</v>
+        <v>0.166</v>
       </c>
       <c r="G125" t="n">
         <v>18697211</v>
@@ -25641,7 +25641,7 @@
         <v>4975037</v>
       </c>
       <c r="I125" t="n">
-        <v>1594009</v>
+        <v>1590101</v>
       </c>
       <c r="J125" t="n">
         <v>33.58</v>
@@ -26288,7 +26288,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2865</v>
+        <v>26.2922</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>123.110001</v>
+        <v>124.010002</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28825,7 +28825,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>235.470001</v>
+        <v>231.009995</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28865,7 +28865,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>485</v>
+        <v>486.76001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28905,7 +28905,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>119.919998</v>
+        <v>119.529999</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28945,7 +28945,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>32.400002</v>
+        <v>30.91</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -28985,7 +28985,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>187.179993</v>
+        <v>183.580002</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -29025,7 +29025,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>173.460007</v>
+        <v>176.330002</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -29065,7 +29065,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>187.899994</v>
+        <v>185.729996</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29105,7 +29105,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>187.919998</v>
+        <v>189.169998</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29145,7 +29145,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1183.459961</v>
+        <v>1184.780029</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29185,7 +29185,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>78.69000200000001</v>
+        <v>77.970001</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29225,7 +29225,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1367.430054</v>
+        <v>1351.199951</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29265,7 +29265,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>159.029999</v>
+        <v>155.960007</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29305,7 +29305,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>225.070007</v>
+        <v>228.860001</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29345,7 +29345,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>77.389999</v>
+        <v>75.470001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29385,7 +29385,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>117.970001</v>
+        <v>116.300003</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29425,7 +29425,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>398.380005</v>
+        <v>401.299988</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29465,7 +29465,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>372.109985</v>
+        <v>357.450012</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29505,7 +29505,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>39.599998</v>
+        <v>40.360001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29545,7 +29545,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>66.660004</v>
+        <v>64.470001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29585,7 +29585,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>341.070007</v>
+        <v>338.399994</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29625,7 +29625,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>195.110001</v>
+        <v>191.789993</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29665,7 +29665,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>751.659973</v>
+        <v>715.619995</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29729,7 +29729,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>148.32</v>
+        <v>147.48</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29745,7 +29745,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>153.075705</v>
+        <v>153.770107</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29769,7 +29769,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>759</v>
+        <v>756.45</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29785,7 +29785,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>776.9721919999999</v>
+        <v>778.696702</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29809,7 +29809,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83003</v>
+        <v>82923</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29825,7 +29825,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83939.33669</v>
+        <v>84060.184905</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29849,7 +29849,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009263</v>
+        <v>0.009202999999999999</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29865,7 +29865,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010196</v>
+        <v>0.010317</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29889,7 +29889,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017797</v>
+        <v>0.01763</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29905,7 +29905,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018415</v>
+        <v>0.018578</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29929,7 +29929,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>117.62</v>
+        <v>117.03</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29945,7 +29945,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>121.397702</v>
+        <v>121.973698</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -29969,7 +29969,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -29985,7 +29985,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.103229</v>
+        <v>2.119578</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30049,7 +30049,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.034583</v>
+        <v>0.034527</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30065,7 +30065,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035428</v>
+        <v>0.035519</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30089,7 +30089,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.674059</v>
+        <v>6.577718</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30105,7 +30105,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.471092</v>
+        <v>7.532407</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30129,7 +30129,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>38.2812</v>
+        <v>37.9454</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30145,7 +30145,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>42.494846</v>
+        <v>42.905374</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30169,7 +30169,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.162933</v>
+        <v>0.161825</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30185,7 +30185,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.168201</v>
+        <v>0.167841</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30209,7 +30209,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25487.22</v>
+        <v>25401.591</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30225,7 +30225,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>26090.726219</v>
+        <v>26148.635248</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30249,7 +30249,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2787240.74</v>
+        <v>2784554.34</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30265,7 +30265,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2818682.926056</v>
+        <v>2822741.009108</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30289,7 +30289,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.130227</v>
+        <v>3.112631</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30305,7 +30305,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.226912</v>
+        <v>3.254249</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30329,7 +30329,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89656.5852</v>
+        <v>89400.7056</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30345,7 +30345,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89578.405182</v>
+        <v>89782.272371</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30369,7 +30369,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.380071</v>
+        <v>20.433867</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30385,7 +30385,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.748141</v>
+        <v>20.758237</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30409,7 +30409,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83003</v>
+        <v>82923</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30425,7 +30425,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83939.33669</v>
+        <v>84060.184905</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30449,7 +30449,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.2</v>
+        <v>23.13</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30465,7 +30465,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>24.245012</v>
+        <v>24.319578</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30563,7 +30563,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009263</v>
+        <v>0.009202999999999999</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30579,7 +30579,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010196</v>
+        <v>0.010317</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30603,7 +30603,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>117.62</v>
+        <v>117.03</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30619,7 +30619,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>121.397702</v>
+        <v>121.973698</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-09-30
FX 33.53 · 78 updated · 1 MF carried · 25 manual
SEC NAV: matched 33/34 via SEC /v2/fund; no NAV: ASP-EVOCHINA
Total ฿26,754,452 · P&L +16.99%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L125"/>
+  <dimension ref="B2:L126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25647,6 +25647,40 @@
         <v>33.58</v>
       </c>
       <c r="K125" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="72" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C126" t="n">
+        <v>26754452</v>
+      </c>
+      <c r="D126" t="n">
+        <v>22868910</v>
+      </c>
+      <c r="E126" t="n">
+        <v>3885542</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.1699</v>
+      </c>
+      <c r="G126" t="n">
+        <v>18808354</v>
+      </c>
+      <c r="H126" t="n">
+        <v>4959053</v>
+      </c>
+      <c r="I126" t="n">
+        <v>1589626</v>
+      </c>
+      <c r="J126" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="K126" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26224,7 +26258,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26239,11 +26273,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.58</v>
+        <v>33.53</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-29</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26288,11 +26322,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2922</v>
+        <v>26.2531</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-29</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26407,27 +26441,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.5084</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.342</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>21.1679</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26452,27 +26486,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7058</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7052</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.705</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26497,27 +26531,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3708</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3252</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.3983</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26587,27 +26621,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.790100000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.764799999999999</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.7212</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26632,27 +26666,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.3977</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.1793</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2248</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26677,27 +26711,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.4542</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.4245</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.3761</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26722,27 +26756,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>30.0092</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.8452</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.6109</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26767,27 +26801,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.6041</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.7421</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.6601</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26812,27 +26846,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.2903</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.3637</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.3337</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26857,27 +26891,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.2563</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.1799</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.4512</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26902,27 +26936,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>82.3947</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.71299999999999</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.50620000000001</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26947,27 +26981,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.8912</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.9916</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.9241</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26992,27 +27026,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.491</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.507</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.5022</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27037,27 +27071,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4522</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4506</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4501</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27082,27 +27116,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>42.117</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.9076</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.9156</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27127,27 +27161,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.1193</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.4409</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.6242</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27172,27 +27206,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9451</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>14.0265</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0312</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27217,27 +27251,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.2439</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.28</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.2785</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27262,27 +27296,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9674</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.8488</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.9426</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27307,27 +27341,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.8056</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.818300000000001</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.797499999999999</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27352,27 +27386,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7566</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7694</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7415</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27397,27 +27431,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.2761</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.3119</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.2831</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27442,27 +27476,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.1891</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.8739</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.7148</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27487,27 +27521,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>25.1552</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>24.5455</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.9323</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27532,27 +27566,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>38.0854</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>37.3329</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.6929</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27577,27 +27611,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.2913</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.3333</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.298</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27622,27 +27656,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7234</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7228</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7226</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27667,27 +27701,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.1201</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1493</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1539</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27712,27 +27746,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2422</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2412</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2408</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27757,27 +27791,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>28.2312</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.2031</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.0982</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -27802,27 +27836,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0153</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0603</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0415</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27847,27 +27881,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.5537</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.6325</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.5898</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27892,7 +27926,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>21.96</v>
+        <v>21.97</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27900,7 +27934,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27908,7 +27942,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.969999</v>
+        <v>21.889999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27940,7 +27974,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27948,7 +27982,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.056</v>
+        <v>1.051</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -27972,7 +28006,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>783.58</v>
+        <v>771.5700000000001</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -27980,7 +28014,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -27988,7 +28022,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>771.570007</v>
+        <v>774.6099850000001</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28052,7 +28086,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>208.19</v>
+        <v>205.38</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -28060,7 +28094,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28068,7 +28102,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>205.380005</v>
+        <v>206.169998</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -28100,7 +28134,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28132,23 +28166,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>189</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>192</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>193</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28172,7 +28206,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28180,7 +28214,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28188,7 +28222,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28212,7 +28246,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28220,7 +28254,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28329,23 +28363,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>60</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>60.75</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>60.5</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28369,7 +28403,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28377,7 +28411,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28385,7 +28419,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.9</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28409,7 +28443,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28417,7 +28451,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28425,7 +28459,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.4</v>
+        <v>16.200001</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28449,7 +28483,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28457,7 +28491,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28465,7 +28499,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28489,7 +28523,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.55</v>
+        <v>5.45</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28497,7 +28531,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28505,7 +28539,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.55</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28529,7 +28563,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28537,7 +28571,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28545,7 +28579,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.299999</v>
+        <v>22.4</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28569,7 +28603,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.4</v>
+        <v>3.38</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28577,7 +28611,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28585,7 +28619,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.4</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28609,7 +28643,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.5</v>
+        <v>4.46</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28617,7 +28651,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28649,7 +28683,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.22</v>
+        <v>3.2</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28657,7 +28691,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28665,7 +28699,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.22</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28689,7 +28723,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28697,7 +28731,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28729,7 +28763,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>17.1</v>
+        <v>16.9</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28737,7 +28771,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28745,7 +28779,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>17.1</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28769,7 +28803,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>124.01</v>
+        <v>128.69</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28777,7 +28811,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28809,7 +28843,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>231.01</v>
+        <v>233.17</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28817,7 +28851,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28849,7 +28883,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>486.76</v>
+        <v>512.01</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28857,7 +28891,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28889,7 +28923,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>119.53</v>
+        <v>120.8</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28897,7 +28931,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28929,7 +28963,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>30.91</v>
+        <v>31.83</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28937,7 +28971,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -28969,7 +29003,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>183.58</v>
+        <v>187.1</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -28977,7 +29011,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29009,7 +29043,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>176.33</v>
+        <v>175.96</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -29017,7 +29051,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29049,7 +29083,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>185.73</v>
+        <v>185.85</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29057,7 +29091,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29089,7 +29123,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>189.17</v>
+        <v>196.53</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29097,7 +29131,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29129,7 +29163,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1184.78</v>
+        <v>1184.63</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29137,7 +29171,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29169,7 +29203,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>77.97</v>
+        <v>78.78</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29177,7 +29211,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29209,7 +29243,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1351.2</v>
+        <v>1355.99</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29217,7 +29251,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29249,7 +29283,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>155.96</v>
+        <v>155.64</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29257,7 +29291,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29289,7 +29323,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>228.86</v>
+        <v>227.21</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29297,7 +29331,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29329,7 +29363,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>75.47</v>
+        <v>76.16</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29337,7 +29371,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29369,7 +29403,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>116.3</v>
+        <v>116.75</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29377,7 +29411,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29409,7 +29443,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>401.3</v>
+        <v>403.02</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29417,7 +29451,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29449,7 +29483,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>357.45</v>
+        <v>352.84</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29457,7 +29491,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29489,7 +29523,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>40.36</v>
+        <v>41.22</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29497,7 +29531,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29529,7 +29563,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>64.47</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29537,7 +29571,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29569,7 +29603,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>338.4</v>
+        <v>329.4</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29577,7 +29611,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29609,7 +29643,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>191.79</v>
+        <v>190.02</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29617,7 +29651,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29649,7 +29683,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>715.62</v>
+        <v>738.79</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29657,7 +29691,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29689,7 +29723,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>28.17</v>
+        <v>29.74</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29697,7 +29731,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29705,7 +29739,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>28.17</v>
+        <v>29.74</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29741,7 +29775,7 @@
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -29781,7 +29815,7 @@
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -29821,7 +29855,7 @@
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -29861,7 +29895,7 @@
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -29901,7 +29935,7 @@
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -29941,7 +29975,7 @@
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -29981,7 +30015,7 @@
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -30017,7 +30051,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30061,7 +30095,7 @@
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -30101,7 +30135,7 @@
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -30141,7 +30175,7 @@
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -30181,7 +30215,7 @@
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -30221,7 +30255,7 @@
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I96" t="n">
@@ -30261,7 +30295,7 @@
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I97" t="n">
@@ -30301,7 +30335,7 @@
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I98" t="n">
@@ -30341,7 +30375,7 @@
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -30381,7 +30415,7 @@
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -30421,7 +30455,7 @@
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -30461,7 +30495,7 @@
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I102" t="n">
@@ -30575,7 +30609,7 @@
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -30615,7 +30649,7 @@
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I106" t="n">
@@ -30651,7 +30685,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30683,27 +30717,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.6933</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.8045</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46288</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.9698</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-09-30
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25657,28 +25657,28 @@
         <v>46295</v>
       </c>
       <c r="C126" t="n">
-        <v>26754452</v>
+        <v>26772756</v>
       </c>
       <c r="D126" t="n">
-        <v>22868910</v>
+        <v>22873765</v>
       </c>
       <c r="E126" t="n">
-        <v>3885542</v>
+        <v>3898991</v>
       </c>
       <c r="F126" t="n">
-        <v>0.1699</v>
+        <v>0.1705</v>
       </c>
       <c r="G126" t="n">
-        <v>18808354</v>
+        <v>18807241</v>
       </c>
       <c r="H126" t="n">
-        <v>4959053</v>
+        <v>4963921</v>
       </c>
       <c r="I126" t="n">
-        <v>1589626</v>
+        <v>1604458</v>
       </c>
       <c r="J126" t="n">
-        <v>33.53</v>
+        <v>33.58</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -26273,7 +26273,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.53</v>
+        <v>33.58</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -26322,7 +26322,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2531</v>
+        <v>26.2478</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -26576,27 +26576,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.5023</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.5817</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.6309</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -28819,7 +28819,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>124.010002</v>
+        <v>128.690002</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28859,7 +28859,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>231.009995</v>
+        <v>233.169998</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28899,7 +28899,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>486.76001</v>
+        <v>512.01001</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28939,7 +28939,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>119.529999</v>
+        <v>120.800003</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -28979,7 +28979,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>30.91</v>
+        <v>31.83</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -29019,7 +29019,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>183.580002</v>
+        <v>187.100006</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -29059,7 +29059,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>176.330002</v>
+        <v>175.960007</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -29099,7 +29099,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>185.729996</v>
+        <v>185.850006</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29139,7 +29139,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>189.169998</v>
+        <v>196.529999</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29179,7 +29179,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1184.780029</v>
+        <v>1184.630005</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29219,7 +29219,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>77.970001</v>
+        <v>78.779999</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29259,7 +29259,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1351.199951</v>
+        <v>1355.98999</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29299,7 +29299,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>155.960007</v>
+        <v>155.639999</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29339,7 +29339,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>228.860001</v>
+        <v>227.210007</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29379,7 +29379,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>75.470001</v>
+        <v>76.160004</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29459,7 +29459,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>401.299988</v>
+        <v>403.019989</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29499,7 +29499,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>357.450012</v>
+        <v>352.839996</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29539,7 +29539,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>40.360001</v>
+        <v>41.220001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29579,7 +29579,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>64.470001</v>
+        <v>64.790001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29619,7 +29619,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>338.399994</v>
+        <v>329.399994</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29659,7 +29659,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>191.789993</v>
+        <v>190.020004</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29699,7 +29699,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>715.619995</v>
+        <v>738.789978</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29763,7 +29763,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>147.48</v>
+        <v>161.33</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29771,15 +29771,15 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>153.770107</v>
+        <v>147.48389</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29803,7 +29803,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>756.45</v>
+        <v>759.1900000000001</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29811,15 +29811,15 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>778.696702</v>
+        <v>756.545927</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29843,7 +29843,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>82923</v>
+        <v>83360</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29851,15 +29851,15 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84060.184905</v>
+        <v>82926.635348</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29883,7 +29883,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009202999999999999</v>
+        <v>0.010097</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29891,15 +29891,15 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010317</v>
+        <v>0.009113</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29923,7 +29923,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01763</v>
+        <v>0.017888</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29931,15 +29931,15 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018578</v>
+        <v>0.017651</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29963,7 +29963,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>117.03</v>
+        <v>119.42</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -29971,15 +29971,15 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I89" t="n">
-        <v>121.973698</v>
+        <v>116.887138</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30003,7 +30003,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>1.96</v>
+        <v>2.07</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30011,15 +30011,15 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.119578</v>
+        <v>1.953803</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30083,7 +30083,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.034527</v>
+        <v>0.034964</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30091,15 +30091,15 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035519</v>
+        <v>0.034433</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30123,7 +30123,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.577718</v>
+        <v>6.867379</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30131,15 +30131,15 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I93" t="n">
-        <v>7.532407</v>
+        <v>6.530205</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30163,7 +30163,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>37.9454</v>
+        <v>38.9528</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30171,15 +30171,15 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I94" t="n">
-        <v>42.905374</v>
+        <v>37.579493</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30203,7 +30203,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.161825</v>
+        <v>0.170098</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30211,15 +30211,15 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.167841</v>
+        <v>0.162199</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30243,7 +30243,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25401.591</v>
+        <v>25493.6002</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30251,15 +30251,15 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I96" t="n">
-        <v>26148.635248</v>
+        <v>25404.812224</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30283,7 +30283,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2784554.34</v>
+        <v>2799228.8</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30291,15 +30291,15 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2822741.009108</v>
+        <v>2784676.415002</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30323,7 +30323,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.112631</v>
+        <v>3.15652</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30331,15 +30331,15 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.254249</v>
+        <v>3.109963</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30363,7 +30363,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89400.7056</v>
+        <v>89647.1828</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30371,15 +30371,15 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89782.272371</v>
+        <v>89402.23489199999</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30403,7 +30403,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.433867</v>
+        <v>20.389709</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30411,15 +30411,15 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.758237</v>
+        <v>20.37769</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30443,7 +30443,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>82923</v>
+        <v>83360</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30451,15 +30451,15 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84060.184905</v>
+        <v>82926.635348</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30483,7 +30483,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.13</v>
+        <v>26.36</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30491,15 +30491,15 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>24.319578</v>
+        <v>23.082113</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30597,7 +30597,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009202999999999999</v>
+        <v>0.010097</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30605,15 +30605,15 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010317</v>
+        <v>0.009113</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30637,7 +30637,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>117.03</v>
+        <v>119.42</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30645,15 +30645,15 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I106" t="n">
-        <v>121.973698</v>
+        <v>116.887138</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-01
FX 33.6 · 77 updated · 2 MF carried · 25 manual
SEC NAV: matched 32/34 via SEC /v2/fund; no NAV: ASP-EVOCHINA, BFLRMF
Total ฿26,591,009 · P&L +16.23%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L126"/>
+  <dimension ref="B2:L127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25681,6 +25681,40 @@
         <v>33.58</v>
       </c>
       <c r="K126" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="72" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C127" t="n">
+        <v>26591009</v>
+      </c>
+      <c r="D127" t="n">
+        <v>22877177</v>
+      </c>
+      <c r="E127" t="n">
+        <v>3713831</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.1623</v>
+      </c>
+      <c r="G127" t="n">
+        <v>18658234</v>
+      </c>
+      <c r="H127" t="n">
+        <v>4928393</v>
+      </c>
+      <c r="I127" t="n">
+        <v>1604651</v>
+      </c>
+      <c r="J127" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="K127" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26258,7 +26292,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26273,11 +26307,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.58</v>
+        <v>33.6</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-30</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -26322,11 +26356,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2478</v>
+        <v>26.2901</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-09-30</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -26441,27 +26475,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>20.7113</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.5084</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>21.342</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26486,27 +26520,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.706</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7058</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7052</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26531,27 +26565,27 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
+        <v>7.3848</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>7.3708</v>
       </c>
-      <c r="F7" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G7" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>7.3252</v>
-      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26621,27 +26655,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.7706</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.790100000000001</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.764799999999999</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26666,27 +26700,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.3384</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.3977</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.1793</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26711,27 +26745,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.5855</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.4542</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.4245</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26756,27 +26790,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>30.3077</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>30.0092</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>29.8452</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26801,27 +26835,27 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
+        <v>36.3408</v>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>36.6041</v>
       </c>
-      <c r="F13" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G13" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H13" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>36.7421</v>
-      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26846,27 +26880,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>26.1286</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.2903</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.3637</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26891,27 +26925,27 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
+        <v>16.2768</v>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>16.2563</v>
       </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G15" s="28" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H15" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>16.1799</v>
-      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26936,27 +26970,27 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
+        <v>81.7975</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>82.3947</v>
       </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G16" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H16" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>82.71299999999999</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27026,27 +27060,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4844</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.491</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.507</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27071,27 +27105,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4526</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4522</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4506</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27116,27 +27150,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.8107</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>42.117</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.9076</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27161,27 +27195,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.119</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.1193</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.4409</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27206,27 +27240,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9984</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9451</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>14.0265</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27251,27 +27285,27 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
+        <v>13.1412</v>
+      </c>
+      <c r="F23" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G23" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>13.2439</v>
       </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>13.28</v>
-      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27296,27 +27330,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9325</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9674</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.8488</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27341,27 +27375,27 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
+        <v>9.7807</v>
+      </c>
+      <c r="F25" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>9.8056</v>
       </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G25" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H25" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>9.818300000000001</v>
-      </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27386,27 +27420,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7199</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7566</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7694</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27431,27 +27465,27 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
+        <v>18.1354</v>
+      </c>
+      <c r="F27" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>18.2761</v>
       </c>
-      <c r="F27" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H27" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>18.3119</v>
-      </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27476,27 +27510,27 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
+        <v>18.196</v>
+      </c>
+      <c r="F28" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>18.1891</v>
       </c>
-      <c r="F28" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G28" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H28" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>18.8739</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27521,27 +27555,27 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
+        <v>24.6967</v>
+      </c>
+      <c r="F29" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>25.1552</v>
       </c>
-      <c r="F29" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G29" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H29" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>24.5455</v>
-      </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27566,27 +27600,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>37.3627</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>38.0854</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.3329</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27611,27 +27645,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.2197</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.2913</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.3333</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27656,27 +27690,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7236</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7234</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7228</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27701,27 +27735,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>13.0209</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.1201</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1493</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27746,27 +27780,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2426</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2422</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2412</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27791,27 +27825,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.3289</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>28.2312</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.2031</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27836,27 +27870,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>9.9907</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0153</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0603</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27881,27 +27915,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.3975</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.5537</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.6325</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27926,7 +27960,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>21.97</v>
+        <v>21.89</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27934,7 +27968,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27942,7 +27976,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.889999</v>
+        <v>21.780001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -27966,7 +28000,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.056</v>
+        <v>1.051</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -27974,7 +28008,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -27982,7 +28016,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.051</v>
+        <v>1.052</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -28006,7 +28040,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>771.5700000000001</v>
+        <v>774.61</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -28014,7 +28048,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28022,7 +28056,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>774.6099850000001</v>
+        <v>780.169983</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28086,7 +28120,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>205.38</v>
+        <v>206.17</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -28094,7 +28128,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28102,7 +28136,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>206.169998</v>
+        <v>206.539993</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -28126,7 +28160,7 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
-        <v>14.6</v>
+        <v>14.5</v>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
@@ -28134,7 +28168,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28166,23 +28200,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>184.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>189</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>192</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28206,7 +28240,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28214,7 +28248,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28222,7 +28256,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28254,7 +28288,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28363,23 +28397,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>59</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>60</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>60.75</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28403,7 +28437,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28411,7 +28445,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28419,7 +28453,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28443,7 +28477,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>16.2</v>
+        <v>15.8</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28451,7 +28485,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28459,7 +28493,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>16.200001</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28483,7 +28517,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28491,7 +28525,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28531,7 +28565,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28563,7 +28597,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>22.4</v>
+        <v>21.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28571,7 +28605,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28579,7 +28613,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22.4</v>
+        <v>21.799999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28611,7 +28645,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28651,7 +28685,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28683,7 +28717,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.2</v>
+        <v>3.08</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28691,7 +28725,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28699,7 +28733,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.2</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28723,7 +28757,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28731,7 +28765,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28739,7 +28773,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28763,7 +28797,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.9</v>
+        <v>16.7</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28771,7 +28805,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28779,7 +28813,7 @@
         </is>
       </c>
       <c r="I59" t="n">
-        <v>16.9</v>
+        <v>16.700001</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="58">
@@ -28803,7 +28837,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>128.69</v>
+        <v>131.18</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28811,7 +28845,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28843,7 +28877,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>233.17</v>
+        <v>239.94</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28851,7 +28885,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28883,7 +28917,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>512.01</v>
+        <v>511.38</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28891,7 +28925,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28923,7 +28957,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>120.8</v>
+        <v>119.97</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28931,7 +28965,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28963,7 +28997,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>31.83</v>
+        <v>32.99</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -28971,7 +29005,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -29003,7 +29037,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>187.1</v>
+        <v>182.78</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -29011,7 +29045,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29043,7 +29077,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>175.96</v>
+        <v>178.76</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -29051,7 +29085,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29083,7 +29117,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>185.85</v>
+        <v>186.54</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29091,7 +29125,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29123,7 +29157,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>196.53</v>
+        <v>194.93</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29131,7 +29165,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29163,7 +29197,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1184.63</v>
+        <v>1157.08</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29171,7 +29205,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29203,7 +29237,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>78.78</v>
+        <v>77.77</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29211,7 +29245,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29243,7 +29277,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1355.99</v>
+        <v>1347.22</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29251,7 +29285,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29283,7 +29317,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>155.64</v>
+        <v>156.32</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29291,7 +29325,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29323,7 +29357,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>227.21</v>
+        <v>228.38</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29331,7 +29365,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29363,7 +29397,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>76.16</v>
+        <v>77.04000000000001</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29371,7 +29405,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29403,23 +29437,23 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
+        <v>114.48</v>
+      </c>
+      <c r="F75" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G75" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H75" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
         <v>116.75</v>
-      </c>
-      <c r="F75" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G75" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H75" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I75" t="n">
-        <v>116.300003</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29443,7 +29477,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>403.02</v>
+        <v>400.91</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29451,7 +29485,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29483,7 +29517,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>352.84</v>
+        <v>354.81</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29491,7 +29525,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29523,7 +29557,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>41.22</v>
+        <v>41.95</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29531,7 +29565,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29563,7 +29597,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>64.79000000000001</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29571,7 +29605,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29603,7 +29637,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>329.4</v>
+        <v>333.02</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29611,7 +29645,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29643,7 +29677,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>190.02</v>
+        <v>186.41</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29651,7 +29685,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29683,7 +29717,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>738.79</v>
+        <v>725.1799999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29691,7 +29725,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29723,7 +29757,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>29.74</v>
+        <v>29.62</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29731,7 +29765,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29739,7 +29773,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>29.74</v>
+        <v>29.620001</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29775,7 +29809,7 @@
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I84" t="n">
@@ -29815,7 +29849,7 @@
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I85" t="n">
@@ -29855,7 +29889,7 @@
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -29895,7 +29929,7 @@
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I87" t="n">
@@ -29935,7 +29969,7 @@
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I88" t="n">
@@ -29975,7 +30009,7 @@
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -30015,7 +30049,7 @@
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -30051,7 +30085,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30095,7 +30129,7 @@
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -30135,7 +30169,7 @@
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I93" t="n">
@@ -30175,7 +30209,7 @@
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -30215,7 +30249,7 @@
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I95" t="n">
@@ -30255,7 +30289,7 @@
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I96" t="n">
@@ -30295,7 +30329,7 @@
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I97" t="n">
@@ -30335,7 +30369,7 @@
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I98" t="n">
@@ -30375,7 +30409,7 @@
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I99" t="n">
@@ -30415,7 +30449,7 @@
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I100" t="n">
@@ -30455,7 +30489,7 @@
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I101" t="n">
@@ -30495,7 +30529,7 @@
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I102" t="n">
@@ -30609,7 +30643,7 @@
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I105" t="n">
@@ -30649,7 +30683,7 @@
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="I106" t="n">
@@ -30685,7 +30719,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30717,27 +30751,27 @@
         </is>
       </c>
       <c r="E108" t="n">
+        <v>24.9637</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G108" s="47" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
         <v>24.6933</v>
       </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G108" s="47" t="n">
-        <v>46289</v>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I108" t="n">
-        <v>24.8045</v>
-      </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-10-01
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25691,28 +25691,28 @@
         <v>46296</v>
       </c>
       <c r="C127" t="n">
-        <v>26591009</v>
+        <v>26598603</v>
       </c>
       <c r="D127" t="n">
-        <v>22877177</v>
+        <v>22880851</v>
       </c>
       <c r="E127" t="n">
-        <v>3713831</v>
+        <v>3717752</v>
       </c>
       <c r="F127" t="n">
-        <v>0.1623</v>
+        <v>0.1625</v>
       </c>
       <c r="G127" t="n">
-        <v>18658234</v>
+        <v>18651061</v>
       </c>
       <c r="H127" t="n">
-        <v>4928393</v>
+        <v>4931299</v>
       </c>
       <c r="I127" t="n">
-        <v>1604651</v>
+        <v>1615457</v>
       </c>
       <c r="J127" t="n">
-        <v>33.6</v>
+        <v>33.63</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -26307,7 +26307,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.6</v>
+        <v>33.63</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -26356,7 +26356,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2901</v>
+        <v>26.3099</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -26610,27 +26610,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.408799999999999</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.5023</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.5817</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27015,27 +27015,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>54.5252</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>54.8912</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>54.9916</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -28853,7 +28853,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>128.690002</v>
+        <v>131.179993</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28893,7 +28893,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>233.169998</v>
+        <v>239.940002</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28933,7 +28933,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>512.01001</v>
+        <v>511.380005</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28973,7 +28973,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>120.800003</v>
+        <v>119.970001</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -29013,7 +29013,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>31.83</v>
+        <v>32.990002</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -29053,7 +29053,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>187.100006</v>
+        <v>182.779999</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -29093,7 +29093,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>175.960007</v>
+        <v>178.759995</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -29133,7 +29133,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>185.850006</v>
+        <v>186.539993</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29173,7 +29173,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>196.529999</v>
+        <v>194.929993</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29213,7 +29213,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1184.630005</v>
+        <v>1157.079956</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29253,7 +29253,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>78.779999</v>
+        <v>77.769997</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29293,7 +29293,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1355.98999</v>
+        <v>1347.219971</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29333,7 +29333,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>155.639999</v>
+        <v>156.320007</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29373,7 +29373,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>227.210007</v>
+        <v>228.380005</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29413,7 +29413,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>76.160004</v>
+        <v>77.040001</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29453,7 +29453,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>116.75</v>
+        <v>114.480003</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29493,7 +29493,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>403.019989</v>
+        <v>400.910004</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29533,7 +29533,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>352.839996</v>
+        <v>354.809998</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29573,7 +29573,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>41.220001</v>
+        <v>41.950001</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29613,7 +29613,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>64.790001</v>
+        <v>64.260002</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29653,7 +29653,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>329.399994</v>
+        <v>333.019989</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29693,7 +29693,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>190.020004</v>
+        <v>186.410004</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29733,7 +29733,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>738.789978</v>
+        <v>725.179993</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29797,7 +29797,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>161.33</v>
+        <v>161.28</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29805,15 +29805,15 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>147.48389</v>
+        <v>161.517523</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29837,7 +29837,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>759.1900000000001</v>
+        <v>768.84</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29845,15 +29845,15 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>756.545927</v>
+        <v>759.08778</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29877,7 +29877,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83360</v>
+        <v>83462</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29885,15 +29885,15 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I86" t="n">
-        <v>82926.635348</v>
+        <v>83329.66761600001</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29917,7 +29917,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.010097</v>
+        <v>0.00966</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29925,15 +29925,15 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009113</v>
+        <v>0.010065</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29957,7 +29957,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017888</v>
+        <v>0.019326</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29965,15 +29965,15 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017651</v>
+        <v>0.017887</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29997,7 +29997,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>119.42</v>
+        <v>118.01</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30005,15 +30005,15 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I89" t="n">
-        <v>116.887138</v>
+        <v>119.12118</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30037,7 +30037,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.07</v>
+        <v>2.06</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30045,15 +30045,15 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I90" t="n">
-        <v>1.953803</v>
+        <v>2.07229</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30117,23 +30117,23 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
+        <v>0.035332</v>
+      </c>
+      <c r="F92" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G92" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H92" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
         <v>0.034964</v>
-      </c>
-      <c r="F92" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G92" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H92" s="34" t="inlineStr">
-        <is>
-          <t>MANUAL</t>
-        </is>
-      </c>
-      <c r="I92" t="n">
-        <v>0.034433</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30157,7 +30157,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.867379</v>
+        <v>6.843032</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30165,15 +30165,15 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.530205</v>
+        <v>6.875088</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30197,7 +30197,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>38.9528</v>
+        <v>39.6834</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30205,15 +30205,15 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I94" t="n">
-        <v>37.579493</v>
+        <v>39.054854</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30237,7 +30237,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.170098</v>
+        <v>0.181365</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30245,15 +30245,15 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.162199</v>
+        <v>0.170189</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30277,7 +30277,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25493.6002</v>
+        <v>25856.0892</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30285,15 +30285,15 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25404.812224</v>
+        <v>25528.122027</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30317,7 +30317,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2799228.8</v>
+        <v>2806827.06</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30325,15 +30325,15 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2784676.415002</v>
+        <v>2802376.721932</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30357,7 +30357,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.15652</v>
+        <v>3.185837</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30365,15 +30365,15 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.109963</v>
+        <v>3.153116</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30397,7 +30397,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89647.1828</v>
+        <v>90367.8456</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30405,15 +30405,15 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89402.23489199999</v>
+        <v>89733.06937700001</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30437,7 +30437,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.389709</v>
+        <v>20.499301</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30445,15 +30445,15 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.37769</v>
+        <v>20.369568</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30477,7 +30477,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83360</v>
+        <v>83462</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30485,15 +30485,15 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>82926.635348</v>
+        <v>83329.66761600001</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30517,7 +30517,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>26.36</v>
+        <v>24.58</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30525,15 +30525,15 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.082113</v>
+        <v>26.334778</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30631,7 +30631,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.010097</v>
+        <v>0.00966</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30639,15 +30639,15 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009113</v>
+        <v>0.010065</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30671,7 +30671,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>119.42</v>
+        <v>118.01</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30679,15 +30679,15 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="I106" t="n">
-        <v>116.887138</v>
+        <v>119.12118</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-02
FX 33.66 · 91 updated · 8 MF carried · 5 manual
SEC NAV: matched 26/34 via SEC /v2/fund; no NAV: ASP-JHC, ASP-SME-A, ES-US500RMF, K-CHX, K-TNZ-ThaiESG, KF-ASET50-L, SCBGOLDH, UTSB-THAIESG
Total ฿26,590,978 · P&L +16.20%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L127"/>
+  <dimension ref="B2:L128"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25715,6 +25715,40 @@
         <v>33.63</v>
       </c>
       <c r="K127" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" s="72" t="n">
+        <v>46297</v>
+      </c>
+      <c r="C128" t="n">
+        <v>26590978</v>
+      </c>
+      <c r="D128" t="n">
+        <v>22883121</v>
+      </c>
+      <c r="E128" t="n">
+        <v>3707857</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="G128" t="n">
+        <v>18614282</v>
+      </c>
+      <c r="H128" t="n">
+        <v>4939736</v>
+      </c>
+      <c r="I128" t="n">
+        <v>1634280</v>
+      </c>
+      <c r="J128" t="n">
+        <v>33.66</v>
+      </c>
+      <c r="K128" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26292,7 +26326,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26307,11 +26341,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.63</v>
+        <v>33.66</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-01</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -26356,11 +26390,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.3099</v>
+        <v>26.2873</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-01</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -26475,7 +26509,7 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
-        <v>20.7113</v>
+        <v>21.1169</v>
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
@@ -26483,7 +26517,7 @@
         </is>
       </c>
       <c r="G5" s="28" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="H5" s="34" t="inlineStr">
         <is>
@@ -26520,7 +26554,7 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>10.706</v>
+        <v>10.7061</v>
       </c>
       <c r="F6" s="34" t="inlineStr">
         <is>
@@ -26528,7 +26562,7 @@
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
@@ -26565,7 +26599,7 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
-        <v>7.3848</v>
+        <v>7.3252</v>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
@@ -26573,7 +26607,7 @@
         </is>
       </c>
       <c r="G7" s="28" t="n">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
@@ -26581,11 +26615,11 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7.3708</v>
+        <v>7.3983</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -26655,7 +26689,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.7706</v>
+        <v>9.724399999999999</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26663,7 +26697,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26790,27 +26824,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.6694</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>30.3077</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>30.0092</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26851,11 +26885,11 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>36.6041</v>
+        <v>36.7421</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -26880,27 +26914,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.652</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>26.1286</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.2903</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27015,7 +27049,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>54.5252</v>
+        <v>54.8912</v>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -27023,7 +27057,7 @@
         </is>
       </c>
       <c r="G17" s="28" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
@@ -27031,11 +27065,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.8912</v>
+        <v>54.9916</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27060,27 +27094,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.503</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.4844</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.491</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27105,27 +27139,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4534</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4526</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4522</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27240,27 +27274,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.9416</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9984</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.9451</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27330,27 +27364,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9228</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9325</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.9674</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27420,27 +27454,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.6983</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7199</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7566</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27555,7 +27589,7 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>24.6967</v>
+        <v>24.5455</v>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
@@ -27563,7 +27597,7 @@
         </is>
       </c>
       <c r="G29" s="28" t="n">
-        <v>46293</v>
+        <v>46289</v>
       </c>
       <c r="H29" s="34" t="inlineStr">
         <is>
@@ -27600,27 +27634,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>38.3251</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>37.3627</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>38.0854</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27645,27 +27679,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9176</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>13.2197</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.2913</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27690,27 +27724,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7238</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7236</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7234</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27735,27 +27769,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.7601</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>13.0209</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.1201</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27825,27 +27859,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.6783</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.3289</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46293</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>28.2312</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27915,27 +27949,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.8402</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>23.3975</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.5537</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27960,7 +27994,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>21.89</v>
+        <v>21.78</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -27968,7 +28002,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -27976,7 +28010,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.780001</v>
+        <v>21.35</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -28000,7 +28034,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.051</v>
+        <v>1.052</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -28008,7 +28042,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -28016,7 +28050,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.052</v>
+        <v>1.044</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -28040,7 +28074,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>774.61</v>
+        <v>780.17</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -28048,7 +28082,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28056,7 +28090,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>780.169983</v>
+        <v>779.789978</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28120,7 +28154,7 @@
         </is>
       </c>
       <c r="E42" s="33" t="n">
-        <v>206.17</v>
+        <v>206.54</v>
       </c>
       <c r="F42" s="34" t="inlineStr">
         <is>
@@ -28128,7 +28162,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28160,23 +28194,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.5</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.6</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -28208,7 +28242,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -28240,7 +28274,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28248,7 +28282,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28256,7 +28290,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28280,7 +28314,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28288,7 +28322,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28296,7 +28330,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -28405,7 +28439,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28445,7 +28479,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28477,7 +28511,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28485,7 +28519,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28493,7 +28527,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.8</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28517,7 +28551,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15</v>
+        <v>14.8</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28525,7 +28559,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28533,7 +28567,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28557,7 +28591,7 @@
         </is>
       </c>
       <c r="E53" s="33" t="n">
-        <v>5.45</v>
+        <v>5.55</v>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
@@ -28565,7 +28599,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28573,7 +28607,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>5.45</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="58">
@@ -28597,7 +28631,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.8</v>
+        <v>21.4</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28605,7 +28639,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28613,7 +28647,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.799999</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28637,7 +28671,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.38</v>
+        <v>3.36</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28645,7 +28679,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28653,7 +28687,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.38</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28677,7 +28711,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.46</v>
+        <v>4.42</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28685,7 +28719,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28693,7 +28727,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.46</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28717,7 +28751,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.08</v>
+        <v>3.12</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28725,7 +28759,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28733,7 +28767,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.08</v>
+        <v>3.12</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28757,7 +28791,7 @@
         </is>
       </c>
       <c r="E58" s="33" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
       <c r="F58" s="34" t="inlineStr">
         <is>
@@ -28765,7 +28799,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28773,7 +28807,7 @@
         </is>
       </c>
       <c r="I58" t="n">
-        <v>12.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="58">
@@ -28805,7 +28839,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28837,7 +28871,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>131.18</v>
+        <v>136.71</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28845,7 +28879,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28877,7 +28911,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>239.94</v>
+        <v>241.28</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28885,7 +28919,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28917,7 +28951,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>511.38</v>
+        <v>529.3</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28925,7 +28959,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28957,7 +28991,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>119.97</v>
+        <v>120.17</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28965,7 +28999,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -28997,7 +29031,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>32.99</v>
+        <v>32.82</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -29005,7 +29039,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -29037,7 +29071,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>182.78</v>
+        <v>186.11</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -29045,7 +29079,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29077,7 +29111,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>178.76</v>
+        <v>178.72</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -29085,7 +29119,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29117,7 +29151,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>186.54</v>
+        <v>192.8</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29125,7 +29159,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29157,7 +29191,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>194.93</v>
+        <v>200.33</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29165,7 +29199,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29197,7 +29231,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1157.08</v>
+        <v>1149.85</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29205,7 +29239,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29237,7 +29271,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>77.77</v>
+        <v>78.5</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29245,7 +29279,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29277,7 +29311,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1347.22</v>
+        <v>1360.97</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29285,7 +29319,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29317,7 +29351,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>156.32</v>
+        <v>161.33</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29325,7 +29359,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29357,7 +29391,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>228.38</v>
+        <v>230.86</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29365,7 +29399,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29397,7 +29431,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.04000000000001</v>
+        <v>77.39</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29405,7 +29439,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29437,7 +29471,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>114.48</v>
+        <v>112.21</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29445,7 +29479,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29477,7 +29511,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>400.91</v>
+        <v>415.79</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29485,7 +29519,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29517,7 +29551,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>354.81</v>
+        <v>354.11</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29525,7 +29559,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29557,7 +29591,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>41.95</v>
+        <v>41.74</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29565,7 +29599,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29597,7 +29631,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>64.26000000000001</v>
+        <v>62.95</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29605,7 +29639,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29637,7 +29671,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>333.02</v>
+        <v>330.32</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29645,7 +29679,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29677,7 +29711,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>186.41</v>
+        <v>189.29</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29685,7 +29719,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29717,7 +29751,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>725.1799999999999</v>
+        <v>725.9299999999999</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29725,7 +29759,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29757,7 +29791,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>29.62</v>
+        <v>29.88</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29765,7 +29799,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29773,7 +29807,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>29.620001</v>
+        <v>29.879999</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29797,7 +29831,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>161.28</v>
+        <v>173.86</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29805,7 +29839,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29813,7 +29847,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>161.517523</v>
+        <v>159.681438</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29837,7 +29871,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>768.84</v>
+        <v>770.13</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29845,7 +29879,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29853,7 +29887,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>759.08778</v>
+        <v>769.273701</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29877,7 +29911,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>83462</v>
+        <v>84653</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29885,7 +29919,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29893,7 +29927,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83329.66761600001</v>
+        <v>83493.882698</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29917,7 +29951,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.00966</v>
+        <v>0.009407</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29925,7 +29959,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29933,7 +29967,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.010065</v>
+        <v>0.009648</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29957,7 +29991,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.019326</v>
+        <v>0.018477</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29965,7 +29999,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -29973,7 +30007,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017887</v>
+        <v>0.019125</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -29997,7 +30031,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>118.01</v>
+        <v>118.76</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30005,7 +30039,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -30013,7 +30047,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>119.12118</v>
+        <v>117.940752</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30037,7 +30071,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.06</v>
+        <v>2.05</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30045,7 +30079,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -30053,7 +30087,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.07229</v>
+        <v>2.067139</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30085,7 +30119,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30117,7 +30151,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035332</v>
+        <v>0.033815</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30125,7 +30159,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30133,7 +30167,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.034964</v>
+        <v>0.03552</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30157,7 +30191,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.843032</v>
+        <v>6.724494</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30165,7 +30199,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30173,7 +30207,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.875088</v>
+        <v>6.83665</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30197,7 +30231,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.6834</v>
+        <v>39.3822</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30205,7 +30239,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30213,7 +30247,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.054854</v>
+        <v>39.758106</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30237,7 +30271,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.181365</v>
+        <v>0.201956</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30245,7 +30279,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30253,7 +30287,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.170189</v>
+        <v>0.180643</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30277,7 +30311,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25856.0892</v>
+        <v>25922.5758</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30285,7 +30319,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30293,7 +30327,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25528.122027</v>
+        <v>25893.752771</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30317,7 +30351,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2806827.06</v>
+        <v>2849419.98</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30325,7 +30359,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30333,7 +30367,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2802376.721932</v>
+        <v>2810404.091623</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30357,7 +30391,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.185837</v>
+        <v>3.157005</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30365,7 +30399,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30373,7 +30407,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.153116</v>
+        <v>3.18709</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30397,7 +30431,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>90367.8456</v>
+        <v>90984.663</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30405,7 +30439,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30413,7 +30447,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89733.06937700001</v>
+        <v>90372.59649500001</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30437,7 +30471,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.499301</v>
+        <v>20.548858</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30445,7 +30479,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30453,7 +30487,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.369568</v>
+        <v>20.487974</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30477,7 +30511,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>83462</v>
+        <v>84653</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30485,7 +30519,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30493,7 +30527,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83329.66761600001</v>
+        <v>83493.882698</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30517,7 +30551,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.58</v>
+        <v>23.85</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30525,7 +30559,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30533,7 +30567,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>26.334778</v>
+        <v>24.743398</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30631,7 +30665,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.00966</v>
+        <v>0.009407</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30639,7 +30673,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30647,7 +30681,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.010065</v>
+        <v>0.009648</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30671,7 +30705,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>118.01</v>
+        <v>118.76</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30679,7 +30713,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30687,7 +30721,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>119.12118</v>
+        <v>117.940752</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30719,7 +30753,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30751,7 +30785,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>24.9637</v>
+        <v>24.8045</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -30759,7 +30793,7 @@
         </is>
       </c>
       <c r="G108" s="47" t="n">
-        <v>46290</v>
+        <v>46288</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-10-02
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25725,28 +25725,28 @@
         <v>46297</v>
       </c>
       <c r="C128" t="n">
-        <v>26590978</v>
+        <v>26582660</v>
       </c>
       <c r="D128" t="n">
-        <v>22883121</v>
+        <v>22883938</v>
       </c>
       <c r="E128" t="n">
-        <v>3707857</v>
+        <v>3698722</v>
       </c>
       <c r="F128" t="n">
-        <v>0.162</v>
+        <v>0.1616</v>
       </c>
       <c r="G128" t="n">
-        <v>18614282</v>
+        <v>18606223</v>
       </c>
       <c r="H128" t="n">
-        <v>4939736</v>
+        <v>4940707</v>
       </c>
       <c r="I128" t="n">
-        <v>1634280</v>
+        <v>1633353</v>
       </c>
       <c r="J128" t="n">
-        <v>33.66</v>
+        <v>33.67</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -26341,7 +26341,7 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.66</v>
+        <v>33.67</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
@@ -26390,7 +26390,7 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2873</v>
+        <v>26.2816</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
@@ -26779,27 +26779,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.3038</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.5855</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.4542</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -29831,7 +29831,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>173.86</v>
+        <v>175.18</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29847,7 +29847,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>159.681438</v>
+        <v>161.376239</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29871,7 +29871,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>770.13</v>
+        <v>769.71</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29887,7 +29887,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>769.273701</v>
+        <v>769.15517</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29911,7 +29911,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84653</v>
+        <v>84592</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29927,7 +29927,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83493.882698</v>
+        <v>83471.055997</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29951,7 +29951,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009407</v>
+        <v>0.009428000000000001</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29967,7 +29967,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009648</v>
+        <v>0.009675</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29991,7 +29991,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018477</v>
+        <v>0.01844</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -30007,7 +30007,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.019125</v>
+        <v>0.019329</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30031,7 +30031,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>118.76</v>
+        <v>118.75</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30047,7 +30047,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>117.940752</v>
+        <v>118.196025</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30087,7 +30087,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.067139</v>
+        <v>2.065183</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30151,7 +30151,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.033815</v>
+        <v>0.033869</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30167,7 +30167,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.03552</v>
+        <v>0.035444</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30191,7 +30191,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.724494</v>
+        <v>6.738175</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30207,7 +30207,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.83665</v>
+        <v>6.86409</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30231,7 +30231,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.3822</v>
+        <v>39.3939</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30247,7 +30247,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.758106</v>
+        <v>39.920963</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30271,7 +30271,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.201956</v>
+        <v>0.199459</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30287,7 +30287,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.180643</v>
+        <v>0.181707</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30311,7 +30311,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25922.5758</v>
+        <v>25916.1357</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30327,7 +30327,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25893.752771</v>
+        <v>25897.454589</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30351,7 +30351,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2849419.98</v>
+        <v>2848212.64</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30367,7 +30367,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2810404.091623</v>
+        <v>2810470.455414</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30391,7 +30391,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.157005</v>
+        <v>3.145317</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30407,7 +30407,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.18709</v>
+        <v>3.198611</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30431,7 +30431,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>90984.663</v>
+        <v>90918.0909</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30447,7 +30447,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90372.59649500001</v>
+        <v>90537.366803</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30471,7 +30471,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.548858</v>
+        <v>20.535804</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30487,7 +30487,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.487974</v>
+        <v>20.574333</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30511,7 +30511,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84653</v>
+        <v>84592</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30527,7 +30527,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83493.882698</v>
+        <v>83471.055997</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30551,7 +30551,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.85</v>
+        <v>23.89</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30567,7 +30567,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>24.743398</v>
+        <v>24.679847</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30665,7 +30665,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009407</v>
+        <v>0.009428000000000001</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30681,7 +30681,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009648</v>
+        <v>0.009675</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30705,7 +30705,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>118.76</v>
+        <v>118.75</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30721,7 +30721,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>117.940752</v>
+        <v>118.196025</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-03
FX 33.53 · 98 updated · 1 MF carried · 5 manual
SEC NAV: matched 33/34 via SEC /v2/fund; no NAV: ASP-DGOV-R
Total ฿26,555,815 · P&L +16.13% · 156 history point(s) · perf history 156d
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L128"/>
+  <dimension ref="B2:L129"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25749,6 +25749,40 @@
         <v>33.67</v>
       </c>
       <c r="K128" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" s="72" t="n">
+        <v>46298</v>
+      </c>
+      <c r="C129" t="n">
+        <v>26555815</v>
+      </c>
+      <c r="D129" t="n">
+        <v>22867967</v>
+      </c>
+      <c r="E129" t="n">
+        <v>3687848</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.1613</v>
+      </c>
+      <c r="G129" t="n">
+        <v>18558778</v>
+      </c>
+      <c r="H129" t="n">
+        <v>4984525</v>
+      </c>
+      <c r="I129" t="n">
+        <v>1620863</v>
+      </c>
+      <c r="J129" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="K129" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26326,7 +26360,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26341,11 +26375,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.67</v>
+        <v>33.53</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-02</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -26390,11 +26424,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2816</v>
+        <v>26.2246</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-02</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -26509,27 +26543,27 @@
         </is>
       </c>
       <c r="E5" s="33" t="n">
+        <v>21.1578</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>21.1169</v>
       </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G5" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>21.5084</v>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26599,7 +26633,7 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
-        <v>7.3252</v>
+        <v>7.3419</v>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
@@ -26607,7 +26641,7 @@
         </is>
       </c>
       <c r="G7" s="28" t="n">
-        <v>46289</v>
+        <v>46295</v>
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
@@ -26615,11 +26649,11 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7.3983</v>
+        <v>7.3561</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26644,7 +26678,7 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
-        <v>8.408799999999999</v>
+        <v>8.4193</v>
       </c>
       <c r="F8" s="34" t="inlineStr">
         <is>
@@ -26652,7 +26686,7 @@
         </is>
       </c>
       <c r="G8" s="28" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
@@ -26660,11 +26694,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>8.5023</v>
+        <v>8.4344</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26689,27 +26723,27 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
+        <v>9.712300000000001</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>9.724399999999999</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G9" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H9" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>9.790100000000001</v>
-      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26734,7 +26768,7 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
-        <v>13.3384</v>
+        <v>13.5094</v>
       </c>
       <c r="F10" s="34" t="inlineStr">
         <is>
@@ -26742,7 +26776,7 @@
         </is>
       </c>
       <c r="G10" s="28" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="H10" s="34" t="inlineStr">
         <is>
@@ -26750,11 +26784,11 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>13.3977</v>
+        <v>13.2537</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26779,27 +26813,27 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
+        <v>15.2871</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>15.3038</v>
       </c>
-      <c r="F11" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G11" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H11" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>15.5855</v>
-      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26824,27 +26858,27 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
+        <v>29.7623</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29.6694</v>
       </c>
-      <c r="F12" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H12" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>30.3077</v>
-      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26869,7 +26903,7 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
-        <v>36.3408</v>
+        <v>35.5333</v>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
@@ -26877,7 +26911,7 @@
         </is>
       </c>
       <c r="G13" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H13" s="34" t="inlineStr">
         <is>
@@ -26885,11 +26919,11 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>36.7421</v>
+        <v>35.4712</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26914,27 +26948,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.6722</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.652</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>26.1286</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26959,7 +26993,7 @@
         </is>
       </c>
       <c r="E15" s="33" t="n">
-        <v>16.2768</v>
+        <v>16.3138</v>
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
@@ -26967,7 +27001,7 @@
         </is>
       </c>
       <c r="G15" s="28" t="n">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="H15" s="34" t="inlineStr">
         <is>
@@ -26975,11 +27009,11 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>16.2563</v>
+        <v>16.3605</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27004,7 +27038,7 @@
         </is>
       </c>
       <c r="E16" s="33" t="n">
-        <v>81.7975</v>
+        <v>79.9799</v>
       </c>
       <c r="F16" s="34" t="inlineStr">
         <is>
@@ -27012,7 +27046,7 @@
         </is>
       </c>
       <c r="G16" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
@@ -27020,11 +27054,11 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>82.3947</v>
+        <v>79.81489999999999</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27049,7 +27083,7 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
-        <v>54.8912</v>
+        <v>53.5737</v>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
@@ -27057,7 +27091,7 @@
         </is>
       </c>
       <c r="G17" s="28" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
@@ -27065,11 +27099,11 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>54.9916</v>
+        <v>53.5184</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27094,27 +27128,27 @@
         </is>
       </c>
       <c r="E18" s="33" t="n">
+        <v>16.4993</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>16.503</v>
       </c>
-      <c r="F18" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G18" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H18" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>16.4844</v>
-      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27139,27 +27173,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4537</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4534</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4526</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27184,7 +27218,7 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
-        <v>41.8107</v>
+        <v>41.6209</v>
       </c>
       <c r="F20" s="34" t="inlineStr">
         <is>
@@ -27192,7 +27226,7 @@
         </is>
       </c>
       <c r="G20" s="28" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="H20" s="34" t="inlineStr">
         <is>
@@ -27200,11 +27234,11 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>42.117</v>
+        <v>41.7227</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27229,27 +27263,27 @@
         </is>
       </c>
       <c r="E21" s="33" t="n">
+        <v>12.1988</v>
+      </c>
+      <c r="F21" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>12.119</v>
       </c>
-      <c r="F21" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H21" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>12.1193</v>
-      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27274,27 +27308,27 @@
         </is>
       </c>
       <c r="E22" s="33" t="n">
+        <v>13.8965</v>
+      </c>
+      <c r="F22" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G22" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>13.9416</v>
       </c>
-      <c r="F22" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G22" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H22" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>13.9984</v>
-      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27319,7 +27353,7 @@
         </is>
       </c>
       <c r="E23" s="33" t="n">
-        <v>13.1412</v>
+        <v>12.8301</v>
       </c>
       <c r="F23" s="34" t="inlineStr">
         <is>
@@ -27327,7 +27361,7 @@
         </is>
       </c>
       <c r="G23" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H23" s="34" t="inlineStr">
         <is>
@@ -27335,11 +27369,11 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>13.2439</v>
+        <v>12.8186</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27364,27 +27398,27 @@
         </is>
       </c>
       <c r="E24" s="33" t="n">
+        <v>11.9893</v>
+      </c>
+      <c r="F24" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>11.9228</v>
       </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G24" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H24" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>11.9325</v>
-      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27409,7 +27443,7 @@
         </is>
       </c>
       <c r="E25" s="33" t="n">
-        <v>9.7807</v>
+        <v>9.8133</v>
       </c>
       <c r="F25" s="34" t="inlineStr">
         <is>
@@ -27417,7 +27451,7 @@
         </is>
       </c>
       <c r="G25" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H25" s="34" t="inlineStr">
         <is>
@@ -27425,11 +27459,11 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>9.8056</v>
+        <v>9.763999999999999</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27454,27 +27488,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.7767</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.6983</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.7199</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27499,7 +27533,7 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>18.1354</v>
+        <v>17.6594</v>
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
@@ -27507,7 +27541,7 @@
         </is>
       </c>
       <c r="G27" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H27" s="34" t="inlineStr">
         <is>
@@ -27515,11 +27549,11 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>18.2761</v>
+        <v>17.6761</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27544,7 +27578,7 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
-        <v>18.196</v>
+        <v>18.2549</v>
       </c>
       <c r="F28" s="34" t="inlineStr">
         <is>
@@ -27552,7 +27586,7 @@
         </is>
       </c>
       <c r="G28" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H28" s="34" t="inlineStr">
         <is>
@@ -27560,11 +27594,11 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>18.1891</v>
+        <v>18.3728</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27589,7 +27623,7 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>24.5455</v>
+        <v>24.5761</v>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
@@ -27597,7 +27631,7 @@
         </is>
       </c>
       <c r="G29" s="28" t="n">
-        <v>46289</v>
+        <v>46295</v>
       </c>
       <c r="H29" s="34" t="inlineStr">
         <is>
@@ -27605,11 +27639,11 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>25.1552</v>
+        <v>25.169</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27634,27 +27668,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>38.2335</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>38.3251</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>37.3627</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27679,27 +27713,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>12.9558</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.9176</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>13.2197</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27724,27 +27758,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.724</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.7238</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7236</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27769,27 +27803,27 @@
         </is>
       </c>
       <c r="E33" s="33" t="n">
+        <v>12.7845</v>
+      </c>
+      <c r="F33" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>12.7601</v>
       </c>
-      <c r="F33" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H33" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>13.0209</v>
-      </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27814,7 +27848,7 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
-        <v>16.2426</v>
+        <v>16.2432</v>
       </c>
       <c r="F34" s="34" t="inlineStr">
         <is>
@@ -27822,7 +27856,7 @@
         </is>
       </c>
       <c r="G34" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H34" s="34" t="inlineStr">
         <is>
@@ -27830,11 +27864,11 @@
         </is>
       </c>
       <c r="I34" t="n">
-        <v>16.2422</v>
+        <v>16.2428</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27859,27 +27893,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.4916</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.6783</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46294</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.3289</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27904,7 +27938,7 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
-        <v>9.9907</v>
+        <v>10.0351</v>
       </c>
       <c r="F36" s="34" t="inlineStr">
         <is>
@@ -27912,7 +27946,7 @@
         </is>
       </c>
       <c r="G36" s="28" t="n">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="H36" s="34" t="inlineStr">
         <is>
@@ -27920,11 +27954,11 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>10.0153</v>
+        <v>10.0396</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27949,27 +27983,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>22.8658</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.8402</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>23.3975</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27994,7 +28028,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>21.78</v>
+        <v>21.35</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -28002,7 +28036,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -28010,7 +28044,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.35</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -28034,7 +28068,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.052</v>
+        <v>1.044</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -28042,7 +28076,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -28050,7 +28084,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.044</v>
+        <v>1.041</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -28074,7 +28108,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>780.17</v>
+        <v>779.79</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -28082,7 +28116,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28090,7 +28124,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>779.789978</v>
+        <v>795.179993</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28162,7 +28196,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28194,23 +28228,23 @@
         </is>
       </c>
       <c r="E43" s="33" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="F43" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>14.4</v>
-      </c>
-      <c r="F43" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G43" s="28" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H43" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I43" t="n">
-        <v>14.5</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -28234,23 +28268,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>185.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>184.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>189</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28274,7 +28308,7 @@
         </is>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
@@ -28282,7 +28316,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28290,7 +28324,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="58">
@@ -28322,7 +28356,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28431,23 +28465,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>59</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28471,7 +28505,7 @@
         </is>
       </c>
       <c r="E50" s="33" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
       <c r="F50" s="34" t="inlineStr">
         <is>
@@ -28479,7 +28513,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28487,7 +28521,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="58">
@@ -28511,7 +28545,7 @@
         </is>
       </c>
       <c r="E51" s="33" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
@@ -28519,7 +28553,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28527,7 +28561,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>15.9</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="58">
@@ -28551,7 +28585,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>14.8</v>
+        <v>15</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28559,7 +28593,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28599,7 +28633,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28631,7 +28665,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28639,7 +28673,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28679,7 +28713,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28711,7 +28745,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.42</v>
+        <v>4.46</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28719,7 +28753,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28727,7 +28761,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.42</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28751,7 +28785,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.12</v>
+        <v>3.16</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28759,7 +28793,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28767,7 +28801,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.12</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28799,7 +28833,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28831,7 +28865,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28839,7 +28873,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28871,7 +28905,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>136.71</v>
+        <v>147.77</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28879,7 +28913,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28887,7 +28921,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>131.179993</v>
+        <v>136.710007</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28911,7 +28945,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>241.28</v>
+        <v>237.69</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -28919,7 +28953,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28927,7 +28961,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>239.940002</v>
+        <v>241.279999</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28951,7 +28985,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>529.3</v>
+        <v>540.04</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -28959,7 +28993,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -28967,7 +29001,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>511.380005</v>
+        <v>529.299988</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -28991,7 +29025,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>120.17</v>
+        <v>121.17</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -28999,7 +29033,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -29007,7 +29041,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>119.970001</v>
+        <v>120.169998</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -29031,23 +29065,23 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
+        <v>33.47</v>
+      </c>
+      <c r="F64" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G64" s="28" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H64" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
         <v>32.82</v>
-      </c>
-      <c r="F64" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G64" s="28" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H64" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I64" t="n">
-        <v>32.990002</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -29071,7 +29105,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>186.11</v>
+        <v>191.88</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -29079,7 +29113,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29087,7 +29121,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>182.779999</v>
+        <v>186.110001</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -29111,7 +29145,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>178.72</v>
+        <v>180.95</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -29119,7 +29153,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29127,7 +29161,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>178.759995</v>
+        <v>178.720001</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -29151,7 +29185,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>192.8</v>
+        <v>184.8</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29159,7 +29193,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29167,7 +29201,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>186.539993</v>
+        <v>192.800003</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29191,7 +29225,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>200.33</v>
+        <v>206.89</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29199,7 +29233,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29207,7 +29241,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>194.929993</v>
+        <v>200.330002</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29231,7 +29265,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1149.85</v>
+        <v>1142.85</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29239,7 +29273,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29247,7 +29281,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1157.079956</v>
+        <v>1149.849976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29271,23 +29305,23 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
+        <v>81.31999999999999</v>
+      </c>
+      <c r="F70" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G70" s="28" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H70" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
         <v>78.5</v>
-      </c>
-      <c r="F70" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G70" s="28" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H70" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I70" t="n">
-        <v>77.769997</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29311,7 +29345,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1360.97</v>
+        <v>1439.73</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29319,7 +29353,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29327,7 +29361,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1347.219971</v>
+        <v>1360.969971</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29351,7 +29385,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>161.33</v>
+        <v>160.66</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29359,7 +29393,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29367,7 +29401,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>156.320007</v>
+        <v>161.330002</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29391,7 +29425,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>230.86</v>
+        <v>233.95</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29399,7 +29433,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29407,7 +29441,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>228.380005</v>
+        <v>230.860001</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29431,7 +29465,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>77.39</v>
+        <v>80.37</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29439,7 +29473,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29447,7 +29481,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>77.040001</v>
+        <v>77.389999</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29471,7 +29505,7 @@
         </is>
       </c>
       <c r="E75" s="33" t="n">
-        <v>112.21</v>
+        <v>114.17</v>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
@@ -29479,7 +29513,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29487,7 +29521,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>114.480003</v>
+        <v>112.209999</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29511,7 +29545,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>415.79</v>
+        <v>449.04</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29519,7 +29553,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29527,7 +29561,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>400.910004</v>
+        <v>415.790009</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29551,7 +29585,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>354.11</v>
+        <v>370.59</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29559,7 +29593,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29567,7 +29601,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>354.809998</v>
+        <v>354.109985</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29591,7 +29625,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>41.74</v>
+        <v>41.55</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29599,7 +29633,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29607,7 +29641,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>41.950001</v>
+        <v>41.740002</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29631,7 +29665,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>62.95</v>
+        <v>63.21</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29639,7 +29673,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29647,7 +29681,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>64.260002</v>
+        <v>62.950001</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29671,7 +29705,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>330.32</v>
+        <v>333.69</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29679,7 +29713,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29687,7 +29721,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>333.019989</v>
+        <v>330.320007</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29711,7 +29745,7 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
-        <v>189.29</v>
+        <v>183</v>
       </c>
       <c r="F81" s="34" t="inlineStr">
         <is>
@@ -29719,7 +29753,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29727,7 +29761,7 @@
         </is>
       </c>
       <c r="I81" t="n">
-        <v>186.410004</v>
+        <v>189.289993</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29751,7 +29785,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>725.9299999999999</v>
+        <v>728.08</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29759,7 +29793,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29767,7 +29801,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>725.179993</v>
+        <v>725.929993</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29791,7 +29825,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>29.88</v>
+        <v>29.83</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29799,7 +29833,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29807,7 +29841,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>29.879999</v>
+        <v>29.83</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29831,7 +29865,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>175.18</v>
+        <v>179.59</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29839,7 +29873,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29847,7 +29881,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>161.376239</v>
+        <v>173.841574</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29871,7 +29905,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>769.71</v>
+        <v>768.83</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29879,7 +29913,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29887,7 +29921,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>769.15517</v>
+        <v>770.123472</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29911,7 +29945,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84592</v>
+        <v>84640</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29919,7 +29953,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29927,7 +29961,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>83471.055997</v>
+        <v>84638.16114</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29951,7 +29985,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009428000000000001</v>
+        <v>0.009053</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29959,7 +29993,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -29967,7 +30001,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009675</v>
+        <v>0.009412999999999999</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -29991,7 +30025,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.01844</v>
+        <v>0.018134</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -29999,7 +30033,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -30007,7 +30041,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.019329</v>
+        <v>0.018484</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30031,7 +30065,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>118.75</v>
+        <v>119.2</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30039,7 +30073,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -30047,7 +30081,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>118.196025</v>
+        <v>118.761285</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30071,7 +30105,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.05</v>
+        <v>2.11</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30079,7 +30113,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -30087,7 +30121,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.065183</v>
+        <v>2.052748</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30119,7 +30153,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30151,7 +30185,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.033869</v>
+        <v>0.035356</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30159,7 +30193,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30167,7 +30201,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035444</v>
+        <v>0.033831</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30191,7 +30225,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.738175</v>
+        <v>6.609735</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30199,7 +30233,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30207,7 +30241,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.86409</v>
+        <v>6.698396</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30231,7 +30265,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.3939</v>
+        <v>39.9007</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30239,7 +30273,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30247,7 +30281,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.920963</v>
+        <v>39.194876</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30271,7 +30305,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.199459</v>
+        <v>0.185703</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30279,7 +30313,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30287,7 +30321,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.181707</v>
+        <v>0.200895</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30311,7 +30345,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25916.1357</v>
+        <v>25778.8699</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30319,7 +30353,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30327,7 +30361,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25897.454589</v>
+        <v>25822.240015</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30351,7 +30385,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2848212.64</v>
+        <v>2837979.2</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30359,7 +30393,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30367,7 +30401,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2810470.455414</v>
+        <v>2837917.543015</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30391,7 +30425,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.145317</v>
+        <v>3.129321</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30399,7 +30433,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30407,7 +30441,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.198611</v>
+        <v>3.144483</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30431,7 +30465,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>90918.0909</v>
+        <v>89835.58779999999</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30439,7 +30473,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30447,7 +30481,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90537.366803</v>
+        <v>90630.72941</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30471,7 +30505,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.535804</v>
+        <v>20.43459</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30479,7 +30513,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30487,7 +30521,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.574333</v>
+        <v>20.471774</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30511,7 +30545,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84592</v>
+        <v>84640</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30519,7 +30553,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30527,7 +30561,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>83471.055997</v>
+        <v>84638.16114</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30551,7 +30585,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>23.89</v>
+        <v>24.59</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30559,7 +30593,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30567,7 +30601,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>24.679847</v>
+        <v>23.85412</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30665,7 +30699,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009428000000000001</v>
+        <v>0.009053</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30673,7 +30707,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30681,7 +30715,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009675</v>
+        <v>0.009412999999999999</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30705,7 +30739,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>118.75</v>
+        <v>119.2</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30713,7 +30747,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30721,7 +30755,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>118.196025</v>
+        <v>118.761285</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30753,7 +30787,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30785,7 +30819,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>24.8045</v>
+        <v>24.8512</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -30793,7 +30827,7 @@
         </is>
       </c>
       <c r="G108" s="47" t="n">
-        <v>46288</v>
+        <v>46294</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -30801,11 +30835,11 @@
         </is>
       </c>
       <c r="I108" t="n">
-        <v>24.6933</v>
+        <v>24.5046</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-10-03
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln w="0">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln w="12600">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln>
+                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr wrap="square"/>
-                <a:lstStyle/>
-                <a:p>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln w="12600">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill/>
-              <a:ln>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr wrap="square"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9360">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln w="9360">
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln w="0">
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln w="9360">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25759,16 +25759,16 @@
         <v>46298</v>
       </c>
       <c r="C129" t="n">
-        <v>26555815</v>
+        <v>26554996</v>
       </c>
       <c r="D129" t="n">
         <v>22867967</v>
       </c>
       <c r="E129" t="n">
-        <v>3687848</v>
+        <v>3687029</v>
       </c>
       <c r="F129" t="n">
-        <v>0.1613</v>
+        <v>0.1612</v>
       </c>
       <c r="G129" t="n">
         <v>18558778</v>
@@ -25777,7 +25777,7 @@
         <v>4984525</v>
       </c>
       <c r="I129" t="n">
-        <v>1620863</v>
+        <v>1620044</v>
       </c>
       <c r="J129" t="n">
         <v>33.53</v>
@@ -26588,27 +26588,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7064</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7061</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7058</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -29865,7 +29865,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>179.59</v>
+        <v>180.25</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29881,7 +29881,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>173.841574</v>
+        <v>175.231682</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29905,7 +29905,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>768.83</v>
+        <v>768.35</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29921,7 +29921,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>770.123472</v>
+        <v>769.622295</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29945,7 +29945,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84640</v>
+        <v>84597</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29961,7 +29961,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84638.16114</v>
+        <v>84587.37276499999</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29985,7 +29985,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009053</v>
+        <v>0.009016</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -30001,7 +30001,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009412999999999999</v>
+        <v>0.009428000000000001</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -30025,7 +30025,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018134</v>
+        <v>0.018085</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -30041,7 +30041,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018484</v>
+        <v>0.01844</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30065,7 +30065,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>119.2</v>
+        <v>119.16</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30081,7 +30081,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>118.761285</v>
+        <v>118.744475</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30105,7 +30105,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.11</v>
+        <v>2.1</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30121,7 +30121,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.052748</v>
+        <v>2.049575</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30185,7 +30185,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035356</v>
+        <v>0.035366</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30201,7 +30201,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.033831</v>
+        <v>0.033869</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30225,7 +30225,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.609735</v>
+        <v>6.598369</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30241,7 +30241,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.698396</v>
+        <v>6.709072</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30281,7 +30281,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.194876</v>
+        <v>39.31141</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30305,7 +30305,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.185703</v>
+        <v>0.18588</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30321,7 +30321,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.200895</v>
+        <v>0.19845</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30345,7 +30345,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25778.8699</v>
+        <v>25762.7755</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30361,7 +30361,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25822.240015</v>
+        <v>25805.435536</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30385,7 +30385,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2837979.2</v>
+        <v>2836537.41</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30401,7 +30401,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2837917.543015</v>
+        <v>2836214.608808</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30425,7 +30425,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.129321</v>
+        <v>3.128953</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30441,7 +30441,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.144483</v>
+        <v>3.132526</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30465,7 +30465,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89835.58779999999</v>
+        <v>89790.9929</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30481,7 +30481,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90630.72941</v>
+        <v>90531.641667</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30505,7 +30505,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.43459</v>
+        <v>20.420306</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30521,7 +30521,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.471774</v>
+        <v>20.450408</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30545,7 +30545,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84640</v>
+        <v>84597</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30561,7 +30561,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84638.16114</v>
+        <v>84587.37276499999</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30585,7 +30585,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.59</v>
+        <v>24.57</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30601,7 +30601,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.85412</v>
+        <v>23.889271</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30699,7 +30699,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009053</v>
+        <v>0.009016</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30715,7 +30715,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009412999999999999</v>
+        <v>0.009428000000000001</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30739,7 +30739,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>119.2</v>
+        <v>119.16</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30755,7 +30755,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>118.761285</v>
+        <v>118.744475</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-04
FX 33.53 · 99 updated · 0 MF carried · 5 manual
SEC NAV: matched 34/34 via SEC /v2/fund
Total ฿26,577,241 · P&L +16.22%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -754,10 +754,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -766,10 +766,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4F81BD"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:ln w="0">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -779,10 +779,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="C0504D"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -792,10 +792,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="9BBB59"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -805,10 +805,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8064A2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -818,10 +818,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4BACC6"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -831,10 +831,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="F79646"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -844,14 +844,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -877,14 +877,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -910,14 +910,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -943,14 +943,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -976,14 +976,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1009,14 +1009,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1040,16 +1040,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1144,16 +1144,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1174,10 +1174,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1189,14 +1189,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1218,8 +1218,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1244,10 +1244,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1256,10 +1256,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4672A8"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1269,10 +1269,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="AB4744"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1282,10 +1282,10 @@
             <idx val="2"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="8AA64F"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1295,10 +1295,10 @@
             <idx val="3"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="725990"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1308,10 +1308,10 @@
             <idx val="4"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="4299B0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1321,10 +1321,10 @@
             <idx val="5"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="DC853E"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1334,10 +1334,10 @@
             <idx val="6"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="93A9CE"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1347,10 +1347,10 @@
             <idx val="7"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="D09493"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1360,10 +1360,10 @@
             <idx val="8"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="B8CD97"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+              <a:ln w="12600">
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -1373,14 +1373,14 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1407,14 +1407,14 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1441,14 +1441,14 @@
             <dLbl>
               <idx val="2"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1475,14 +1475,14 @@
             <dLbl>
               <idx val="3"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1509,14 +1509,14 @@
             <dLbl>
               <idx val="4"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1543,14 +1543,14 @@
             <dLbl>
               <idx val="5"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1577,14 +1577,14 @@
             <dLbl>
               <idx val="6"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1611,14 +1611,14 @@
             <dLbl>
               <idx val="7"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1645,14 +1645,14 @@
             <dLbl>
               <idx val="8"/>
               <spPr>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:ln>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" strike="noStrike">
                       <a:solidFill>
@@ -1677,16 +1677,16 @@
               <showBubbleSize val="1"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -1793,16 +1793,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -1823,10 +1823,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -1838,14 +1838,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -1867,8 +1867,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1895,10 +1895,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1906,16 +1906,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2018,7 +2018,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2027,9 +2027,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2061,7 +2061,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2075,7 +2075,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2084,9 +2084,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2111,16 +2111,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2141,10 +2141,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2156,14 +2156,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -2185,8 +2185,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -2202,10 +2202,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4F81BD"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12600">
+            <a:ln w="12600">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2213,16 +2213,16 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" wrap="square"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike">
                     <a:solidFill>
@@ -2413,7 +2413,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2422,9 +2422,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2456,7 +2456,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+            <a:ln w="9360">
               <a:solidFill>
                 <a:srgbClr val="878787"/>
               </a:solidFill>
@@ -2470,7 +2470,7 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+          <a:ln w="9360">
             <a:solidFill>
               <a:srgbClr val="878787"/>
             </a:solidFill>
@@ -2479,9 +2479,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" strike="noStrike">
                 <a:solidFill>
@@ -2506,16 +2506,16 @@
       <legendPos val="r"/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+        <a:noFill/>
+        <a:ln w="0">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" strike="noStrike">
               <a:solidFill>
@@ -2536,10 +2536,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:srgbClr val="FFFFFF"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9360">
+    <a:ln w="9360">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -2551,7 +2551,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
       <col>1</col>
@@ -2571,9 +2571,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2598,9 +2598,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2625,9 +2625,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2652,9 +2652,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L129"/>
+  <dimension ref="B2:L130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25783,6 +25783,40 @@
         <v>33.53</v>
       </c>
       <c r="K129" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="72" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C130" t="n">
+        <v>26577241</v>
+      </c>
+      <c r="D130" t="n">
+        <v>22867967</v>
+      </c>
+      <c r="E130" t="n">
+        <v>3709274</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="G130" t="n">
+        <v>18558778</v>
+      </c>
+      <c r="H130" t="n">
+        <v>4984525</v>
+      </c>
+      <c r="I130" t="n">
+        <v>1631301</v>
+      </c>
+      <c r="J130" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="K130" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26360,7 +26394,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26379,7 +26413,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-03</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -26428,7 +26462,7 @@
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-03</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -28028,7 +28062,7 @@
         </is>
       </c>
       <c r="E38" s="33" t="n">
-        <v>21.35</v>
+        <v>21.4</v>
       </c>
       <c r="F38" s="34" t="inlineStr">
         <is>
@@ -28036,7 +28070,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -28068,7 +28102,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.044</v>
+        <v>1.041</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -28076,7 +28110,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -28108,7 +28142,7 @@
         </is>
       </c>
       <c r="E40" s="33" t="n">
-        <v>779.79</v>
+        <v>795.1799999999999</v>
       </c>
       <c r="F40" s="34" t="inlineStr">
         <is>
@@ -28116,7 +28150,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28196,7 +28230,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28236,7 +28270,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28276,7 +28310,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -28316,7 +28350,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28356,7 +28390,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28473,7 +28507,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28513,7 +28547,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28553,7 +28587,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28593,7 +28627,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28633,7 +28667,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28673,7 +28707,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28713,7 +28747,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28753,7 +28787,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28793,7 +28827,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28833,7 +28867,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28873,7 +28907,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28913,7 +28947,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28921,7 +28955,7 @@
         </is>
       </c>
       <c r="I60" t="n">
-        <v>136.710007</v>
+        <v>147.770004</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="58">
@@ -28953,7 +28987,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -28961,7 +28995,7 @@
         </is>
       </c>
       <c r="I61" t="n">
-        <v>241.279999</v>
+        <v>237.690002</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="58">
@@ -28993,7 +29027,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -29001,7 +29035,7 @@
         </is>
       </c>
       <c r="I62" t="n">
-        <v>529.299988</v>
+        <v>540.039978</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="58">
@@ -29033,7 +29067,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -29041,7 +29075,7 @@
         </is>
       </c>
       <c r="I63" t="n">
-        <v>120.169998</v>
+        <v>121.169998</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="58">
@@ -29073,7 +29107,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -29081,7 +29115,7 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>32.82</v>
+        <v>33.470001</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="58">
@@ -29113,7 +29147,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29121,7 +29155,7 @@
         </is>
       </c>
       <c r="I65" t="n">
-        <v>186.110001</v>
+        <v>191.880005</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="58">
@@ -29153,7 +29187,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29161,7 +29195,7 @@
         </is>
       </c>
       <c r="I66" t="n">
-        <v>178.720001</v>
+        <v>180.949997</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="58">
@@ -29193,7 +29227,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29201,7 +29235,7 @@
         </is>
       </c>
       <c r="I67" t="n">
-        <v>192.800003</v>
+        <v>184.800003</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="58">
@@ -29233,7 +29267,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29241,7 +29275,7 @@
         </is>
       </c>
       <c r="I68" t="n">
-        <v>200.330002</v>
+        <v>206.889999</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="58">
@@ -29273,7 +29307,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29281,7 +29315,7 @@
         </is>
       </c>
       <c r="I69" t="n">
-        <v>1149.849976</v>
+        <v>1142.849976</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="58">
@@ -29313,7 +29347,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29321,7 +29355,7 @@
         </is>
       </c>
       <c r="I70" t="n">
-        <v>78.5</v>
+        <v>81.31999999999999</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="58">
@@ -29353,7 +29387,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29361,7 +29395,7 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>1360.969971</v>
+        <v>1439.72998</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="58">
@@ -29393,7 +29427,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29401,7 +29435,7 @@
         </is>
       </c>
       <c r="I72" t="n">
-        <v>161.330002</v>
+        <v>160.660004</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="58">
@@ -29433,7 +29467,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29441,7 +29475,7 @@
         </is>
       </c>
       <c r="I73" t="n">
-        <v>230.860001</v>
+        <v>233.949997</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="58">
@@ -29473,7 +29507,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29481,7 +29515,7 @@
         </is>
       </c>
       <c r="I74" t="n">
-        <v>77.389999</v>
+        <v>80.370003</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="58">
@@ -29513,7 +29547,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29521,7 +29555,7 @@
         </is>
       </c>
       <c r="I75" t="n">
-        <v>112.209999</v>
+        <v>114.169998</v>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="58">
@@ -29553,7 +29587,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29561,7 +29595,7 @@
         </is>
       </c>
       <c r="I76" t="n">
-        <v>415.790009</v>
+        <v>449.040009</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="58">
@@ -29593,7 +29627,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29601,7 +29635,7 @@
         </is>
       </c>
       <c r="I77" t="n">
-        <v>354.109985</v>
+        <v>370.589996</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="58">
@@ -29633,7 +29667,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29641,7 +29675,7 @@
         </is>
       </c>
       <c r="I78" t="n">
-        <v>41.740002</v>
+        <v>41.549999</v>
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="58">
@@ -29673,7 +29707,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29681,7 +29715,7 @@
         </is>
       </c>
       <c r="I79" t="n">
-        <v>62.950001</v>
+        <v>63.209999</v>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="58">
@@ -29713,7 +29747,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29721,7 +29755,7 @@
         </is>
       </c>
       <c r="I80" t="n">
-        <v>330.320007</v>
+        <v>333.690002</v>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="58">
@@ -29753,7 +29787,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29793,7 +29827,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29801,7 +29835,7 @@
         </is>
       </c>
       <c r="I82" t="n">
-        <v>725.929993</v>
+        <v>728.080017</v>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="58">
@@ -29833,7 +29867,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29865,7 +29899,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>180.25</v>
+        <v>182.44</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29873,7 +29907,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29881,7 +29915,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>175.231682</v>
+        <v>180.204071</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29905,7 +29939,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>768.35</v>
+        <v>784.02</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29913,7 +29947,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29921,7 +29955,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>769.622295</v>
+        <v>768.882826</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29945,7 +29979,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84597</v>
+        <v>84759</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29953,7 +29987,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29961,7 +29995,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84587.37276499999</v>
+        <v>84659.121575</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -29985,7 +30019,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009016</v>
+        <v>0.009188</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -29993,7 +30027,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -30001,7 +30035,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009428000000000001</v>
+        <v>0.009068</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -30025,7 +30059,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018085</v>
+        <v>0.017882</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -30033,7 +30067,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -30041,7 +30075,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.01844</v>
+        <v>0.018154</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30065,7 +30099,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>119.16</v>
+        <v>120.2</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30073,7 +30107,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -30081,7 +30115,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>118.744475</v>
+        <v>119.418969</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30105,7 +30139,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.1</v>
+        <v>2.04</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30113,7 +30147,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -30121,7 +30155,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.049575</v>
+        <v>2.114726</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30153,7 +30187,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30185,7 +30219,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.035366</v>
+        <v>0.037164</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30193,7 +30227,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30201,7 +30235,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.033869</v>
+        <v>0.035398</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30225,7 +30259,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.598369</v>
+        <v>6.763135</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30233,7 +30267,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30241,7 +30275,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.709072</v>
+        <v>6.607348</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30265,7 +30299,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.9007</v>
+        <v>39.5654</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30273,7 +30307,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30281,7 +30315,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.31141</v>
+        <v>39.888271</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30305,7 +30339,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.18588</v>
+        <v>0.183786</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30313,7 +30347,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30321,7 +30355,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.19845</v>
+        <v>0.185664</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30345,7 +30379,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>25762.7755</v>
+        <v>26288.1906</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30353,7 +30387,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30361,7 +30395,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25805.435536</v>
+        <v>25780.64116</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30385,7 +30419,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2836537.41</v>
+        <v>2841969.27</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30393,7 +30427,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30401,7 +30435,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2836214.608808</v>
+        <v>2838620.346404</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30425,7 +30459,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.128953</v>
+        <v>3.114702</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30433,7 +30467,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30441,7 +30475,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.132526</v>
+        <v>3.13277</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30465,7 +30499,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>89790.9929</v>
+        <v>90310.0373</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30473,7 +30507,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30481,7 +30515,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90531.641667</v>
+        <v>89860.838848</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30505,7 +30539,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.420306</v>
+        <v>20.316833</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30513,7 +30547,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30521,7 +30555,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.450408</v>
+        <v>20.436366</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30545,7 +30579,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84597</v>
+        <v>84759</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30553,7 +30587,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30561,7 +30595,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84587.37276499999</v>
+        <v>84659.121575</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30585,7 +30619,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>24.57</v>
+        <v>25.38</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30593,7 +30627,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30601,7 +30635,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>23.889271</v>
+        <v>24.577247</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30699,7 +30733,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009016</v>
+        <v>0.009188</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30707,7 +30741,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30715,7 +30749,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009428000000000001</v>
+        <v>0.009068</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30739,7 +30773,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>119.16</v>
+        <v>120.2</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30747,7 +30781,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30755,7 +30789,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>118.744475</v>
+        <v>119.418969</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30787,7 +30821,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-05
FX 33.53 · 94 updated · 5 MF carried · 5 manual
SEC NAV: matched 29/34 via SEC /v2/fund; no NAV: ASP-AIEQ, BCARERMF, BERMF, K-TNZ-ThaiESG, K-VIETNAMRMF
Total ฿26,719,546 · P&L +16.84% · 158 history point(s) · perf history 158d
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L130"/>
+  <dimension ref="B2:L131"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25817,6 +25817,40 @@
         <v>33.53</v>
       </c>
       <c r="K130" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" s="72" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C131" t="n">
+        <v>26719546</v>
+      </c>
+      <c r="D131" t="n">
+        <v>22868430</v>
+      </c>
+      <c r="E131" t="n">
+        <v>3851116</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.1684</v>
+      </c>
+      <c r="G131" t="n">
+        <v>18669564</v>
+      </c>
+      <c r="H131" t="n">
+        <v>4984525</v>
+      </c>
+      <c r="I131" t="n">
+        <v>1662071</v>
+      </c>
+      <c r="J131" t="n">
+        <v>33.53</v>
+      </c>
+      <c r="K131" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26394,7 +26428,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26413,7 +26447,7 @@
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-04</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -26458,11 +26492,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2246</v>
+        <v>26.2386</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-04</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -26622,27 +26656,27 @@
         </is>
       </c>
       <c r="E6" s="33" t="n">
+        <v>10.7065</v>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>10.7064</v>
       </c>
-      <c r="F6" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G6" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H6" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>10.7061</v>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -26667,7 +26701,7 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
-        <v>7.3419</v>
+        <v>7.2379</v>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
@@ -26675,7 +26709,7 @@
         </is>
       </c>
       <c r="G7" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
@@ -26683,11 +26717,11 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7.3561</v>
+        <v>7.3252</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -26712,27 +26746,27 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
+        <v>8.432</v>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>8.4193</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H8" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8.4344</v>
-      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26757,7 +26791,7 @@
         </is>
       </c>
       <c r="E9" s="33" t="n">
-        <v>9.712300000000001</v>
+        <v>9.7706</v>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
@@ -26765,7 +26799,7 @@
         </is>
       </c>
       <c r="G9" s="28" t="n">
-        <v>46296</v>
+        <v>46294</v>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
@@ -26773,11 +26807,11 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>9.724399999999999</v>
+        <v>9.790100000000001</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -26802,27 +26836,27 @@
         </is>
       </c>
       <c r="E10" s="33" t="n">
+        <v>13.6496</v>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>13.5094</v>
       </c>
-      <c r="F10" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G10" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H10" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>13.2537</v>
-      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -26847,7 +26881,7 @@
         </is>
       </c>
       <c r="E11" s="33" t="n">
-        <v>15.2871</v>
+        <v>15.4145</v>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
@@ -26855,7 +26889,7 @@
         </is>
       </c>
       <c r="G11" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
@@ -26863,11 +26897,11 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>15.3038</v>
+        <v>15.5855</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26892,7 +26926,7 @@
         </is>
       </c>
       <c r="E12" s="33" t="n">
-        <v>29.7623</v>
+        <v>30.0187</v>
       </c>
       <c r="F12" s="34" t="inlineStr">
         <is>
@@ -26900,7 +26934,7 @@
         </is>
       </c>
       <c r="G12" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H12" s="34" t="inlineStr">
         <is>
@@ -26937,7 +26971,7 @@
         </is>
       </c>
       <c r="E13" s="33" t="n">
-        <v>35.5333</v>
+        <v>35.4712</v>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
@@ -26945,7 +26979,7 @@
         </is>
       </c>
       <c r="G13" s="28" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="H13" s="34" t="inlineStr">
         <is>
@@ -26953,11 +26987,11 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>35.4712</v>
+        <v>36.3408</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -26982,27 +27016,27 @@
         </is>
       </c>
       <c r="E14" s="33" t="n">
+        <v>25.7829</v>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>25.6722</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G14" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H14" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
-        <v>25.652</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27117,27 +27151,27 @@
         </is>
       </c>
       <c r="E17" s="33" t="n">
+        <v>53.8182</v>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>53.5737</v>
       </c>
-      <c r="F17" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G17" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H17" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>53.5184</v>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27170,7 +27204,7 @@
         </is>
       </c>
       <c r="G18" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H18" s="34" t="inlineStr">
         <is>
@@ -27178,11 +27212,11 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>16.503</v>
+        <v>16.4993</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27207,27 +27241,27 @@
         </is>
       </c>
       <c r="E19" s="33" t="n">
+        <v>23.4545</v>
+      </c>
+      <c r="F19" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>23.4537</v>
       </c>
-      <c r="F19" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G19" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H19" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>23.4534</v>
-      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27252,27 +27286,27 @@
         </is>
       </c>
       <c r="E20" s="33" t="n">
+        <v>41.7148</v>
+      </c>
+      <c r="F20" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>41.6209</v>
       </c>
-      <c r="F20" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G20" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H20" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>41.7227</v>
-      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27313,11 +27347,11 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>12.119</v>
+        <v>12.1193</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27358,11 +27392,11 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>13.9416</v>
+        <v>13.9984</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -27522,27 +27556,27 @@
         </is>
       </c>
       <c r="E26" s="33" t="n">
+        <v>13.6171</v>
+      </c>
+      <c r="F26" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>13.7767</v>
       </c>
-      <c r="F26" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G26" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H26" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>13.6983</v>
-      </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27567,7 +27601,7 @@
         </is>
       </c>
       <c r="E27" s="33" t="n">
-        <v>17.6594</v>
+        <v>17.8031</v>
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
@@ -27575,7 +27609,7 @@
         </is>
       </c>
       <c r="G27" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H27" s="34" t="inlineStr">
         <is>
@@ -27612,7 +27646,7 @@
         </is>
       </c>
       <c r="E28" s="33" t="n">
-        <v>18.2549</v>
+        <v>18.3661</v>
       </c>
       <c r="F28" s="34" t="inlineStr">
         <is>
@@ -27620,7 +27654,7 @@
         </is>
       </c>
       <c r="G28" s="28" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="H28" s="34" t="inlineStr">
         <is>
@@ -27628,11 +27662,11 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>18.3728</v>
+        <v>18.196</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -27657,7 +27691,7 @@
         </is>
       </c>
       <c r="E29" s="33" t="n">
-        <v>24.5761</v>
+        <v>25.0436</v>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
@@ -27665,7 +27699,7 @@
         </is>
       </c>
       <c r="G29" s="28" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H29" s="34" t="inlineStr">
         <is>
@@ -27673,11 +27707,11 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>25.169</v>
+        <v>25.1552</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -27702,27 +27736,27 @@
         </is>
       </c>
       <c r="E30" s="33" t="n">
+        <v>38.2161</v>
+      </c>
+      <c r="F30" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>38.2335</v>
       </c>
-      <c r="F30" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G30" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H30" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>38.3251</v>
-      </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27747,27 +27781,27 @@
         </is>
       </c>
       <c r="E31" s="33" t="n">
+        <v>13.022</v>
+      </c>
+      <c r="F31" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>12.9558</v>
       </c>
-      <c r="F31" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G31" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H31" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>12.9176</v>
-      </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27792,27 +27826,27 @@
         </is>
       </c>
       <c r="E32" s="33" t="n">
+        <v>21.7242</v>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>21.724</v>
       </c>
-      <c r="F32" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G32" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H32" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>21.7238</v>
-      </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27882,27 +27916,27 @@
         </is>
       </c>
       <c r="E34" s="33" t="n">
+        <v>16.2436</v>
+      </c>
+      <c r="F34" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>16.2432</v>
       </c>
-      <c r="F34" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G34" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H34" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>16.2428</v>
-      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -27927,27 +27961,27 @@
         </is>
       </c>
       <c r="E35" s="33" t="n">
+        <v>27.7618</v>
+      </c>
+      <c r="F35" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G35" s="28" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>27.4916</v>
       </c>
-      <c r="F35" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G35" s="28" t="n">
-        <v>46295</v>
-      </c>
-      <c r="H35" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>27.6783</v>
-      </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
     </row>
@@ -27972,27 +28006,27 @@
         </is>
       </c>
       <c r="E36" s="33" t="n">
+        <v>10.0322</v>
+      </c>
+      <c r="F36" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G36" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>10.0351</v>
       </c>
-      <c r="F36" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H36" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>10.0396</v>
-      </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -28017,27 +28051,27 @@
         </is>
       </c>
       <c r="E37" s="33" t="n">
+        <v>23.0074</v>
+      </c>
+      <c r="F37" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G37" s="28" t="n">
+        <v>46297</v>
+      </c>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>22.8658</v>
       </c>
-      <c r="F37" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="n">
-        <v>46296</v>
-      </c>
-      <c r="H37" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>22.8402</v>
-      </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -28070,7 +28104,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -28110,7 +28144,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -28150,7 +28184,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28230,7 +28264,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28270,7 +28304,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28310,7 +28344,7 @@
         </is>
       </c>
       <c r="G44" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H44" s="34" t="inlineStr">
         <is>
@@ -28350,7 +28384,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28390,7 +28424,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28507,7 +28541,7 @@
         </is>
       </c>
       <c r="G49" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H49" s="34" t="inlineStr">
         <is>
@@ -28547,7 +28581,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28587,7 +28621,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28627,7 +28661,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28667,7 +28701,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28707,7 +28741,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28747,7 +28781,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28787,7 +28821,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28827,7 +28861,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28867,7 +28901,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28907,7 +28941,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28947,7 +28981,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -28987,7 +29021,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -29027,7 +29061,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -29067,7 +29101,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -29107,7 +29141,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -29147,7 +29181,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29187,7 +29221,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29227,7 +29261,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29267,7 +29301,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29307,7 +29341,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29347,7 +29381,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29387,7 +29421,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29427,7 +29461,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29467,7 +29501,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29507,7 +29541,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29547,7 +29581,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29587,7 +29621,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29627,7 +29661,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29667,7 +29701,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29707,7 +29741,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29747,7 +29781,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29787,7 +29821,7 @@
         </is>
       </c>
       <c r="G81" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H81" s="34" t="inlineStr">
         <is>
@@ -29827,7 +29861,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29867,7 +29901,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29899,7 +29933,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>182.44</v>
+        <v>181.06</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29907,7 +29941,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29915,7 +29949,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>180.204071</v>
+        <v>182.200119</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29939,7 +29973,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>784.02</v>
+        <v>796.74</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29947,7 +29981,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29955,7 +29989,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>768.882826</v>
+        <v>783.494331</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -29979,7 +30013,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>84759</v>
+        <v>86696</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -29987,7 +30021,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -29995,7 +30029,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84659.121575</v>
+        <v>84736.368927</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -30019,7 +30053,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009188</v>
+        <v>0.009781</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -30027,7 +30061,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -30035,7 +30069,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009068</v>
+        <v>0.009183</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -30059,7 +30093,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.017882</v>
+        <v>0.018975</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -30067,7 +30101,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -30075,7 +30109,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.018154</v>
+        <v>0.017883</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30099,7 +30133,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>120.2</v>
+        <v>121.3</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30107,7 +30141,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -30115,7 +30149,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>119.418969</v>
+        <v>120.086725</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30139,7 +30173,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.04</v>
+        <v>2.07</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30147,7 +30181,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -30155,7 +30189,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.114726</v>
+        <v>2.033853</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30187,7 +30221,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30219,7 +30253,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.037164</v>
+        <v>0.03822</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30227,7 +30261,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30235,7 +30269,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.035398</v>
+        <v>0.037168</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30259,7 +30293,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.763135</v>
+        <v>6.846088</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30267,7 +30301,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30275,7 +30309,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.607348</v>
+        <v>6.751371</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30299,7 +30333,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>39.5654</v>
+        <v>41.2419</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30307,7 +30341,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30315,7 +30349,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.888271</v>
+        <v>39.45072</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30339,7 +30373,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.183786</v>
+        <v>0.187808</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30347,7 +30381,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30355,7 +30389,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.185664</v>
+        <v>0.18367</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30379,7 +30413,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>26288.1906</v>
+        <v>26714.6922</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30387,7 +30421,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30395,7 +30429,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>25780.64116</v>
+        <v>26270.564934</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30419,7 +30453,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2841969.27</v>
+        <v>2906916.88</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30427,7 +30461,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30435,7 +30469,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2838620.346404</v>
+        <v>2841210.45012</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30459,7 +30493,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.114702</v>
+        <v>3.24158</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30467,7 +30501,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30475,7 +30509,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.13277</v>
+        <v>3.112177</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30499,7 +30533,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>90310.0373</v>
+        <v>91513.0937</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30507,7 +30541,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30515,7 +30549,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>89860.838848</v>
+        <v>90267.775478</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30539,7 +30573,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.316833</v>
+        <v>20.2374</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30547,7 +30581,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30555,7 +30589,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.436366</v>
+        <v>20.316806</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30579,7 +30613,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>84759</v>
+        <v>86696</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30587,7 +30621,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30595,7 +30629,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84659.121575</v>
+        <v>84736.368927</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30619,7 +30653,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>25.38</v>
+        <v>25.28</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30627,7 +30661,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30635,7 +30669,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>24.577247</v>
+        <v>25.37638</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30733,7 +30767,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009188</v>
+        <v>0.009781</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30741,7 +30775,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30749,7 +30783,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009068</v>
+        <v>0.009183</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30773,7 +30807,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>120.2</v>
+        <v>121.3</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30781,7 +30815,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30789,7 +30823,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>119.418969</v>
+        <v>120.086725</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30821,7 +30855,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>
@@ -30853,7 +30887,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>24.8512</v>
+        <v>24.8916</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -30861,7 +30895,7 @@
         </is>
       </c>
       <c r="G108" s="47" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
@@ -30869,11 +30903,11 @@
         </is>
       </c>
       <c r="I108" t="n">
-        <v>24.5046</v>
+        <v>24.6933</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily dashboard update (cloud) — 2026-10-06
FX 33.65 · 65 updated · 34 MF carried · 5 manual
SEC NAV: matched 0/34 via SEC /v2/fund
Total ฿26,751,710 · P&L +16.91%
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -21452,7 +21452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:L131"/>
+  <dimension ref="B2:L132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="58" min="1" max="1"/>
@@ -25851,6 +25851,40 @@
         <v>33.53</v>
       </c>
       <c r="K131" t="inlineStr">
+        <is>
+          <t>Auto weekly snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="72" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C132" t="n">
+        <v>26751710</v>
+      </c>
+      <c r="D132" t="n">
+        <v>22883088</v>
+      </c>
+      <c r="E132" t="n">
+        <v>3868622</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.1691</v>
+      </c>
+      <c r="G132" t="n">
+        <v>18669564</v>
+      </c>
+      <c r="H132" t="n">
+        <v>5017701</v>
+      </c>
+      <c r="I132" t="n">
+        <v>1659429</v>
+      </c>
+      <c r="J132" t="n">
+        <v>33.65</v>
+      </c>
+      <c r="K132" t="inlineStr">
         <is>
           <t>Auto weekly snapshot</t>
         </is>
@@ -26428,7 +26462,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="D5" s="64" t="inlineStr">
         <is>
@@ -26443,11 +26477,11 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>33.53</v>
+        <v>33.65</v>
       </c>
       <c r="D6" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-05</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -26492,11 +26526,11 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>26.2386</v>
+        <v>26.3167</v>
       </c>
       <c r="D9" s="64" t="inlineStr">
         <is>
-          <t>Auto-fetched via Yahoo Finance on 2026-10-05</t>
+          <t>Auto-fetched via Yahoo Finance on 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -28104,7 +28138,7 @@
         </is>
       </c>
       <c r="G38" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
@@ -28112,7 +28146,7 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>21.4</v>
+        <v>21.309999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="58">
@@ -28136,7 +28170,7 @@
         </is>
       </c>
       <c r="E39" s="33" t="n">
-        <v>1.041</v>
+        <v>1.031</v>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
@@ -28144,7 +28178,7 @@
         </is>
       </c>
       <c r="G39" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H39" s="34" t="inlineStr">
         <is>
@@ -28152,7 +28186,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1.041</v>
+        <v>1.031</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="58">
@@ -28184,7 +28218,7 @@
         </is>
       </c>
       <c r="G40" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H40" s="34" t="inlineStr">
         <is>
@@ -28192,7 +28226,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>795.179993</v>
+        <v>797.299988</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="58">
@@ -28264,7 +28298,7 @@
         </is>
       </c>
       <c r="G42" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H42" s="34" t="inlineStr">
         <is>
@@ -28272,7 +28306,7 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>206.539993</v>
+        <v>206.17</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="58">
@@ -28304,7 +28338,7 @@
         </is>
       </c>
       <c r="G43" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H43" s="34" t="inlineStr">
         <is>
@@ -28312,7 +28346,7 @@
         </is>
       </c>
       <c r="I43" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="58">
@@ -28336,23 +28370,23 @@
         </is>
       </c>
       <c r="E44" s="33" t="n">
+        <v>184.5</v>
+      </c>
+      <c r="F44" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>185.5</v>
-      </c>
-      <c r="F44" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G44" s="28" t="n">
-        <v>46300</v>
-      </c>
-      <c r="H44" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I44" t="n">
-        <v>184.5</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="58">
@@ -28384,7 +28418,7 @@
         </is>
       </c>
       <c r="G45" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H45" s="34" t="inlineStr">
         <is>
@@ -28416,7 +28450,7 @@
         </is>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="F46" s="34" t="inlineStr">
         <is>
@@ -28424,7 +28458,7 @@
         </is>
       </c>
       <c r="G46" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H46" s="34" t="inlineStr">
         <is>
@@ -28432,7 +28466,7 @@
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="58">
@@ -28533,23 +28567,23 @@
         </is>
       </c>
       <c r="E49" s="33" t="n">
+        <v>59.75</v>
+      </c>
+      <c r="F49" s="34" t="inlineStr">
+        <is>
+          <t>THB</t>
+        </is>
+      </c>
+      <c r="G49" s="28" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>59.25</v>
-      </c>
-      <c r="F49" s="34" t="inlineStr">
-        <is>
-          <t>THB</t>
-        </is>
-      </c>
-      <c r="G49" s="28" t="n">
-        <v>46300</v>
-      </c>
-      <c r="H49" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>59</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="58">
@@ -28581,7 +28615,7 @@
         </is>
       </c>
       <c r="G50" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H50" s="34" t="inlineStr">
         <is>
@@ -28621,7 +28655,7 @@
         </is>
       </c>
       <c r="G51" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H51" s="34" t="inlineStr">
         <is>
@@ -28653,7 +28687,7 @@
         </is>
       </c>
       <c r="E52" s="33" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="F52" s="34" t="inlineStr">
         <is>
@@ -28661,7 +28695,7 @@
         </is>
       </c>
       <c r="G52" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H52" s="34" t="inlineStr">
         <is>
@@ -28669,7 +28703,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>14.8</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="58">
@@ -28701,7 +28735,7 @@
         </is>
       </c>
       <c r="G53" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H53" s="34" t="inlineStr">
         <is>
@@ -28733,7 +28767,7 @@
         </is>
       </c>
       <c r="E54" s="33" t="n">
-        <v>21.5</v>
+        <v>21.8</v>
       </c>
       <c r="F54" s="34" t="inlineStr">
         <is>
@@ -28741,7 +28775,7 @@
         </is>
       </c>
       <c r="G54" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H54" s="34" t="inlineStr">
         <is>
@@ -28749,7 +28783,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>21.4</v>
+        <v>21.799999</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="58">
@@ -28773,7 +28807,7 @@
         </is>
       </c>
       <c r="E55" s="33" t="n">
-        <v>3.36</v>
+        <v>3.38</v>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
@@ -28781,7 +28815,7 @@
         </is>
       </c>
       <c r="G55" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H55" s="34" t="inlineStr">
         <is>
@@ -28789,7 +28823,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.36</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="58">
@@ -28813,7 +28847,7 @@
         </is>
       </c>
       <c r="E56" s="33" t="n">
-        <v>4.46</v>
+        <v>4.44</v>
       </c>
       <c r="F56" s="34" t="inlineStr">
         <is>
@@ -28821,7 +28855,7 @@
         </is>
       </c>
       <c r="G56" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H56" s="34" t="inlineStr">
         <is>
@@ -28829,7 +28863,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>4.46</v>
+        <v>4.44</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="58">
@@ -28853,7 +28887,7 @@
         </is>
       </c>
       <c r="E57" s="33" t="n">
-        <v>3.16</v>
+        <v>3.18</v>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
@@ -28861,7 +28895,7 @@
         </is>
       </c>
       <c r="G57" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H57" s="34" t="inlineStr">
         <is>
@@ -28869,7 +28903,7 @@
         </is>
       </c>
       <c r="I57" t="n">
-        <v>3.16</v>
+        <v>3.18</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="58">
@@ -28901,7 +28935,7 @@
         </is>
       </c>
       <c r="G58" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H58" s="34" t="inlineStr">
         <is>
@@ -28933,7 +28967,7 @@
         </is>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16.5</v>
+        <v>16.7</v>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
@@ -28941,7 +28975,7 @@
         </is>
       </c>
       <c r="G59" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H59" s="34" t="inlineStr">
         <is>
@@ -28973,7 +29007,7 @@
         </is>
       </c>
       <c r="E60" s="33" t="n">
-        <v>147.77</v>
+        <v>142.31</v>
       </c>
       <c r="F60" s="34" t="inlineStr">
         <is>
@@ -28981,7 +29015,7 @@
         </is>
       </c>
       <c r="G60" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H60" s="34" t="inlineStr">
         <is>
@@ -29013,7 +29047,7 @@
         </is>
       </c>
       <c r="E61" s="33" t="n">
-        <v>237.69</v>
+        <v>238.785</v>
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
@@ -29021,7 +29055,7 @@
         </is>
       </c>
       <c r="G61" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H61" s="34" t="inlineStr">
         <is>
@@ -29053,7 +29087,7 @@
         </is>
       </c>
       <c r="E62" s="33" t="n">
-        <v>540.04</v>
+        <v>542.28</v>
       </c>
       <c r="F62" s="34" t="inlineStr">
         <is>
@@ -29061,7 +29095,7 @@
         </is>
       </c>
       <c r="G62" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H62" s="34" t="inlineStr">
         <is>
@@ -29093,7 +29127,7 @@
         </is>
       </c>
       <c r="E63" s="33" t="n">
-        <v>121.17</v>
+        <v>121.35</v>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
@@ -29101,7 +29135,7 @@
         </is>
       </c>
       <c r="G63" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H63" s="34" t="inlineStr">
         <is>
@@ -29133,7 +29167,7 @@
         </is>
       </c>
       <c r="E64" s="33" t="n">
-        <v>33.47</v>
+        <v>33.45</v>
       </c>
       <c r="F64" s="34" t="inlineStr">
         <is>
@@ -29141,7 +29175,7 @@
         </is>
       </c>
       <c r="G64" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H64" s="34" t="inlineStr">
         <is>
@@ -29173,7 +29207,7 @@
         </is>
       </c>
       <c r="E65" s="33" t="n">
-        <v>191.88</v>
+        <v>191.46</v>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
@@ -29181,7 +29215,7 @@
         </is>
       </c>
       <c r="G65" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H65" s="34" t="inlineStr">
         <is>
@@ -29213,7 +29247,7 @@
         </is>
       </c>
       <c r="E66" s="33" t="n">
-        <v>180.95</v>
+        <v>184.13</v>
       </c>
       <c r="F66" s="34" t="inlineStr">
         <is>
@@ -29221,7 +29255,7 @@
         </is>
       </c>
       <c r="G66" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H66" s="34" t="inlineStr">
         <is>
@@ -29253,7 +29287,7 @@
         </is>
       </c>
       <c r="E67" s="33" t="n">
-        <v>184.8</v>
+        <v>187.76</v>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
@@ -29261,7 +29295,7 @@
         </is>
       </c>
       <c r="G67" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H67" s="34" t="inlineStr">
         <is>
@@ -29293,7 +29327,7 @@
         </is>
       </c>
       <c r="E68" s="33" t="n">
-        <v>206.89</v>
+        <v>206.85</v>
       </c>
       <c r="F68" s="34" t="inlineStr">
         <is>
@@ -29301,7 +29335,7 @@
         </is>
       </c>
       <c r="G68" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H68" s="34" t="inlineStr">
         <is>
@@ -29333,7 +29367,7 @@
         </is>
       </c>
       <c r="E69" s="33" t="n">
-        <v>1142.85</v>
+        <v>1143.12</v>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
@@ -29341,7 +29375,7 @@
         </is>
       </c>
       <c r="G69" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H69" s="34" t="inlineStr">
         <is>
@@ -29373,7 +29407,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>81.31999999999999</v>
+        <v>81.48999999999999</v>
       </c>
       <c r="F70" s="34" t="inlineStr">
         <is>
@@ -29381,7 +29415,7 @@
         </is>
       </c>
       <c r="G70" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H70" s="34" t="inlineStr">
         <is>
@@ -29413,7 +29447,7 @@
         </is>
       </c>
       <c r="E71" s="33" t="n">
-        <v>1439.73</v>
+        <v>1479.89</v>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
@@ -29421,7 +29455,7 @@
         </is>
       </c>
       <c r="G71" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H71" s="34" t="inlineStr">
         <is>
@@ -29453,7 +29487,7 @@
         </is>
       </c>
       <c r="E72" s="33" t="n">
-        <v>160.66</v>
+        <v>159.39</v>
       </c>
       <c r="F72" s="34" t="inlineStr">
         <is>
@@ -29461,7 +29495,7 @@
         </is>
       </c>
       <c r="G72" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H72" s="34" t="inlineStr">
         <is>
@@ -29493,7 +29527,7 @@
         </is>
       </c>
       <c r="E73" s="33" t="n">
-        <v>233.95</v>
+        <v>238.9</v>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
@@ -29501,7 +29535,7 @@
         </is>
       </c>
       <c r="G73" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H73" s="34" t="inlineStr">
         <is>
@@ -29533,7 +29567,7 @@
         </is>
       </c>
       <c r="E74" s="33" t="n">
-        <v>80.37</v>
+        <v>79.8</v>
       </c>
       <c r="F74" s="34" t="inlineStr">
         <is>
@@ -29541,7 +29575,7 @@
         </is>
       </c>
       <c r="G74" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H74" s="34" t="inlineStr">
         <is>
@@ -29581,7 +29615,7 @@
         </is>
       </c>
       <c r="G75" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H75" s="34" t="inlineStr">
         <is>
@@ -29613,7 +29647,7 @@
         </is>
       </c>
       <c r="E76" s="33" t="n">
-        <v>449.04</v>
+        <v>444.53</v>
       </c>
       <c r="F76" s="34" t="inlineStr">
         <is>
@@ -29621,7 +29655,7 @@
         </is>
       </c>
       <c r="G76" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H76" s="34" t="inlineStr">
         <is>
@@ -29653,7 +29687,7 @@
         </is>
       </c>
       <c r="E77" s="33" t="n">
-        <v>370.59</v>
+        <v>378.73</v>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
@@ -29661,7 +29695,7 @@
         </is>
       </c>
       <c r="G77" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H77" s="34" t="inlineStr">
         <is>
@@ -29693,7 +29727,7 @@
         </is>
       </c>
       <c r="E78" s="33" t="n">
-        <v>41.55</v>
+        <v>41.25</v>
       </c>
       <c r="F78" s="34" t="inlineStr">
         <is>
@@ -29701,7 +29735,7 @@
         </is>
       </c>
       <c r="G78" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H78" s="34" t="inlineStr">
         <is>
@@ -29733,7 +29767,7 @@
         </is>
       </c>
       <c r="E79" s="33" t="n">
-        <v>63.21</v>
+        <v>63.54</v>
       </c>
       <c r="F79" s="34" t="inlineStr">
         <is>
@@ -29741,7 +29775,7 @@
         </is>
       </c>
       <c r="G79" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H79" s="34" t="inlineStr">
         <is>
@@ -29773,7 +29807,7 @@
         </is>
       </c>
       <c r="E80" s="33" t="n">
-        <v>333.69</v>
+        <v>332.89</v>
       </c>
       <c r="F80" s="34" t="inlineStr">
         <is>
@@ -29781,7 +29815,7 @@
         </is>
       </c>
       <c r="G80" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H80" s="34" t="inlineStr">
         <is>
@@ -29813,23 +29847,23 @@
         </is>
       </c>
       <c r="E81" s="33" t="n">
+        <v>188.22</v>
+      </c>
+      <c r="F81" s="34" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G81" s="28" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H81" s="34" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
         <v>183</v>
-      </c>
-      <c r="F81" s="34" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G81" s="28" t="n">
-        <v>46300</v>
-      </c>
-      <c r="H81" s="34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I81" t="n">
-        <v>189.289993</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="58">
@@ -29853,7 +29887,7 @@
         </is>
       </c>
       <c r="E82" s="33" t="n">
-        <v>728.08</v>
+        <v>741.9</v>
       </c>
       <c r="F82" s="34" t="inlineStr">
         <is>
@@ -29861,7 +29895,7 @@
         </is>
       </c>
       <c r="G82" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H82" s="34" t="inlineStr">
         <is>
@@ -29893,7 +29927,7 @@
         </is>
       </c>
       <c r="E83" s="33" t="n">
-        <v>29.83</v>
+        <v>29.8</v>
       </c>
       <c r="F83" s="34" t="inlineStr">
         <is>
@@ -29901,7 +29935,7 @@
         </is>
       </c>
       <c r="G83" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H83" s="34" t="inlineStr">
         <is>
@@ -29909,7 +29943,7 @@
         </is>
       </c>
       <c r="I83" t="n">
-        <v>29.83</v>
+        <v>29.799999</v>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="58">
@@ -29933,7 +29967,7 @@
         </is>
       </c>
       <c r="E84" s="33" t="n">
-        <v>181.06</v>
+        <v>184.68</v>
       </c>
       <c r="F84" s="34" t="inlineStr">
         <is>
@@ -29941,7 +29975,7 @@
         </is>
       </c>
       <c r="G84" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H84" s="34" t="inlineStr">
         <is>
@@ -29949,7 +29983,7 @@
         </is>
       </c>
       <c r="I84" t="n">
-        <v>182.200119</v>
+        <v>180.844116</v>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="58">
@@ -29973,7 +30007,7 @@
         </is>
       </c>
       <c r="E85" s="33" t="n">
-        <v>796.74</v>
+        <v>785.5599999999999</v>
       </c>
       <c r="F85" s="34" t="inlineStr">
         <is>
@@ -29981,7 +30015,7 @@
         </is>
       </c>
       <c r="G85" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H85" s="34" t="inlineStr">
         <is>
@@ -29989,7 +30023,7 @@
         </is>
       </c>
       <c r="I85" t="n">
-        <v>783.494331</v>
+        <v>796.534344</v>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="58">
@@ -30013,7 +30047,7 @@
         </is>
       </c>
       <c r="E86" s="33" t="n">
-        <v>86696</v>
+        <v>86046</v>
       </c>
       <c r="F86" s="34" t="inlineStr">
         <is>
@@ -30021,7 +30055,7 @@
         </is>
       </c>
       <c r="G86" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H86" s="34" t="inlineStr">
         <is>
@@ -30029,7 +30063,7 @@
         </is>
       </c>
       <c r="I86" t="n">
-        <v>84736.368927</v>
+        <v>86687.958273</v>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="58">
@@ -30053,7 +30087,7 @@
         </is>
       </c>
       <c r="E87" s="33" t="n">
-        <v>0.009781</v>
+        <v>0.009594999999999999</v>
       </c>
       <c r="F87" s="34" t="inlineStr">
         <is>
@@ -30061,7 +30095,7 @@
         </is>
       </c>
       <c r="G87" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H87" s="34" t="inlineStr">
         <is>
@@ -30069,7 +30103,7 @@
         </is>
       </c>
       <c r="I87" t="n">
-        <v>0.009183</v>
+        <v>0.009769999999999999</v>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="58">
@@ -30093,7 +30127,7 @@
         </is>
       </c>
       <c r="E88" s="33" t="n">
-        <v>0.018975</v>
+        <v>0.019527</v>
       </c>
       <c r="F88" s="34" t="inlineStr">
         <is>
@@ -30101,7 +30135,7 @@
         </is>
       </c>
       <c r="G88" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H88" s="34" t="inlineStr">
         <is>
@@ -30109,7 +30143,7 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>0.017883</v>
+        <v>0.018984</v>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="58">
@@ -30133,7 +30167,7 @@
         </is>
       </c>
       <c r="E89" s="33" t="n">
-        <v>121.3</v>
+        <v>121.1</v>
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
@@ -30141,7 +30175,7 @@
         </is>
       </c>
       <c r="G89" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H89" s="34" t="inlineStr">
         <is>
@@ -30149,7 +30183,7 @@
         </is>
       </c>
       <c r="I89" t="n">
-        <v>120.086725</v>
+        <v>121.2639</v>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="58">
@@ -30173,7 +30207,7 @@
         </is>
       </c>
       <c r="E90" s="33" t="n">
-        <v>2.07</v>
+        <v>2.05</v>
       </c>
       <c r="F90" s="34" t="inlineStr">
         <is>
@@ -30181,7 +30215,7 @@
         </is>
       </c>
       <c r="G90" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H90" s="34" t="inlineStr">
         <is>
@@ -30189,7 +30223,7 @@
         </is>
       </c>
       <c r="I90" t="n">
-        <v>2.033853</v>
+        <v>2.074941</v>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="58">
@@ -30221,7 +30255,7 @@
         </is>
       </c>
       <c r="G91" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H91" s="34" t="inlineStr">
         <is>
@@ -30253,7 +30287,7 @@
         </is>
       </c>
       <c r="E92" s="33" t="n">
-        <v>0.03822</v>
+        <v>0.036966</v>
       </c>
       <c r="F92" s="34" t="inlineStr">
         <is>
@@ -30261,7 +30295,7 @@
         </is>
       </c>
       <c r="G92" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H92" s="34" t="inlineStr">
         <is>
@@ -30269,7 +30303,7 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>0.037168</v>
+        <v>0.038189</v>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="58">
@@ -30293,7 +30327,7 @@
         </is>
       </c>
       <c r="E93" s="33" t="n">
-        <v>6.846088</v>
+        <v>6.93116</v>
       </c>
       <c r="F93" s="34" t="inlineStr">
         <is>
@@ -30301,7 +30335,7 @@
         </is>
       </c>
       <c r="G93" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H93" s="34" t="inlineStr">
         <is>
@@ -30309,7 +30343,7 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>6.751371</v>
+        <v>6.868174</v>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="58">
@@ -30333,7 +30367,7 @@
         </is>
       </c>
       <c r="E94" s="33" t="n">
-        <v>41.2419</v>
+        <v>40.7165</v>
       </c>
       <c r="F94" s="34" t="inlineStr">
         <is>
@@ -30341,7 +30375,7 @@
         </is>
       </c>
       <c r="G94" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H94" s="34" t="inlineStr">
         <is>
@@ -30349,7 +30383,7 @@
         </is>
       </c>
       <c r="I94" t="n">
-        <v>39.45072</v>
+        <v>41.577444</v>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="58">
@@ -30373,7 +30407,7 @@
         </is>
       </c>
       <c r="E95" s="33" t="n">
-        <v>0.187808</v>
+        <v>0.201918</v>
       </c>
       <c r="F95" s="34" t="inlineStr">
         <is>
@@ -30381,7 +30415,7 @@
         </is>
       </c>
       <c r="G95" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H95" s="34" t="inlineStr">
         <is>
@@ -30389,7 +30423,7 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>0.18367</v>
+        <v>0.189127</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="58">
@@ -30413,7 +30447,7 @@
         </is>
       </c>
       <c r="E96" s="33" t="n">
-        <v>26714.6922</v>
+        <v>26434.094</v>
       </c>
       <c r="F96" s="34" t="inlineStr">
         <is>
@@ -30421,7 +30455,7 @@
         </is>
       </c>
       <c r="G96" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H96" s="34" t="inlineStr">
         <is>
@@ -30429,7 +30463,7 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>26270.564934</v>
+        <v>26803.380666</v>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="58">
@@ -30453,7 +30487,7 @@
         </is>
       </c>
       <c r="E97" s="33" t="n">
-        <v>2906916.88</v>
+        <v>2895447.9</v>
       </c>
       <c r="F97" s="34" t="inlineStr">
         <is>
@@ -30461,7 +30495,7 @@
         </is>
       </c>
       <c r="G97" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H97" s="34" t="inlineStr">
         <is>
@@ -30469,7 +30503,7 @@
         </is>
       </c>
       <c r="I97" t="n">
-        <v>2841210.45012</v>
+        <v>2917049.79588</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="58">
@@ -30493,7 +30527,7 @@
         </is>
       </c>
       <c r="E98" s="33" t="n">
-        <v>3.24158</v>
+        <v>3.211152</v>
       </c>
       <c r="F98" s="34" t="inlineStr">
         <is>
@@ -30501,7 +30535,7 @@
         </is>
       </c>
       <c r="G98" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H98" s="34" t="inlineStr">
         <is>
@@ -30509,7 +30543,7 @@
         </is>
       </c>
       <c r="I98" t="n">
-        <v>3.112177</v>
+        <v>3.253846</v>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="58">
@@ -30533,7 +30567,7 @@
         </is>
       </c>
       <c r="E99" s="33" t="n">
-        <v>91513.0937</v>
+        <v>91477.52499999999</v>
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
@@ -30541,7 +30575,7 @@
         </is>
       </c>
       <c r="G99" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H99" s="34" t="inlineStr">
         <is>
@@ -30549,7 +30583,7 @@
         </is>
       </c>
       <c r="I99" t="n">
-        <v>90267.775478</v>
+        <v>91794.999436</v>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="58">
@@ -30573,7 +30607,7 @@
         </is>
       </c>
       <c r="E100" s="33" t="n">
-        <v>20.2374</v>
+        <v>20.396645</v>
       </c>
       <c r="F100" s="34" t="inlineStr">
         <is>
@@ -30581,7 +30615,7 @@
         </is>
       </c>
       <c r="G100" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H100" s="34" t="inlineStr">
         <is>
@@ -30589,7 +30623,7 @@
         </is>
       </c>
       <c r="I100" t="n">
-        <v>20.316806</v>
+        <v>20.363267</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="58">
@@ -30613,7 +30647,7 @@
         </is>
       </c>
       <c r="E101" s="33" t="n">
-        <v>86696</v>
+        <v>86046</v>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
@@ -30621,7 +30655,7 @@
         </is>
       </c>
       <c r="G101" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H101" s="34" t="inlineStr">
         <is>
@@ -30629,7 +30663,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>84736.368927</v>
+        <v>86687.958273</v>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="58">
@@ -30653,7 +30687,7 @@
         </is>
       </c>
       <c r="E102" s="33" t="n">
-        <v>25.28</v>
+        <v>24.78</v>
       </c>
       <c r="F102" s="34" t="inlineStr">
         <is>
@@ -30661,7 +30695,7 @@
         </is>
       </c>
       <c r="G102" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H102" s="34" t="inlineStr">
         <is>
@@ -30669,7 +30703,7 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>25.37638</v>
+        <v>25.276803</v>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="58">
@@ -30767,7 +30801,7 @@
         </is>
       </c>
       <c r="E105" s="33" t="n">
-        <v>0.009781</v>
+        <v>0.009594999999999999</v>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
@@ -30775,7 +30809,7 @@
         </is>
       </c>
       <c r="G105" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H105" s="34" t="inlineStr">
         <is>
@@ -30783,7 +30817,7 @@
         </is>
       </c>
       <c r="I105" t="n">
-        <v>0.009183</v>
+        <v>0.009769999999999999</v>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="58">
@@ -30807,7 +30841,7 @@
         </is>
       </c>
       <c r="E106" s="33" t="n">
-        <v>121.3</v>
+        <v>121.1</v>
       </c>
       <c r="F106" s="34" t="inlineStr">
         <is>
@@ -30815,7 +30849,7 @@
         </is>
       </c>
       <c r="G106" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H106" s="34" t="inlineStr">
         <is>
@@ -30823,7 +30857,7 @@
         </is>
       </c>
       <c r="I106" t="n">
-        <v>120.086725</v>
+        <v>121.2639</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="58">
@@ -30855,7 +30889,7 @@
         </is>
       </c>
       <c r="G107" s="28" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="H107" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily dashboard update — 2026-10-06
</commit_message>
<xml_diff>
--- a/TH Investment - Private Banking Summary.xlsx
+++ b/TH Investment - Private Banking Summary.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-42660" yWindow="-540" windowWidth="32460" windowHeight="17180" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Realized" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prices" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Reference" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flows" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realized" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX &amp; Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - Lots" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MF - by Fund" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - Lots" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equities - by Ticker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - Lots" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crypto - by Coin" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Trust (SGD)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AsOfDate">'FX &amp; Assumptions'!$C$5</definedName>
@@ -699,14 +699,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1300" b="0" strike="noStrike">
                 <a:uFillTx/>
@@ -728,8 +728,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFi